<commit_message>
ETL pipeline: Scopus/Dimensions/OpenAlex, patches, dashboard-tolerant deserialization
</commit_message>
<xml_diff>
--- a/sources/samples/openalex_standardized.xlsx
+++ b/sources/samples/openalex_standardized.xlsx
@@ -601,7 +601,7 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>63749</v>
+        <v>63750</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
@@ -939,7 +939,7 @@
         </is>
       </c>
       <c r="K6" t="n">
-        <v>25718</v>
+        <v>25719</v>
       </c>
       <c r="L6" t="inlineStr">
         <is>
@@ -1026,7 +1026,7 @@
         </is>
       </c>
       <c r="K7" t="n">
-        <v>22084</v>
+        <v>22085</v>
       </c>
       <c r="L7" t="inlineStr">
         <is>
@@ -1125,7 +1125,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>David E. Goldberg</t>
+          <t>David E. Goldberg;David Robson</t>
         </is>
       </c>
       <c r="M8" t="inlineStr"/>
@@ -1237,20 +1237,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>https://openalex.org/W1503398984</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr"/>
+          <t>https://openalex.org/W1746819321</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.7551/mitpress/3206.001.0001</t>
+        </is>
+      </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Machine learning a probabilistic perspective</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
+          <t>Gaussian Processes for Machine Learning</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>The MIT Press eBooks</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>The MIT Press eBooks</t>
+        </is>
+      </c>
       <c r="H10" t="n">
-        <v>2012</v>
+        <v>2005</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
@@ -1263,26 +1275,34 @@
         </is>
       </c>
       <c r="K10" t="n">
-        <v>9328</v>
+        <v>10489</v>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>Kevin P. Murphy</t>
+          <t>Carl Edward Rasmussen;Christopher K. I. Williams</t>
         </is>
       </c>
       <c r="M10" t="inlineStr"/>
-      <c r="N10" t="inlineStr"/>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>Carl Edward Rasmussen, Max Planck Institute for Biological Cybernetics, Max Planck Society;Christopher K. I. Williams, School of Informatics</t>
+        </is>
+      </c>
       <c r="O10" t="inlineStr"/>
-      <c r="P10" t="inlineStr"/>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>https://openalex.org/W14377099; https://openalex.org/W44447720; https://openalex.org/W61071295; https://openalex.org/W131514509; https://openalex.org/W186419298; https://openalex.org/W336602872; https://openalex.org/W1213006044; https://openalex.org/W1484867920; https://openalex.org/W1486089539; https://openalex.org/W1486164486; https://openalex.org/W1496317909; https://openalex.org/W1497675750; https://openalex.org/W1505043854; https://openalex.org/W1506153731; https://openalex.org/W1510355813; https://openalex.org/W1512098439; https://openalex.org/W1512149552; https://openalex.org/W1515272691; https://openalex.org/W1543996294; https://openalex.org/W1549258098; https://openalex.org/W1550570395; https://openalex.org/W1551209770; https://openalex.org/W1554663460; https://openalex.org/W1564947197; https://openalex.org/W1567512734; https://openalex.org/W1571894236; https://openalex.org/W1574225613; https://openalex.org/W1598589417; https://openalex.org/W1601740268; https://openalex.org/W1604293137; https://openalex.org/W1607751291; https://openalex.org/W1618393386; https://openalex.org/W1618449801; https://openalex.org/W1628829797; https://openalex.org/W1633751774; https://openalex.org/W1642427530; https://openalex.org/W1648445109; https://openalex.org/W1654787807; https://openalex.org/W1755117326; https://openalex.org/W1859781365; https://openalex.org/W1963533512; https://openalex.org/W1965999112; https://openalex.org/W1967396577; https://openalex.org/W1975780894; https://openalex.org/W1976382401; https://openalex.org/W1976625337; https://openalex.org/W1978188282; https://openalex.org/W1978394996; https://openalex.org/W1981025032; https://openalex.org/W1982032418; https://openalex.org/W1982276155; https://openalex.org/W1986280275; https://openalex.org/W1995672551; https://openalex.org/W1998167411; https://openalex.org/W2000241167; https://openalex.org/W2003706076; https://openalex.org/W2003870625; https://openalex.org/W2006314423; https://openalex.org/W2008827410; https://openalex.org/W2014831690; https://openalex.org/W2015904350; https://openalex.org/W2018044188; https://openalex.org/W2019363670; https://openalex.org/W2020999234; https://openalex.org/W2023163512; https://openalex.org/W2033839039; https://openalex.org/W2041863660; https://openalex.org/W2047028564; https://openalex.org/W2049387919; https://openalex.org/W2056735347; https://openalex.org/W2062291655; https://openalex.org/W2063852603; https://openalex.org/W2065540158; https://openalex.org/W2069371995; https://openalex.org/W2069527924; https://openalex.org/W2072555316; https://openalex.org/W2078206416; https://openalex.org/W2081873601; https://openalex.org/W2085877024; https://openalex.org/W2087978636; https://openalex.org/W2088538739; https://openalex.org/W2090102379; https://openalex.org/W2090353374; https://openalex.org/W2093268114; https://openalex.org/W2094169479; https://openalex.org/W2094212611; https://openalex.org/W2096335861; https://openalex.org/W2098115979; https://openalex.org/W2098626000; https://openalex.org/W2098949458; https://openalex.org/W2100136038; https://openalex.org/W2101709642; https://openalex.org/W2103972570; https://openalex.org/W2104533781; https://openalex.org/W2106868411; https://openalex.org/W2107152312; https://openalex.org/W2107636931; https://openalex.org/W2107725114; https://openalex.org/W2108966602; https://openalex.org/W2111176881; https://openalex.org/W2111494971; https://openalex.org/W2112545207; https://openalex.org/W2114229504; https://openalex.org/W2114412769; https://openalex.org/W2115606304; https://openalex.org/W2116723448; https://openalex.org/W2117063635; https://openalex.org/W2117812871; https://openalex.org/W2118195892; https://openalex.org/W2123687908; https://openalex.org/W2124101779; https://openalex.org/W2124225821; https://openalex.org/W2126455177; https://openalex.org/W2127713198; https://openalex.org/W2129564505; https://openalex.org/W2129869373; https://openalex.org/W2130475491; https://openalex.org/W2130859329; https://openalex.org/W2137467792; https://openalex.org/W2137557016; https://openalex.org/W2137956165; https://openalex.org/W2139479120; https://openalex.org/W2140170995; https://openalex.org/W2140251433; https://openalex.org/W2141274633; https://openalex.org/W2141436719; https://openalex.org/W2142182841; https://openalex.org/W2142387771; https://openalex.org/W2142575165; https://openalex.org/W2143022286; https://openalex.org/W2143956139; https://openalex.org/W2144286620; https://openalex.org/W2145295623; https://openalex.org/W2146766088; https://openalex.org/W2148603752; https://openalex.org/W2149417376; https://openalex.org/W2149846618; https://openalex.org/W2151238122; https://openalex.org/W2152701363; https://openalex.org/W2152937653; https://openalex.org/W2153347097; https://openalex.org/W2153756422; https://openalex.org/W2156909104; https://openalex.org/W2158451137; https://openalex.org/W2158529569; https://openalex.org/W2160840682; https://openalex.org/W2161767008; https://openalex.org/W2162114812; https://openalex.org/W2163057507; https://openalex.org/W2167061265; https://openalex.org/W2167986580; https://openalex.org/W2168022998; https://openalex.org/W2169779569; https://openalex.org/W2170076406; https://openalex.org/W2170078560; https://openalex.org/W2170120409; https://openalex.org/W2170334710; https://openalex.org/W2171522835; https://openalex.org/W2172039283; https://openalex.org/W2296319761; https://openalex.org/W2408196097; https://openalex.org/W2464224693; https://openalex.org/W2548695521; https://openalex.org/W2554813760; https://openalex.org/W2782810849; https://openalex.org/W2797583072; https://openalex.org/W2798909945; https://openalex.org/W2904816695; https://openalex.org/W2916304084; https://openalex.org/W2989448192; https://openalex.org/W3014600732; https://openalex.org/W3017143921; https://openalex.org/W3023786531; https://openalex.org/W3048078645; https://openalex.org/W3119264854; https://openalex.org/W3127325877; https://openalex.org/W3134067276; https://openalex.org/W3140968660; https://openalex.org/W3148924112; https://openalex.org/W3165771198</t>
+        </is>
+      </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>Computer science;Probabilistic logic;Artificial intelligence;Field (mathematics);Conditional random field;Heuristic;Machine learning;Graphical model;Regularization (linguistics);Software;Programming language</t>
+          <t>Machine learning;Artificial intelligence;Computer science;Online machine learning;Gaussian process;Probabilistic logic;Relevance vector machine;Support vector machine;Kernel method;Artificial neural network;Gaussian</t>
         </is>
       </c>
       <c r="R10" t="inlineStr"/>
       <c r="S10" t="inlineStr">
         <is>
-          <t>Today's Web-enabled deluge of electronic data calls for automated methods of data analysis. Machine learning provides these, developing methods that can automatically detect patterns in data and then use the uncovered patterns to predict future data. This textbook offers a comprehensive and self-contained introduction to the field of machine learning, based on a unified, probabilistic approach. The coverage combines breadth and depth, offering necessary background material on such topics as probability, optimization, and linear algebra as well as discussion of recent developments in the field, including conditional random fields, L1 regularization, and deep learning. The book is written in an informal, accessible style, complete with pseudo-code for the most important algorithms. All topics are copiously illustrated with color images and worked examples drawn from such application domains as biology, text processing, computer vision, and robotics. Rather than providing a cookbook of different heuristic methods, the book stresses a principled model-based approach, often using the language of graphical models to specify models in a concise and intuitive way. Almost all the models described have been implemented in a MATLAB software package--PMTK (probabilistic modeling toolkit)--that is freely available online. The book is suitable for upper-level undergraduates with an introductory-level college math background and beginning graduate students.</t>
+          <t>A comprehensive and self-contained introduction to Gaussian processes, which provide a principled, practical, probabilistic approach to learning in kernel machines.</t>
         </is>
       </c>
       <c r="T10" t="inlineStr"/>
@@ -1291,12 +1311,12 @@
       <c r="W10" t="inlineStr"/>
       <c r="X10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kevin P. Murphy, 2012, </t>
+          <t>Carl Edward Rasmussen, 2005, The MIT Press eBooks</t>
         </is>
       </c>
       <c r="Y10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kevin P. Murphy, 2012, </t>
+          <t>Carl Edward Rasmussen, 2005, The MIT Press eBooks</t>
         </is>
       </c>
     </row>
@@ -1308,32 +1328,20 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>https://openalex.org/W1746819321</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.7551/mitpress/3206.001.0001</t>
-        </is>
-      </c>
+          <t>https://openalex.org/W1503398984</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Gaussian Processes for Machine Learning</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>The MIT Press eBooks</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>The MIT Press eBooks</t>
-        </is>
-      </c>
+          <t>Machine learning a probabilistic perspective</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr"/>
       <c r="H11" t="n">
-        <v>2005</v>
+        <v>2012</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
@@ -1346,34 +1354,26 @@
         </is>
       </c>
       <c r="K11" t="n">
-        <v>10489</v>
+        <v>9328</v>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>Carl Edward Rasmussen;Christopher K. I. Williams</t>
+          <t>Kevin P. Murphy</t>
         </is>
       </c>
       <c r="M11" t="inlineStr"/>
-      <c r="N11" t="inlineStr">
-        <is>
-          <t>Carl Edward Rasmussen, Max Planck Institute for Biological Cybernetics, Max Planck Society;Christopher K. I. Williams, School of Informatics</t>
-        </is>
-      </c>
+      <c r="N11" t="inlineStr"/>
       <c r="O11" t="inlineStr"/>
-      <c r="P11" t="inlineStr">
-        <is>
-          <t>https://openalex.org/W14377099; https://openalex.org/W44447720; https://openalex.org/W61071295; https://openalex.org/W131514509; https://openalex.org/W186419298; https://openalex.org/W336602872; https://openalex.org/W1213006044; https://openalex.org/W1484867920; https://openalex.org/W1486089539; https://openalex.org/W1486164486; https://openalex.org/W1496317909; https://openalex.org/W1497675750; https://openalex.org/W1505043854; https://openalex.org/W1506153731; https://openalex.org/W1510355813; https://openalex.org/W1512098439; https://openalex.org/W1512149552; https://openalex.org/W1515272691; https://openalex.org/W1543996294; https://openalex.org/W1549258098; https://openalex.org/W1550570395; https://openalex.org/W1551209770; https://openalex.org/W1554663460; https://openalex.org/W1564947197; https://openalex.org/W1567512734; https://openalex.org/W1571894236; https://openalex.org/W1574225613; https://openalex.org/W1598589417; https://openalex.org/W1601740268; https://openalex.org/W1604293137; https://openalex.org/W1607751291; https://openalex.org/W1618393386; https://openalex.org/W1618449801; https://openalex.org/W1628829797; https://openalex.org/W1633751774; https://openalex.org/W1642427530; https://openalex.org/W1648445109; https://openalex.org/W1654787807; https://openalex.org/W1755117326; https://openalex.org/W1859781365; https://openalex.org/W1963533512; https://openalex.org/W1965999112; https://openalex.org/W1967396577; https://openalex.org/W1975780894; https://openalex.org/W1976382401; https://openalex.org/W1976625337; https://openalex.org/W1978188282; https://openalex.org/W1978394996; https://openalex.org/W1981025032; https://openalex.org/W1982032418; https://openalex.org/W1982276155; https://openalex.org/W1986280275; https://openalex.org/W1995672551; https://openalex.org/W1998167411; https://openalex.org/W2000241167; https://openalex.org/W2003706076; https://openalex.org/W2003870625; https://openalex.org/W2006314423; https://openalex.org/W2008827410; https://openalex.org/W2014831690; https://openalex.org/W2015904350; https://openalex.org/W2018044188; https://openalex.org/W2019363670; https://openalex.org/W2020999234; https://openalex.org/W2023163512; https://openalex.org/W2033839039; https://openalex.org/W2041863660; https://openalex.org/W2047028564; https://openalex.org/W2049387919; https://openalex.org/W2056735347; https://openalex.org/W2062291655; https://openalex.org/W2063852603; https://openalex.org/W2065540158; https://openalex.org/W2069371995; https://openalex.org/W2069527924; https://openalex.org/W2072555316; https://openalex.org/W2078206416; https://openalex.org/W2081873601; https://openalex.org/W2085877024; https://openalex.org/W2087978636; https://openalex.org/W2088538739; https://openalex.org/W2090102379; https://openalex.org/W2090353374; https://openalex.org/W2093268114; https://openalex.org/W2094169479; https://openalex.org/W2094212611; https://openalex.org/W2096335861; https://openalex.org/W2098115979; https://openalex.org/W2098626000; https://openalex.org/W2098949458; https://openalex.org/W2100136038; https://openalex.org/W2101709642; https://openalex.org/W2103972570; https://openalex.org/W2104533781; https://openalex.org/W2106868411; https://openalex.org/W2107152312; https://openalex.org/W2107636931; https://openalex.org/W2107725114; https://openalex.org/W2108966602; https://openalex.org/W2111176881; https://openalex.org/W2111494971; https://openalex.org/W2112545207; https://openalex.org/W2114229504; https://openalex.org/W2114412769; https://openalex.org/W2115606304; https://openalex.org/W2116723448; https://openalex.org/W2117063635; https://openalex.org/W2117812871; https://openalex.org/W2118195892; https://openalex.org/W2123687908; https://openalex.org/W2124101779; https://openalex.org/W2124225821; https://openalex.org/W2126455177; https://openalex.org/W2127713198; https://openalex.org/W2129564505; https://openalex.org/W2129869373; https://openalex.org/W2130475491; https://openalex.org/W2130859329; https://openalex.org/W2137467792; https://openalex.org/W2137557016; https://openalex.org/W2137956165; https://openalex.org/W2139479120; https://openalex.org/W2140170995; https://openalex.org/W2140251433; https://openalex.org/W2141274633; https://openalex.org/W2141436719; https://openalex.org/W2142182841; https://openalex.org/W2142387771; https://openalex.org/W2142575165; https://openalex.org/W2143022286; https://openalex.org/W2143956139; https://openalex.org/W2144286620; https://openalex.org/W2145295623; https://openalex.org/W2146766088; https://openalex.org/W2148603752; https://openalex.org/W2149417376; https://openalex.org/W2149846618; https://openalex.org/W2151238122; https://openalex.org/W2152701363; https://openalex.org/W2152937653; https://openalex.org/W2153347097; https://openalex.org/W2153756422; https://openalex.org/W2156909104; https://openalex.org/W2158451137; https://openalex.org/W2158529569; https://openalex.org/W2160840682; https://openalex.org/W2161767008; https://openalex.org/W2162114812; https://openalex.org/W2163057507; https://openalex.org/W2167061265; https://openalex.org/W2167986580; https://openalex.org/W2168022998; https://openalex.org/W2169779569; https://openalex.org/W2170076406; https://openalex.org/W2170078560; https://openalex.org/W2170120409; https://openalex.org/W2170334710; https://openalex.org/W2171522835; https://openalex.org/W2172039283; https://openalex.org/W2296319761; https://openalex.org/W2408196097; https://openalex.org/W2464224693; https://openalex.org/W2548695521; https://openalex.org/W2554813760; https://openalex.org/W2782810849; https://openalex.org/W2797583072; https://openalex.org/W2798909945; https://openalex.org/W2904816695; https://openalex.org/W2916304084; https://openalex.org/W2989448192; https://openalex.org/W3014600732; https://openalex.org/W3017143921; https://openalex.org/W3023786531; https://openalex.org/W3048078645; https://openalex.org/W3119264854; https://openalex.org/W3127325877; https://openalex.org/W3134067276; https://openalex.org/W3140968660; https://openalex.org/W3148924112; https://openalex.org/W3165771198</t>
-        </is>
-      </c>
+      <c r="P11" t="inlineStr"/>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>Machine learning;Artificial intelligence;Computer science;Online machine learning;Gaussian process;Probabilistic logic;Relevance vector machine;Support vector machine;Kernel method;Artificial neural network;Gaussian</t>
+          <t>Computer science;Probabilistic logic;Artificial intelligence;Field (mathematics);Conditional random field;Heuristic;Machine learning;Graphical model;Regularization (linguistics);Software;Programming language</t>
         </is>
       </c>
       <c r="R11" t="inlineStr"/>
       <c r="S11" t="inlineStr">
         <is>
-          <t>A comprehensive and self-contained introduction to Gaussian processes, which provide a principled, practical, probabilistic approach to learning in kernel machines.</t>
+          <t>Today's Web-enabled deluge of electronic data calls for automated methods of data analysis. Machine learning provides these, developing methods that can automatically detect patterns in data and then use the uncovered patterns to predict future data. This textbook offers a comprehensive and self-contained introduction to the field of machine learning, based on a unified, probabilistic approach. The coverage combines breadth and depth, offering necessary background material on such topics as probability, optimization, and linear algebra as well as discussion of recent developments in the field, including conditional random fields, L1 regularization, and deep learning. The book is written in an informal, accessible style, complete with pseudo-code for the most important algorithms. All topics are copiously illustrated with color images and worked examples drawn from such application domains as biology, text processing, computer vision, and robotics. Rather than providing a cookbook of different heuristic methods, the book stresses a principled model-based approach, often using the language of graphical models to specify models in a concise and intuitive way. Almost all the models described have been implemented in a MATLAB software package--PMTK (probabilistic modeling toolkit)--that is freely available online. The book is suitable for upper-level undergraduates with an introductory-level college math background and beginning graduate students.</t>
         </is>
       </c>
       <c r="T11" t="inlineStr"/>
@@ -1382,12 +1382,12 @@
       <c r="W11" t="inlineStr"/>
       <c r="X11" t="inlineStr">
         <is>
-          <t>Carl Edward Rasmussen, 2005, The MIT Press eBooks</t>
+          <t xml:space="preserve">Kevin P. Murphy, 2012, </t>
         </is>
       </c>
       <c r="Y11" t="inlineStr">
         <is>
-          <t>Carl Edward Rasmussen, 2005, The MIT Press eBooks</t>
+          <t xml:space="preserve">Kevin P. Murphy, 2012, </t>
         </is>
       </c>
     </row>
@@ -1437,7 +1437,7 @@
         </is>
       </c>
       <c r="K12" t="n">
-        <v>9603</v>
+        <v>9623</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
@@ -1536,7 +1536,7 @@
         </is>
       </c>
       <c r="K13" t="n">
-        <v>9867</v>
+        <v>9868</v>
       </c>
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="inlineStr"/>
@@ -1686,7 +1686,7 @@
         </is>
       </c>
       <c r="K15" t="n">
-        <v>8230</v>
+        <v>8234</v>
       </c>
       <c r="L15" t="inlineStr">
         <is>
@@ -1860,7 +1860,7 @@
         </is>
       </c>
       <c r="K17" t="n">
-        <v>7906</v>
+        <v>7908</v>
       </c>
       <c r="L17" t="inlineStr">
         <is>
@@ -1929,24 +1929,36 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>https://openalex.org/W1504694836</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr"/>
+          <t>https://openalex.org/W3163993681</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1038/s42254-021-00314-5</t>
+        </is>
+      </c>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Programs for Machine Learning</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr"/>
+          <t>Physics-informed machine learning</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Nature Reviews Physics</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Nature Reviews Physics</t>
+        </is>
+      </c>
       <c r="H18" t="n">
-        <v>1994</v>
+        <v>2021</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>article</t>
+          <t>review</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
@@ -1955,48 +1967,60 @@
         </is>
       </c>
       <c r="K18" t="n">
-        <v>5807</v>
+        <v>6740</v>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>Steven L. Salzberg;Alberto M. Segre</t>
+          <t>George Em Karniadakis;Ioannis G. Kevrekidis;Lu Lu;Paris Perdikaris;Sifan Wang;Liu Yang</t>
         </is>
       </c>
       <c r="M18" t="inlineStr"/>
       <c r="N18" t="inlineStr">
         <is>
-          <t>Steven L. Salzberg, Johns Hopkins University (</t>
+          <t>George Em Karniadakis, Division of Applied Mathematics, Brown University Providence, RI, USA;Ioannis G. Kevrekidis, Department of Applied Mathematics and Statistics, Johns Hopkins University, Baltimore, MD, USA;Ioannis G. Kevrekidis, Department of Chemical and Biomolecular Engineering, Johns Hopkins University, Baltimore, MD, USA;Lu Lu, Department of Mathematics, Massachusetts Institute of Technology, Cambridge, MA, USA;Paris Perdikaris, Department of Mechanical Engineering and Applied Mechanics, University of Pennsylvania, Philadelphia, PA, USA;Sifan Wang, Graduate Group in Applied Mathematics and Computational Science, University of Pennsylvania, Philadelphia, PA, USA;Liu Yang, Division of Applied Mathematics, Brown University Providence, RI, USA</t>
         </is>
       </c>
       <c r="O18" t="inlineStr"/>
       <c r="P18" t="inlineStr">
         <is>
-          <t>https://openalex.org/W1534707631; https://openalex.org/W1573640198; https://openalex.org/W1594031697; https://openalex.org/W1604329830; https://openalex.org/W2149706766; https://openalex.org/W3085162807</t>
+          <t>https://openalex.org/W196871588; https://openalex.org/W1538131130; https://openalex.org/W1543241987; https://openalex.org/W1731081199; https://openalex.org/W1856502440; https://openalex.org/W1899249567; https://openalex.org/W1972005403; https://openalex.org/W1972576201; https://openalex.org/W1976068300; https://openalex.org/W1979769287; https://openalex.org/W2000359198; https://openalex.org/W2002355073; https://openalex.org/W2017880874; https://openalex.org/W2018159038; https://openalex.org/W2019465613; https://openalex.org/W2020561998; https://openalex.org/W2025444507; https://openalex.org/W2060229389; https://openalex.org/W2072072671; https://openalex.org/W2099471712; https://openalex.org/W2101371964; https://openalex.org/W2125645174; https://openalex.org/W2134164499; https://openalex.org/W2142894919; https://openalex.org/W2143225719; https://openalex.org/W2149498546; https://openalex.org/W2158985775; https://openalex.org/W2194775991; https://openalex.org/W2212370034; https://openalex.org/W2234882433; https://openalex.org/W2239232218; https://openalex.org/W2261689926; https://openalex.org/W2277172374; https://openalex.org/W2323851192; https://openalex.org/W2402144811; https://openalex.org/W2474090883; https://openalex.org/W2486824498; https://openalex.org/W2507348356; https://openalex.org/W2534240011; https://openalex.org/W2550848904; https://openalex.org/W2551156993; https://openalex.org/W2558748708; https://openalex.org/W2573864470; https://openalex.org/W2600297185; https://openalex.org/W2605147767; https://openalex.org/W2619381903; https://openalex.org/W2742127985; https://openalex.org/W2749028154; https://openalex.org/W2777417212; https://openalex.org/W2783378529; https://openalex.org/W2786232134; https://openalex.org/W2787931125; https://openalex.org/W2803629276; https://openalex.org/W2809090039; https://openalex.org/W2810026216; https://openalex.org/W2811199191; https://openalex.org/W2856628251; https://openalex.org/W2884775584; https://openalex.org/W2886802770; https://openalex.org/W2887569307; https://openalex.org/W2890889625; https://openalex.org/W2890968382; https://openalex.org/W2893749619; https://openalex.org/W2893813411; https://openalex.org/W2896549049; https://openalex.org/W2897097528; https://openalex.org/W2899283552; https://openalex.org/W2899971035; https://openalex.org/W2900369848; https://openalex.org/W2901203181; https://openalex.org/W2907047316; https://openalex.org/W2908541468; https://openalex.org/W2909320927; https://openalex.org/W2912389156; https://openalex.org/W2912465314; https://openalex.org/W2912649832; https://openalex.org/W2913323966; https://openalex.org/W2914483840; https://openalex.org/W2914520121; https://openalex.org/W2919958648; https://openalex.org/W2936357167; https://openalex.org/W2945102878; https://openalex.org/W2946794331; https://openalex.org/W2946866513; https://openalex.org/W2947072793; https://openalex.org/W2951392159; https://openalex.org/W2952046647; https://openalex.org/W2959995783; https://openalex.org/W2962793481; https://openalex.org/W2963021886; https://openalex.org/W2963063862; https://openalex.org/W2963095610; https://openalex.org/W2963190151; https://openalex.org/W2963518130; https://openalex.org/W2963634130; https://openalex.org/W2963716063; https://openalex.org/W2963755523; https://openalex.org/W2963901342; https://openalex.org/W2964059111; https://openalex.org/W2964088238; https://openalex.org/W2964121744; https://openalex.org/W2964135722; https://openalex.org/W2964212578; https://openalex.org/W2964268978; https://openalex.org/W2966284335; https://openalex.org/W2969381807; https://openalex.org/W2970100546; https://openalex.org/W2970971581; https://openalex.org/W2971095480; https://openalex.org/W2971343405; https://openalex.org/W2972153210; https://openalex.org/W2973886134; https://openalex.org/W2975003945; https://openalex.org/W2977109506; https://openalex.org/W2978281981; https://openalex.org/W2979712029; https://openalex.org/W2979786244; https://openalex.org/W2980147119; https://openalex.org/W2980592884; https://openalex.org/W2980973551; https://openalex.org/W2983902802; https://openalex.org/W2991298115; https://openalex.org/W2991550674; https://openalex.org/W2994626356; https://openalex.org/W2994747787; https://openalex.org/W2997814214; https://openalex.org/W2999026783; https://openalex.org/W2999467285; https://openalex.org/W3003747211; https://openalex.org/W3003922491; https://openalex.org/W3004450693; https://openalex.org/W3005610174; https://openalex.org/W3007470329; https://openalex.org/W3007740214; https://openalex.org/W3008453832; https://openalex.org/W3009784374; https://openalex.org/W3010849941; https://openalex.org/W3011147100; https://openalex.org/W3011806874; https://openalex.org/W3012417314; https://openalex.org/W3012621877; https://openalex.org/W3014009018; https://openalex.org/W3014468003; https://openalex.org/W3015176898; https://openalex.org/W3015606043; https://openalex.org/W3015865829; https://openalex.org/W3016703299; https://openalex.org/W3022657828; https://openalex.org/W3023982288; https://openalex.org/W3025645353; https://openalex.org/W3026222427; https://openalex.org/W3028316595; https://openalex.org/W3028529071; https://openalex.org/W3035493266; https://openalex.org/W3036843665; https://openalex.org/W3037090957; https://openalex.org/W3039304986; https://openalex.org/W3040277050; https://openalex.org/W3041984619; https://openalex.org/W3043174105; https://openalex.org/W3043516796; https://openalex.org/W3045146186; https://openalex.org/W3046173836; https://openalex.org/W3047001618; https://openalex.org/W3048241795; https://openalex.org/W3049075514; https://openalex.org/W3080393992; https://openalex.org/W3081814969; https://openalex.org/W3082908155; https://openalex.org/W3082977546; https://openalex.org/W3084017095; https://openalex.org/W3088681382; https://openalex.org/W3088691598; https://openalex.org/W3088877001; https://openalex.org/W3093018961; https://openalex.org/W3093190107; https://openalex.org/W3093786597; https://openalex.org/W3093990252; https://openalex.org/W3096173239; https://openalex.org/W3096732413; https://openalex.org/W3098172061; https://openalex.org/W3098195931; https://openalex.org/W3098370560; https://openalex.org/W3098546160; https://openalex.org/W3098951945; https://openalex.org/W3099849883; https://openalex.org/W3100156752; https://openalex.org/W3101260193; https://openalex.org/W3101396145; https://openalex.org/W3102139197; https://openalex.org/W3102569296; https://openalex.org/W3102697518; https://openalex.org/W3102845444; https://openalex.org/W3102921872; https://openalex.org/W3103242287; https://openalex.org/W3104150464; https://openalex.org/W3104873019; https://openalex.org/W3105982350; https://openalex.org/W3106050203; https://openalex.org/W3107691001; https://openalex.org/W3107973042; https://openalex.org/W3112233611; https://openalex.org/W3112264320; https://openalex.org/W3116268267; https://openalex.org/W3118310857; https://openalex.org/W3125167458; https://openalex.org/W3128400532; https://openalex.org/W3129530645; https://openalex.org/W3129610195; https://openalex.org/W3132277775; https://openalex.org/W3133338006; https://openalex.org/W3133608513; https://openalex.org/W3137240924; https://openalex.org/W3137474564; https://openalex.org/W3138463430; https://openalex.org/W3145000844; https://openalex.org/W3148629269; https://openalex.org/W3168386838; https://openalex.org/W3181271387; https://openalex.org/W3201460085; https://openalex.org/W3207890637; https://openalex.org/W4230953281; https://openalex.org/W4234008654; https://openalex.org/W6694756022; https://openalex.org/W6713134421; https://openalex.org/W6755308174; https://openalex.org/W6763197053; https://openalex.org/W6787451610</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>Successor cardinal;Artificial intelligence;Computer science;Decision tree;Machine learning;Subject (documents);ID3 algorithm;Decision tree learning;Incremental decision tree;World Wide Web;Mathematics</t>
+          <t>Computer science;Artificial intelligence;Machine learning;Multiphysics;Inference;Artificial neural network;Physical law;Field (mathematics);Discretization;Kernel method;Deep learning;Theoretical computer science;Mathematics;Support vector machine;Finite element method</t>
         </is>
       </c>
       <c r="R18" t="inlineStr"/>
-      <c r="S18" t="inlineStr">
-        <is>
-          <t>Algorithms for constructing decision trees are among the most well known and widely used of all machine learning methods. Among decision tree algorithms, J. Ross Quinlan's ID3 and its successor, C4.5, are probably the most popular in the machine learning community. These algorithms and variations on them have been the subject of numerous research papers since Quinlan introduced ID3. Until recently, most researchers looking for an introduction to decision trees turned to Quinlan's seminal 1986 Machine Learning journal article [Quinlan, 1986]. In his new book, C4.5: Programs for Machine Learning, Quinlan has put together a definitive, much needed description of his complete system, including the latest developments. As such, this book will be a welcome addition to the library of many researchers and students.</t>
-        </is>
-      </c>
-      <c r="T18" t="inlineStr"/>
-      <c r="U18" t="inlineStr"/>
-      <c r="V18" t="inlineStr"/>
-      <c r="W18" t="inlineStr"/>
+      <c r="S18" t="inlineStr"/>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="U18" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="V18" t="inlineStr">
+        <is>
+          <t>422</t>
+        </is>
+      </c>
+      <c r="W18" t="inlineStr">
+        <is>
+          <t>440</t>
+        </is>
+      </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Steven L. Salzberg, 1994, </t>
+          <t>George Em Karniadakis, 2021, Nature Reviews Physics</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Steven L. Salzberg, 1994, </t>
+          <t>George Em Karniadakis, 2021, Nature Reviews Physics</t>
         </is>
       </c>
     </row>
@@ -2008,36 +2032,36 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>https://openalex.org/W3163993681</t>
+          <t>https://openalex.org/W1601795611</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1038/s42254-021-00314-5</t>
+          <t>https://doi.org/10.1108/03684920710743466</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Physics-informed machine learning</t>
+          <t>Pattern Recognition and Machine Learning</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Nature Reviews Physics</t>
+          <t>Kybernetes</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Nature Reviews Physics</t>
+          <t>Kybernetes</t>
         </is>
       </c>
       <c r="H19" t="n">
-        <v>2021</v>
+        <v>2007</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>review</t>
+          <t>article</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
@@ -2046,60 +2070,48 @@
         </is>
       </c>
       <c r="K19" t="n">
-        <v>6698</v>
-      </c>
-      <c r="L19" t="inlineStr">
-        <is>
-          <t>George Em Karniadakis;Ioannis G. Kevrekidis;Lu Lu;Paris Perdikaris;Sifan Wang;Liu Yang</t>
-        </is>
-      </c>
+        <v>8434</v>
+      </c>
+      <c r="L19" t="inlineStr"/>
       <c r="M19" t="inlineStr"/>
-      <c r="N19" t="inlineStr">
-        <is>
-          <t>George Em Karniadakis, Division of Applied Mathematics, Brown University Providence, RI, USA;Ioannis G. Kevrekidis, Department of Applied Mathematics and Statistics, Johns Hopkins University, Baltimore, MD, USA;Ioannis G. Kevrekidis, Department of Chemical and Biomolecular Engineering, Johns Hopkins University, Baltimore, MD, USA;Lu Lu, Department of Mathematics, Massachusetts Institute of Technology, Cambridge, MA, USA;Paris Perdikaris, Department of Mechanical Engineering and Applied Mechanics, University of Pennsylvania, Philadelphia, PA, USA;Sifan Wang, Graduate Group in Applied Mathematics and Computational Science, University of Pennsylvania, Philadelphia, PA, USA;Liu Yang, Division of Applied Mathematics, Brown University Providence, RI, USA</t>
-        </is>
-      </c>
+      <c r="N19" t="inlineStr"/>
       <c r="O19" t="inlineStr"/>
-      <c r="P19" t="inlineStr">
-        <is>
-          <t>https://openalex.org/W196871588; https://openalex.org/W1538131130; https://openalex.org/W1543241987; https://openalex.org/W1731081199; https://openalex.org/W1856502440; https://openalex.org/W1899249567; https://openalex.org/W1972005403; https://openalex.org/W1972576201; https://openalex.org/W1976068300; https://openalex.org/W1979769287; https://openalex.org/W2000359198; https://openalex.org/W2002355073; https://openalex.org/W2017880874; https://openalex.org/W2018159038; https://openalex.org/W2019465613; https://openalex.org/W2020561998; https://openalex.org/W2025444507; https://openalex.org/W2060229389; https://openalex.org/W2072072671; https://openalex.org/W2099471712; https://openalex.org/W2101371964; https://openalex.org/W2125645174; https://openalex.org/W2134164499; https://openalex.org/W2142894919; https://openalex.org/W2143225719; https://openalex.org/W2149498546; https://openalex.org/W2158985775; https://openalex.org/W2194775991; https://openalex.org/W2212370034; https://openalex.org/W2234882433; https://openalex.org/W2239232218; https://openalex.org/W2261689926; https://openalex.org/W2277172374; https://openalex.org/W2323851192; https://openalex.org/W2402144811; https://openalex.org/W2474090883; https://openalex.org/W2486824498; https://openalex.org/W2507348356; https://openalex.org/W2534240011; https://openalex.org/W2550848904; https://openalex.org/W2551156993; https://openalex.org/W2558748708; https://openalex.org/W2573864470; https://openalex.org/W2600297185; https://openalex.org/W2605147767; https://openalex.org/W2619381903; https://openalex.org/W2742127985; https://openalex.org/W2749028154; https://openalex.org/W2777417212; https://openalex.org/W2783378529; https://openalex.org/W2786232134; https://openalex.org/W2787931125; https://openalex.org/W2803629276; https://openalex.org/W2809090039; https://openalex.org/W2810026216; https://openalex.org/W2811199191; https://openalex.org/W2856628251; https://openalex.org/W2884775584; https://openalex.org/W2886802770; https://openalex.org/W2887569307; https://openalex.org/W2890889625; https://openalex.org/W2890968382; https://openalex.org/W2893749619; https://openalex.org/W2893813411; https://openalex.org/W2896549049; https://openalex.org/W2897097528; https://openalex.org/W2899283552; https://openalex.org/W2899971035; https://openalex.org/W2900369848; https://openalex.org/W2901203181; https://openalex.org/W2907047316; https://openalex.org/W2908541468; https://openalex.org/W2909320927; https://openalex.org/W2912389156; https://openalex.org/W2912465314; https://openalex.org/W2912649832; https://openalex.org/W2913323966; https://openalex.org/W2914483840; https://openalex.org/W2914520121; https://openalex.org/W2919958648; https://openalex.org/W2936357167; https://openalex.org/W2945102878; https://openalex.org/W2946794331; https://openalex.org/W2946866513; https://openalex.org/W2947072793; https://openalex.org/W2951392159; https://openalex.org/W2952046647; https://openalex.org/W2959995783; https://openalex.org/W2962793481; https://openalex.org/W2963021886; https://openalex.org/W2963063862; https://openalex.org/W2963095610; https://openalex.org/W2963190151; https://openalex.org/W2963518130; https://openalex.org/W2963634130; https://openalex.org/W2963716063; https://openalex.org/W2963755523; https://openalex.org/W2963901342; https://openalex.org/W2964059111; https://openalex.org/W2964088238; https://openalex.org/W2964121744; https://openalex.org/W2964135722; https://openalex.org/W2964212578; https://openalex.org/W2964268978; https://openalex.org/W2966284335; https://openalex.org/W2969381807; https://openalex.org/W2970100546; https://openalex.org/W2970971581; https://openalex.org/W2971095480; https://openalex.org/W2971343405; https://openalex.org/W2972153210; https://openalex.org/W2973886134; https://openalex.org/W2975003945; https://openalex.org/W2977109506; https://openalex.org/W2978281981; https://openalex.org/W2979712029; https://openalex.org/W2979786244; https://openalex.org/W2980147119; https://openalex.org/W2980592884; https://openalex.org/W2980973551; https://openalex.org/W2983902802; https://openalex.org/W2991298115; https://openalex.org/W2991550674; https://openalex.org/W2994626356; https://openalex.org/W2994747787; https://openalex.org/W2997814214; https://openalex.org/W2999026783; https://openalex.org/W2999467285; https://openalex.org/W3003747211; https://openalex.org/W3003922491; https://openalex.org/W3004450693; https://openalex.org/W3005610174; https://openalex.org/W3007470329; https://openalex.org/W3007740214; https://openalex.org/W3008453832; https://openalex.org/W3009784374; https://openalex.org/W3010849941; https://openalex.org/W3011147100; https://openalex.org/W3011806874; https://openalex.org/W3012417314; https://openalex.org/W3012621877; https://openalex.org/W3014009018; https://openalex.org/W3014468003; https://openalex.org/W3015176898; https://openalex.org/W3015606043; https://openalex.org/W3015865829; https://openalex.org/W3016703299; https://openalex.org/W3022657828; https://openalex.org/W3023982288; https://openalex.org/W3025645353; https://openalex.org/W3026222427; https://openalex.org/W3028316595; https://openalex.org/W3028529071; https://openalex.org/W3035493266; https://openalex.org/W3036843665; https://openalex.org/W3037090957; https://openalex.org/W3039304986; https://openalex.org/W3040277050; https://openalex.org/W3041984619; https://openalex.org/W3043174105; https://openalex.org/W3043516796; https://openalex.org/W3045146186; https://openalex.org/W3046173836; https://openalex.org/W3047001618; https://openalex.org/W3048241795; https://openalex.org/W3049075514; https://openalex.org/W3080393992; https://openalex.org/W3081814969; https://openalex.org/W3082908155; https://openalex.org/W3082977546; https://openalex.org/W3084017095; https://openalex.org/W3088681382; https://openalex.org/W3088691598; https://openalex.org/W3088877001; https://openalex.org/W3093018961; https://openalex.org/W3093190107; https://openalex.org/W3093786597; https://openalex.org/W3093990252; https://openalex.org/W3096173239; https://openalex.org/W3096732413; https://openalex.org/W3098172061; https://openalex.org/W3098195931; https://openalex.org/W3098370560; https://openalex.org/W3098546160; https://openalex.org/W3098951945; https://openalex.org/W3099849883; https://openalex.org/W3100156752; https://openalex.org/W3101260193; https://openalex.org/W3101396145; https://openalex.org/W3102139197; https://openalex.org/W3102569296; https://openalex.org/W3102697518; https://openalex.org/W3102845444; https://openalex.org/W3102921872; https://openalex.org/W3103242287; https://openalex.org/W3104150464; https://openalex.org/W3104873019; https://openalex.org/W3105982350; https://openalex.org/W3106050203; https://openalex.org/W3107691001; https://openalex.org/W3107973042; https://openalex.org/W3112233611; https://openalex.org/W3112264320; https://openalex.org/W3116268267; https://openalex.org/W3118310857; https://openalex.org/W3125167458; https://openalex.org/W3128400532; https://openalex.org/W3129530645; https://openalex.org/W3129610195; https://openalex.org/W3132277775; https://openalex.org/W3133338006; https://openalex.org/W3133608513; https://openalex.org/W3137240924; https://openalex.org/W3137474564; https://openalex.org/W3138463430; https://openalex.org/W3145000844; https://openalex.org/W3148629269; https://openalex.org/W3168386838; https://openalex.org/W3181271387; https://openalex.org/W3201460085; https://openalex.org/W3207890637; https://openalex.org/W4230953281; https://openalex.org/W4234008654; https://openalex.org/W6694756022; https://openalex.org/W6713134421; https://openalex.org/W6755308174; https://openalex.org/W6763197053; https://openalex.org/W6787451610</t>
-        </is>
-      </c>
+      <c r="P19" t="inlineStr"/>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>Computer science;Artificial intelligence;Machine learning;Multiphysics;Inference;Artificial neural network;Physical law;Field (mathematics);Discretization;Kernel method;Deep learning;Theoretical computer science;Mathematics;Support vector machine;Finite element method</t>
+          <t>Computer science;Cybernetics;Artificial intelligence;Machine learning</t>
         </is>
       </c>
       <c r="R19" t="inlineStr"/>
       <c r="S19" t="inlineStr"/>
       <c r="T19" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>36</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>2</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>422</t>
+          <t>275</t>
         </is>
       </c>
       <c r="W19" t="inlineStr">
         <is>
-          <t>440</t>
+          <t>275</t>
         </is>
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>George Em Karniadakis, 2021, Nature Reviews Physics</t>
+          <t>NA, 2007, Kybernetes</t>
         </is>
       </c>
       <c r="Y19" t="inlineStr">
         <is>
-          <t>George Em Karniadakis, 2021, Nature Reviews Physics</t>
+          <t>NA, 2007, Kybernetes</t>
         </is>
       </c>
     </row>
@@ -2111,32 +2123,20 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>https://openalex.org/W1601795611</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.1108/03684920710743466</t>
-        </is>
-      </c>
+          <t>https://openalex.org/W1504694836</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Pattern Recognition and Machine Learning</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>Kybernetes</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>Kybernetes</t>
-        </is>
-      </c>
+          <t>Programs for Machine Learning</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr"/>
       <c r="H20" t="n">
-        <v>2007</v>
+        <v>1994</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
@@ -2149,48 +2149,48 @@
         </is>
       </c>
       <c r="K20" t="n">
-        <v>8434</v>
-      </c>
-      <c r="L20" t="inlineStr"/>
+        <v>5808</v>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>Steven L. Salzberg;Alberto M. Segre</t>
+        </is>
+      </c>
       <c r="M20" t="inlineStr"/>
-      <c r="N20" t="inlineStr"/>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>Steven L. Salzberg, Johns Hopkins University (</t>
+        </is>
+      </c>
       <c r="O20" t="inlineStr"/>
-      <c r="P20" t="inlineStr"/>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>https://openalex.org/W1534707631; https://openalex.org/W1573640198; https://openalex.org/W1594031697; https://openalex.org/W1604329830; https://openalex.org/W2149706766; https://openalex.org/W3085162807</t>
+        </is>
+      </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>Computer science;Cybernetics;Artificial intelligence;Machine learning</t>
+          <t>Successor cardinal;Artificial intelligence;Computer science;Decision tree;Machine learning;Subject (documents);ID3 algorithm;Decision tree learning;Incremental decision tree;World Wide Web;Mathematics</t>
         </is>
       </c>
       <c r="R20" t="inlineStr"/>
-      <c r="S20" t="inlineStr"/>
-      <c r="T20" t="inlineStr">
-        <is>
-          <t>36</t>
-        </is>
-      </c>
-      <c r="U20" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="V20" t="inlineStr">
-        <is>
-          <t>275</t>
-        </is>
-      </c>
-      <c r="W20" t="inlineStr">
-        <is>
-          <t>275</t>
-        </is>
-      </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>Algorithms for constructing decision trees are among the most well known and widely used of all machine learning methods. Among decision tree algorithms, J. Ross Quinlan's ID3 and its successor, C4.5, are probably the most popular in the machine learning community. These algorithms and variations on them have been the subject of numerous research papers since Quinlan introduced ID3. Until recently, most researchers looking for an introduction to decision trees turned to Quinlan's seminal 1986 Machine Learning journal article [Quinlan, 1986]. In his new book, C4.5: Programs for Machine Learning, Quinlan has put together a definitive, much needed description of his complete system, including the latest developments. As such, this book will be a welcome addition to the library of many researchers and students.</t>
+        </is>
+      </c>
+      <c r="T20" t="inlineStr"/>
+      <c r="U20" t="inlineStr"/>
+      <c r="V20" t="inlineStr"/>
+      <c r="W20" t="inlineStr"/>
       <c r="X20" t="inlineStr">
         <is>
-          <t>NA, 2007, Kybernetes</t>
+          <t xml:space="preserve">Steven L. Salzberg, 1994, </t>
         </is>
       </c>
       <c r="Y20" t="inlineStr">
         <is>
-          <t>NA, 2007, Kybernetes</t>
+          <t xml:space="preserve">Steven L. Salzberg, 1994, </t>
         </is>
       </c>
     </row>
@@ -2240,7 +2240,7 @@
         </is>
       </c>
       <c r="K21" t="n">
-        <v>9781</v>
+        <v>9782</v>
       </c>
       <c r="L21" t="inlineStr">
         <is>
@@ -2327,7 +2327,7 @@
         </is>
       </c>
       <c r="K22" t="n">
-        <v>7873</v>
+        <v>7881</v>
       </c>
       <c r="L22" t="inlineStr">
         <is>
@@ -2422,7 +2422,7 @@
         </is>
       </c>
       <c r="K23" t="n">
-        <v>4455</v>
+        <v>4463</v>
       </c>
       <c r="L23" t="inlineStr">
         <is>
@@ -2525,7 +2525,7 @@
         </is>
       </c>
       <c r="K24" t="n">
-        <v>5895</v>
+        <v>5899</v>
       </c>
       <c r="L24" t="inlineStr">
         <is>
@@ -2768,32 +2768,32 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>https://openalex.org/W2155653793</t>
+          <t>https://openalex.org/W2009086942</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1016/s0031-3203(96)00142-2</t>
+          <t>https://doi.org/10.1198/tech.2007.s518</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr">
         <is>
-          <t>The use of the area under the ROC curve in the evaluation of machine learning algorithms</t>
+          <t>Pattern Recognition and Machine Learning</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Pattern Recognition</t>
+          <t>Technometrics</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Pattern Recognition</t>
+          <t>Technometrics</t>
         </is>
       </c>
       <c r="H27" t="n">
-        <v>1997</v>
+        <v>2007</v>
       </c>
       <c r="I27" t="inlineStr">
         <is>
@@ -2806,60 +2806,60 @@
         </is>
       </c>
       <c r="K27" t="n">
-        <v>7241</v>
+        <v>4652</v>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>Andrew P. Bradley</t>
+          <t>Radford M. Neal</t>
         </is>
       </c>
       <c r="M27" t="inlineStr"/>
       <c r="N27" t="inlineStr">
         <is>
-          <t>Andrew P. Bradley, Cooperative Research Centre for Sensor Signal and Information Processing, Department of Electrical and Computer Engineering, The University of Queensland, QLD 4072, Australia</t>
+          <t>Radford M. Neal, University of Toronto</t>
         </is>
       </c>
       <c r="O27" t="inlineStr"/>
-      <c r="P27" t="inlineStr">
-        <is>
-          <t>https://openalex.org/W102612133; https://openalex.org/W1479940792; https://openalex.org/W1488460165; https://openalex.org/W1489095897; https://openalex.org/W1515026043; https://openalex.org/W1533986854; https://openalex.org/W1541145887; https://openalex.org/W1587362683; https://openalex.org/W1588861010; https://openalex.org/W1594031697; https://openalex.org/W1623080549; https://openalex.org/W1704669313; https://openalex.org/W1770825568; https://openalex.org/W1784695092; https://openalex.org/W1967760155; https://openalex.org/W1969341260; https://openalex.org/W1969557815; https://openalex.org/W1983523174; https://openalex.org/W1989164753; https://openalex.org/W1995023359; https://openalex.org/W2002096058; https://openalex.org/W2026980413; https://openalex.org/W2049172236; https://openalex.org/W2050206309; https://openalex.org/W2060136512; https://openalex.org/W2102150307; https://openalex.org/W2110323455; https://openalex.org/W2116939452; https://openalex.org/W2117897510; https://openalex.org/W2125055259; https://openalex.org/W2135346934; https://openalex.org/W2145224695; https://openalex.org/W2157825442; https://openalex.org/W2322002063; https://openalex.org/W2766736793; https://openalex.org/W2921629193; https://openalex.org/W2988864014; https://openalex.org/W3015981925; https://openalex.org/W3085162807; https://openalex.org/W3137161744; https://openalex.org/W4233107852; https://openalex.org/W4254952533; https://openalex.org/W4300993416; https://openalex.org/W4400445037; https://openalex.org/W6629338572; https://openalex.org/W6632481002; https://openalex.org/W6635398855; https://openalex.org/W6642591540; https://openalex.org/W6650814897; https://openalex.org/W6676534550; https://openalex.org/W6682610290; https://openalex.org/W7020983598</t>
-        </is>
-      </c>
+      <c r="P27" t="inlineStr"/>
       <c r="Q27" t="inlineStr">
         <is>
-          <t>Algorithm;Receiver operating characteristic;Machine learning;Artificial intelligence;Perceptron;Computer science;Discriminant;Multilayer perceptron;Mathematics;Artificial neural network</t>
+          <t>Artificial intelligence;Computer science;Machine learning;Pattern recognition (psychology)</t>
         </is>
       </c>
       <c r="R27" t="inlineStr"/>
-      <c r="S27" t="inlineStr"/>
+      <c r="S27" t="inlineStr">
+        <is>
+          <t>(2007). Pattern Recognition and Machine Learning. Technometrics: Vol. 49, No. 3, pp. 366-366.</t>
+        </is>
+      </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>49</t>
         </is>
       </c>
       <c r="U27" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>3</t>
         </is>
       </c>
       <c r="V27" t="inlineStr">
         <is>
-          <t>1145</t>
+          <t>366</t>
         </is>
       </c>
       <c r="W27" t="inlineStr">
         <is>
-          <t>1159</t>
+          <t>366</t>
         </is>
       </c>
       <c r="X27" t="inlineStr">
         <is>
-          <t>Andrew P. Bradley, 1997, Pattern Recognition</t>
+          <t>Radford M. Neal, 2007, Technometrics</t>
         </is>
       </c>
       <c r="Y27" t="inlineStr">
         <is>
-          <t>Andrew P. Bradley, 1997, Pattern Recognition</t>
+          <t>Radford M. Neal, 2007, Technometrics</t>
         </is>
       </c>
     </row>
@@ -2871,32 +2871,32 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>https://openalex.org/W2009086942</t>
+          <t>https://openalex.org/W2155653793</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1198/tech.2007.s518</t>
+          <t>https://doi.org/10.1016/s0031-3203(96)00142-2</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Pattern Recognition and Machine Learning</t>
+          <t>The use of the area under the ROC curve in the evaluation of machine learning algorithms</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Technometrics</t>
+          <t>Pattern Recognition</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Technometrics</t>
+          <t>Pattern Recognition</t>
         </is>
       </c>
       <c r="H28" t="n">
-        <v>2007</v>
+        <v>1997</v>
       </c>
       <c r="I28" t="inlineStr">
         <is>
@@ -2909,60 +2909,60 @@
         </is>
       </c>
       <c r="K28" t="n">
-        <v>4652</v>
+        <v>7247</v>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>Radford M. Neal</t>
+          <t>Andrew P. Bradley</t>
         </is>
       </c>
       <c r="M28" t="inlineStr"/>
       <c r="N28" t="inlineStr">
         <is>
-          <t>Radford M. Neal, University of Toronto</t>
+          <t>Andrew P. Bradley, Cooperative Research Centre for Sensor Signal and Information Processing, Department of Electrical and Computer Engineering, The University of Queensland, QLD 4072, Australia</t>
         </is>
       </c>
       <c r="O28" t="inlineStr"/>
-      <c r="P28" t="inlineStr"/>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>https://openalex.org/W102612133; https://openalex.org/W1479940792; https://openalex.org/W1488460165; https://openalex.org/W1489095897; https://openalex.org/W1515026043; https://openalex.org/W1533986854; https://openalex.org/W1541145887; https://openalex.org/W1587362683; https://openalex.org/W1588861010; https://openalex.org/W1594031697; https://openalex.org/W1623080549; https://openalex.org/W1704669313; https://openalex.org/W1770825568; https://openalex.org/W1784695092; https://openalex.org/W1967760155; https://openalex.org/W1969341260; https://openalex.org/W1969557815; https://openalex.org/W1983523174; https://openalex.org/W1989164753; https://openalex.org/W1995023359; https://openalex.org/W2002096058; https://openalex.org/W2026980413; https://openalex.org/W2049172236; https://openalex.org/W2050206309; https://openalex.org/W2060136512; https://openalex.org/W2102150307; https://openalex.org/W2110323455; https://openalex.org/W2116939452; https://openalex.org/W2117897510; https://openalex.org/W2125055259; https://openalex.org/W2135346934; https://openalex.org/W2145224695; https://openalex.org/W2157825442; https://openalex.org/W2322002063; https://openalex.org/W2766736793; https://openalex.org/W2921629193; https://openalex.org/W2988864014; https://openalex.org/W3015981925; https://openalex.org/W3085162807; https://openalex.org/W3137161744; https://openalex.org/W4233107852; https://openalex.org/W4254952533; https://openalex.org/W4300993416; https://openalex.org/W4400445037; https://openalex.org/W6629338572; https://openalex.org/W6632481002; https://openalex.org/W6635398855; https://openalex.org/W6642591540; https://openalex.org/W6650814897; https://openalex.org/W6676534550; https://openalex.org/W6682610290; https://openalex.org/W7020983598</t>
+        </is>
+      </c>
       <c r="Q28" t="inlineStr">
         <is>
-          <t>Artificial intelligence;Computer science;Machine learning;Pattern recognition (psychology)</t>
+          <t>Algorithm;Receiver operating characteristic;Machine learning;Artificial intelligence;Perceptron;Computer science;Discriminant;Multilayer perceptron;Mathematics;Artificial neural network</t>
         </is>
       </c>
       <c r="R28" t="inlineStr"/>
-      <c r="S28" t="inlineStr">
-        <is>
-          <t>(2007). Pattern Recognition and Machine Learning. Technometrics: Vol. 49, No. 3, pp. 366-366.</t>
-        </is>
-      </c>
+      <c r="S28" t="inlineStr"/>
       <c r="T28" t="inlineStr">
         <is>
-          <t>49</t>
+          <t>30</t>
         </is>
       </c>
       <c r="U28" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="V28" t="inlineStr">
         <is>
-          <t>366</t>
+          <t>1145</t>
         </is>
       </c>
       <c r="W28" t="inlineStr">
         <is>
-          <t>366</t>
+          <t>1159</t>
         </is>
       </c>
       <c r="X28" t="inlineStr">
         <is>
-          <t>Radford M. Neal, 2007, Technometrics</t>
+          <t>Andrew P. Bradley, 1997, Pattern Recognition</t>
         </is>
       </c>
       <c r="Y28" t="inlineStr">
         <is>
-          <t>Radford M. Neal, 2007, Technometrics</t>
+          <t>Andrew P. Bradley, 1997, Pattern Recognition</t>
         </is>
       </c>
     </row>
@@ -2974,36 +2974,36 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>https://openalex.org/W2131241448</t>
+          <t>https://openalex.org/W2934399013</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>https://doi.org/10.48550/arxiv.1206.2944</t>
+          <t>https://doi.org/10.1056/nejmra1814259</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Practical Bayesian Optimization of Machine Learning Algorithms</t>
+          <t>Machine Learning in Medicine</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>arXiv (Cornell University)</t>
+          <t>New England Journal of Medicine</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>arXiv (Cornell University)</t>
+          <t>New England Journal of Medicine</t>
         </is>
       </c>
       <c r="H29" t="n">
-        <v>2012</v>
+        <v>2019</v>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>preprint</t>
+          <t>review</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
@@ -3012,48 +3012,64 @@
         </is>
       </c>
       <c r="K29" t="n">
-        <v>5671</v>
+        <v>4020</v>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>Jasper Snoek;Hugo Larochelle;Ryan P. Adams</t>
+          <t>Alvin Rajkomar;Jay B. Dean;Isaac S. Kohane</t>
         </is>
       </c>
       <c r="M29" t="inlineStr"/>
       <c r="N29" t="inlineStr">
         <is>
-          <t>Jasper Snoek, [Department of Computer Science, University of Toronto];Hugo Larochelle, Department of Computer Science, University of Sherbrooke,;Ryan P. Adams, School of Engineering &amp; Applied Sciences Harvard University</t>
+          <t>Alvin Rajkomar, From Google, Mountain View, CA (A.R., J.D.);and the Department of Biomedical Informatics, Harvard Medical School, Boston (I.K.);Alvin Rajkomar, Google, Mountain View, CA;Jay B. Dean, From Google, Mountain View, CA (A.R., J.D.);and the Department of Biomedical Informatics, Harvard Medical School, Boston (I.K.);Jay B. Dean, Google, Mountain View, CA;Isaac S. Kohane, From Google, Mountain View, CA (A.R., J.D.);and the Department of Biomedical Informatics, Harvard Medical School, Boston (I.K.);Isaac S. Kohane, Department of Biomedical Informatics, Harvard Medical School, Boston</t>
         </is>
       </c>
       <c r="O29" t="inlineStr"/>
       <c r="P29" t="inlineStr">
         <is>
-          <t>https://openalex.org/W60686164; https://openalex.org/W78356000; https://openalex.org/W84569508; https://openalex.org/W1497675750; https://openalex.org/W1746819321; https://openalex.org/W1973333099; https://openalex.org/W2061144551; https://openalex.org/W2097998348; https://openalex.org/W2099201756; https://openalex.org/W2106411961; https://openalex.org/W2106869737; https://openalex.org/W2119595900; https://openalex.org/W2129458072; https://openalex.org/W2132984949; https://openalex.org/W2141125852; https://openalex.org/W2147196093; https://openalex.org/W2151238122; https://openalex.org/W2165599843; https://openalex.org/W2189424119; https://openalex.org/W2197776371; https://openalex.org/W2951665052; https://openalex.org/W2964172739; https://openalex.org/W3118608800</t>
+          <t>https://openalex.org/W1524493166; https://openalex.org/W1529983430; https://openalex.org/W2005440935; https://openalex.org/W2009184733; https://openalex.org/W2009954208; https://openalex.org/W2027540165; https://openalex.org/W2033163059; https://openalex.org/W2033609349; https://openalex.org/W2043092953; https://openalex.org/W2054076956; https://openalex.org/W2083721602; https://openalex.org/W2096849439; https://openalex.org/W2103018059; https://openalex.org/W2103889389; https://openalex.org/W2119472226; https://openalex.org/W2137767404; https://openalex.org/W2147246123; https://openalex.org/W2166187912; https://openalex.org/W2167414941; https://openalex.org/W2174931596; https://openalex.org/W2267932926; https://openalex.org/W2276530525; https://openalex.org/W2337116044; https://openalex.org/W2415841860; https://openalex.org/W2468431774; https://openalex.org/W2512902140; https://openalex.org/W2515682654; https://openalex.org/W2528491735; https://openalex.org/W2530247697; https://openalex.org/W2548723212; https://openalex.org/W2557738935; https://openalex.org/W2581082771; https://openalex.org/W2598272139; https://openalex.org/W2732701910; https://openalex.org/W2734356183; https://openalex.org/W2738975713; https://openalex.org/W2740060821; https://openalex.org/W2752747624; https://openalex.org/W2753059860; https://openalex.org/W2754518417; https://openalex.org/W2758348074; https://openalex.org/W2762741128; https://openalex.org/W2772246530; https://openalex.org/W2772723798; https://openalex.org/W2782945064; https://openalex.org/W2784499877; https://openalex.org/W2785268987; https://openalex.org/W2785526886; https://openalex.org/W2788633781; https://openalex.org/W2789894922; https://openalex.org/W2790444357; https://openalex.org/W2791819448; https://openalex.org/W2792902933; https://openalex.org/W2793267369; https://openalex.org/W2794457162; https://openalex.org/W2799837895; https://openalex.org/W2804685074; https://openalex.org/W2809453031; https://openalex.org/W2886281300; https://openalex.org/W2887623535; https://openalex.org/W2887719255; https://openalex.org/W2888109941; https://openalex.org/W2889242407; https://openalex.org/W2889494558; https://openalex.org/W2894917609; https://openalex.org/W2896385413; https://openalex.org/W2896817483; https://openalex.org/W2897434820; https://openalex.org/W2899560923; https://openalex.org/W2902802452; https://openalex.org/W2908201961; https://openalex.org/W2914579361; https://openalex.org/W2916105049; https://openalex.org/W2919115771; https://openalex.org/W3098949126; https://openalex.org/W4205374244; https://openalex.org/W4212774754; https://openalex.org/W4296220420</t>
         </is>
       </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t>Bayesian optimization;Computer science;Bayesian probability;Machine learning;Artificial intelligence;Optimization algorithm;Algorithm;Mathematical optimization;Mathematics</t>
+          <t>Download;Computer science;Data science;Medicine;Medical education;Artificial intelligence;World Wide Web</t>
         </is>
       </c>
       <c r="R29" t="inlineStr"/>
       <c r="S29" t="inlineStr">
         <is>
-          <t>Machine learning algorithms frequently require careful tuning of model hyperparameters, regularization terms, and optimization parameters. Unfortunately, this tuning is often a "black art" that requires expert experience, unwritten rules of thumb, or sometimes brute-force search. Much more appealing is the idea of developing automatic approaches which can optimize the performance of a given learning algorithm to the task at hand. In this work, we consider the automatic tuning problem within the framework of Bayesian optimization, in which a learning algorithm's generalization performance is modeled as a sample from a Gaussian process (GP). The tractable posterior distribution induced by the GP leads to efficient use of the information gathered by previous experiments, enabling optimal choices about what parameters to try next. Here we show how the effects of the Gaussian process prior and the associated inference procedure can have a large impact on the success or failure of Bayesian optimization. We show that thoughtful choices can lead to results that exceed expert-level performance in tuning machine learning algorithms. We also describe new algorithms that take into account the variable cost (duration) of learning experiments and that can leverage the presence of multiple cores for parallel experimentation. We show that these proposed algorithms improve on previous automatic procedures and can reach or surpass human expert-level optimization on a diverse set of contemporary algorithms including latent Dirichlet allocation, structured SVMs and convolutional neural networks.</t>
-        </is>
-      </c>
-      <c r="T29" t="inlineStr"/>
-      <c r="U29" t="inlineStr"/>
-      <c r="V29" t="inlineStr"/>
-      <c r="W29" t="inlineStr"/>
+          <t>Interview with Dr. Isaac Kohane on machine learning in medicine. (16:31)Download In this view of the future of medicine, patient–provider interactions are informed and supported by massive amounts of data from interactions with similar patients. These data are collected and curated to provide the latest evidence-based assessment and recommendations.</t>
+        </is>
+      </c>
+      <c r="T29" t="inlineStr">
+        <is>
+          <t>380</t>
+        </is>
+      </c>
+      <c r="U29" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="V29" t="inlineStr">
+        <is>
+          <t>1347</t>
+        </is>
+      </c>
+      <c r="W29" t="inlineStr">
+        <is>
+          <t>1358</t>
+        </is>
+      </c>
       <c r="X29" t="inlineStr">
         <is>
-          <t>Jasper Snoek, 2012, arXiv (Cornell University)</t>
+          <t>Alvin Rajkomar, 2019, New England Journal of Medicine</t>
         </is>
       </c>
       <c r="Y29" t="inlineStr">
         <is>
-          <t>Jasper Snoek, 2012, arXiv (Cornell University)</t>
+          <t>Alvin Rajkomar, 2019, New England Journal of Medicine</t>
         </is>
       </c>
     </row>
@@ -3103,7 +3119,7 @@
         </is>
       </c>
       <c r="K30" t="n">
-        <v>4564</v>
+        <v>4578</v>
       </c>
       <c r="L30" t="inlineStr">
         <is>
@@ -3168,36 +3184,36 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>https://openalex.org/W2934399013</t>
+          <t>https://openalex.org/W2131241448</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1056/nejmra1814259</t>
+          <t>https://doi.org/10.48550/arxiv.1206.2944</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Machine Learning in Medicine</t>
+          <t>Practical Bayesian Optimization of Machine Learning Algorithms</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>New England Journal of Medicine</t>
+          <t>arXiv (Cornell University)</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>New England Journal of Medicine</t>
+          <t>arXiv (Cornell University)</t>
         </is>
       </c>
       <c r="H31" t="n">
-        <v>2019</v>
+        <v>2012</v>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>review</t>
+          <t>preprint</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
@@ -3206,64 +3222,48 @@
         </is>
       </c>
       <c r="K31" t="n">
-        <v>4008</v>
+        <v>5673</v>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>Alvin Rajkomar;Jay B. Dean;Isaac S. Kohane</t>
+          <t>Jasper Snoek;Hugo Larochelle;Ryan P. Adams</t>
         </is>
       </c>
       <c r="M31" t="inlineStr"/>
       <c r="N31" t="inlineStr">
         <is>
-          <t>Alvin Rajkomar, From Google, Mountain View, CA (A.R., J.D.);and the Department of Biomedical Informatics, Harvard Medical School, Boston (I.K.);Alvin Rajkomar, Google, Mountain View, CA;Jay B. Dean, From Google, Mountain View, CA (A.R., J.D.);and the Department of Biomedical Informatics, Harvard Medical School, Boston (I.K.);Jay B. Dean, Google, Mountain View, CA;Isaac S. Kohane, From Google, Mountain View, CA (A.R., J.D.);and the Department of Biomedical Informatics, Harvard Medical School, Boston (I.K.);Isaac S. Kohane, Department of Biomedical Informatics, Harvard Medical School, Boston</t>
+          <t>Jasper Snoek, [Department of Computer Science, University of Toronto];Hugo Larochelle, Department of Computer Science, University of Sherbrooke,;Ryan P. Adams, School of Engineering &amp; Applied Sciences Harvard University</t>
         </is>
       </c>
       <c r="O31" t="inlineStr"/>
       <c r="P31" t="inlineStr">
         <is>
-          <t>https://openalex.org/W1524493166; https://openalex.org/W1529983430; https://openalex.org/W2005440935; https://openalex.org/W2009184733; https://openalex.org/W2009954208; https://openalex.org/W2027540165; https://openalex.org/W2033163059; https://openalex.org/W2033609349; https://openalex.org/W2043092953; https://openalex.org/W2054076956; https://openalex.org/W2083721602; https://openalex.org/W2096849439; https://openalex.org/W2103018059; https://openalex.org/W2103889389; https://openalex.org/W2119472226; https://openalex.org/W2137767404; https://openalex.org/W2147246123; https://openalex.org/W2166187912; https://openalex.org/W2167414941; https://openalex.org/W2174931596; https://openalex.org/W2267932926; https://openalex.org/W2276530525; https://openalex.org/W2337116044; https://openalex.org/W2415841860; https://openalex.org/W2468431774; https://openalex.org/W2512902140; https://openalex.org/W2515682654; https://openalex.org/W2528491735; https://openalex.org/W2530247697; https://openalex.org/W2548723212; https://openalex.org/W2557738935; https://openalex.org/W2581082771; https://openalex.org/W2598272139; https://openalex.org/W2732701910; https://openalex.org/W2734356183; https://openalex.org/W2738975713; https://openalex.org/W2740060821; https://openalex.org/W2752747624; https://openalex.org/W2753059860; https://openalex.org/W2754518417; https://openalex.org/W2758348074; https://openalex.org/W2762741128; https://openalex.org/W2772246530; https://openalex.org/W2772723798; https://openalex.org/W2782945064; https://openalex.org/W2784499877; https://openalex.org/W2785268987; https://openalex.org/W2785526886; https://openalex.org/W2788633781; https://openalex.org/W2789894922; https://openalex.org/W2790444357; https://openalex.org/W2791819448; https://openalex.org/W2792902933; https://openalex.org/W2793267369; https://openalex.org/W2794457162; https://openalex.org/W2799837895; https://openalex.org/W2804685074; https://openalex.org/W2809453031; https://openalex.org/W2886281300; https://openalex.org/W2887623535; https://openalex.org/W2887719255; https://openalex.org/W2888109941; https://openalex.org/W2889242407; https://openalex.org/W2889494558; https://openalex.org/W2894917609; https://openalex.org/W2896385413; https://openalex.org/W2896817483; https://openalex.org/W2897434820; https://openalex.org/W2899560923; https://openalex.org/W2902802452; https://openalex.org/W2908201961; https://openalex.org/W2914579361; https://openalex.org/W2916105049; https://openalex.org/W2919115771; https://openalex.org/W3098949126; https://openalex.org/W4205374244; https://openalex.org/W4212774754; https://openalex.org/W4296220420</t>
+          <t>https://openalex.org/W60686164; https://openalex.org/W78356000; https://openalex.org/W84569508; https://openalex.org/W1497675750; https://openalex.org/W1746819321; https://openalex.org/W1973333099; https://openalex.org/W2061144551; https://openalex.org/W2097998348; https://openalex.org/W2099201756; https://openalex.org/W2106411961; https://openalex.org/W2106869737; https://openalex.org/W2119595900; https://openalex.org/W2129458072; https://openalex.org/W2132984949; https://openalex.org/W2141125852; https://openalex.org/W2147196093; https://openalex.org/W2151238122; https://openalex.org/W2165599843; https://openalex.org/W2189424119; https://openalex.org/W2197776371; https://openalex.org/W2951665052; https://openalex.org/W2964172739; https://openalex.org/W3118608800</t>
         </is>
       </c>
       <c r="Q31" t="inlineStr">
         <is>
-          <t>Download;Computer science;Data science;Medicine;Medical education;Artificial intelligence;World Wide Web</t>
+          <t>Bayesian optimization;Computer science;Bayesian probability;Machine learning;Artificial intelligence;Optimization algorithm;Algorithm;Mathematical optimization;Mathematics</t>
         </is>
       </c>
       <c r="R31" t="inlineStr"/>
       <c r="S31" t="inlineStr">
         <is>
-          <t>Interview with Dr. Isaac Kohane on machine learning in medicine. (16:31)Download In this view of the future of medicine, patient–provider interactions are informed and supported by massive amounts of data from interactions with similar patients. These data are collected and curated to provide the latest evidence-based assessment and recommendations.</t>
-        </is>
-      </c>
-      <c r="T31" t="inlineStr">
-        <is>
-          <t>380</t>
-        </is>
-      </c>
-      <c r="U31" t="inlineStr">
-        <is>
-          <t>14</t>
-        </is>
-      </c>
-      <c r="V31" t="inlineStr">
-        <is>
-          <t>1347</t>
-        </is>
-      </c>
-      <c r="W31" t="inlineStr">
-        <is>
-          <t>1358</t>
-        </is>
-      </c>
+          <t>Machine learning algorithms frequently require careful tuning of model hyperparameters, regularization terms, and optimization parameters. Unfortunately, this tuning is often a "black art" that requires expert experience, unwritten rules of thumb, or sometimes brute-force search. Much more appealing is the idea of developing automatic approaches which can optimize the performance of a given learning algorithm to the task at hand. In this work, we consider the automatic tuning problem within the framework of Bayesian optimization, in which a learning algorithm's generalization performance is modeled as a sample from a Gaussian process (GP). The tractable posterior distribution induced by the GP leads to efficient use of the information gathered by previous experiments, enabling optimal choices about what parameters to try next. Here we show how the effects of the Gaussian process prior and the associated inference procedure can have a large impact on the success or failure of Bayesian optimization. We show that thoughtful choices can lead to results that exceed expert-level performance in tuning machine learning algorithms. We also describe new algorithms that take into account the variable cost (duration) of learning experiments and that can leverage the presence of multiple cores for parallel experimentation. We show that these proposed algorithms improve on previous automatic procedures and can reach or surpass human expert-level optimization on a diverse set of contemporary algorithms including latent Dirichlet allocation, structured SVMs and convolutional neural networks.</t>
+        </is>
+      </c>
+      <c r="T31" t="inlineStr"/>
+      <c r="U31" t="inlineStr"/>
+      <c r="V31" t="inlineStr"/>
+      <c r="W31" t="inlineStr"/>
       <c r="X31" t="inlineStr">
         <is>
-          <t>Alvin Rajkomar, 2019, New England Journal of Medicine</t>
+          <t>Jasper Snoek, 2012, arXiv (Cornell University)</t>
         </is>
       </c>
       <c r="Y31" t="inlineStr">
         <is>
-          <t>Alvin Rajkomar, 2019, New England Journal of Medicine</t>
+          <t>Jasper Snoek, 2012, arXiv (Cornell University)</t>
         </is>
       </c>
     </row>
@@ -3482,7 +3482,7 @@
         </is>
       </c>
       <c r="K34" t="n">
-        <v>8000</v>
+        <v>8002</v>
       </c>
       <c r="L34" t="inlineStr">
         <is>
@@ -3577,7 +3577,7 @@
         </is>
       </c>
       <c r="K35" t="n">
-        <v>5122</v>
+        <v>5123</v>
       </c>
       <c r="L35" t="inlineStr">
         <is>
@@ -3634,36 +3634,28 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>https://openalex.org/W2945976633</t>
+          <t>https://openalex.org/W1680797894</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1038/s42256-019-0048-x</t>
+          <t>https://doi.org/10.1007/978-0-387-30164-8</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Stop explaining black box machine learning models for high stakes decisions and use interpretable models instead</t>
-        </is>
-      </c>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t>Nature Machine Intelligence</t>
-        </is>
-      </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>Nature Machine Intelligence</t>
-        </is>
-      </c>
+          <t>Encyclopedia of Machine Learning</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr"/>
+      <c r="G36" t="inlineStr"/>
       <c r="H36" t="n">
-        <v>2019</v>
+        <v>2010</v>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>article</t>
+          <t>book</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
@@ -3672,60 +3664,40 @@
         </is>
       </c>
       <c r="K36" t="n">
-        <v>9072</v>
+        <v>3476</v>
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>Cynthia Rudin</t>
+          <t>Claude Sammut</t>
         </is>
       </c>
       <c r="M36" t="inlineStr"/>
       <c r="N36" t="inlineStr">
         <is>
-          <t>Cynthia Rudin, Duke University;Cynthia Rudin, Duke University, Durham, NC, USA</t>
+          <t>Claude Sammut, University Of New south Wales</t>
         </is>
       </c>
       <c r="O36" t="inlineStr"/>
-      <c r="P36" t="inlineStr">
-        <is>
-          <t>https://openalex.org/W1492170170; https://openalex.org/W1537462412; https://openalex.org/W1731081199; https://openalex.org/W1746506709; https://openalex.org/W1905782493; https://openalex.org/W1973682096; https://openalex.org/W1984314602; https://openalex.org/W1994407253; https://openalex.org/W2013587512; https://openalex.org/W2026905436; https://openalex.org/W2046945713; https://openalex.org/W2072136246; https://openalex.org/W2082262280; https://openalex.org/W2132166479; https://openalex.org/W2134598164; https://openalex.org/W2141097525; https://openalex.org/W2149033360; https://openalex.org/W2163598528; https://openalex.org/W2239135493; https://openalex.org/W2248060815; https://openalex.org/W2467510144; https://openalex.org/W2493343568; https://openalex.org/W2579555219; https://openalex.org/W2604231045; https://openalex.org/W2613140028; https://openalex.org/W2621305858; https://openalex.org/W2743731382; https://openalex.org/W2752988282; https://openalex.org/W2765813195; https://openalex.org/W2767442356; https://openalex.org/W2778670458; https://openalex.org/W2798857668; https://openalex.org/W2811104224; https://openalex.org/W2811374795; https://openalex.org/W2894881080; https://openalex.org/W2895051075; https://openalex.org/W2896176822; https://openalex.org/W2898694742; https://openalex.org/W2899360465; https://openalex.org/W2901939789; https://openalex.org/W2902991393; https://openalex.org/W2910705748; https://openalex.org/W2962689739; https://openalex.org/W2963125461; https://openalex.org/W2963533879; https://openalex.org/W2963816926; https://openalex.org/W2964134873; https://openalex.org/W2964180856; https://openalex.org/W3085162807; https://openalex.org/W3098636317; https://openalex.org/W3102221121; https://openalex.org/W3102834905; https://openalex.org/W3122175177; https://openalex.org/W4234008654; https://openalex.org/W6743543778</t>
-        </is>
-      </c>
+      <c r="P36" t="inlineStr"/>
       <c r="Q36" t="inlineStr">
         <is>
-          <t>Black box;Harm;Computer science;Key (lock);Criminal justice;Artificial intelligence;Economic Justice;Machine learning;Data science;Criminology;Psychology;Computer security;Political science;Social psychology;Law</t>
+          <t>Encyclopedia;Computer science;Artificial intelligence;Data science;Library science</t>
         </is>
       </c>
       <c r="R36" t="inlineStr"/>
       <c r="S36" t="inlineStr"/>
-      <c r="T36" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="U36" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="V36" t="inlineStr">
-        <is>
-          <t>206</t>
-        </is>
-      </c>
-      <c r="W36" t="inlineStr">
-        <is>
-          <t>215</t>
-        </is>
-      </c>
+      <c r="T36" t="inlineStr"/>
+      <c r="U36" t="inlineStr"/>
+      <c r="V36" t="inlineStr"/>
+      <c r="W36" t="inlineStr"/>
       <c r="X36" t="inlineStr">
         <is>
-          <t>Cynthia Rudin, 2019, Nature Machine Intelligence</t>
+          <t xml:space="preserve">Claude Sammut, 2010, </t>
         </is>
       </c>
       <c r="Y36" t="inlineStr">
         <is>
-          <t>Cynthia Rudin, 2019, Nature Machine Intelligence</t>
+          <t xml:space="preserve">Claude Sammut, 2010, </t>
         </is>
       </c>
     </row>
@@ -3767,7 +3739,7 @@
         </is>
       </c>
       <c r="K37" t="n">
-        <v>5637</v>
+        <v>5638</v>
       </c>
       <c r="L37" t="inlineStr">
         <is>
@@ -3828,28 +3800,36 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>https://openalex.org/W1680797894</t>
+          <t>https://openalex.org/W2945976633</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1007/978-0-387-30164-8</t>
+          <t>https://doi.org/10.1038/s42256-019-0048-x</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Encyclopedia of Machine Learning</t>
-        </is>
-      </c>
-      <c r="F38" t="inlineStr"/>
-      <c r="G38" t="inlineStr"/>
+          <t>Stop explaining black box machine learning models for high stakes decisions and use interpretable models instead</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Nature Machine Intelligence</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Nature Machine Intelligence</t>
+        </is>
+      </c>
       <c r="H38" t="n">
-        <v>2010</v>
+        <v>2019</v>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>book</t>
+          <t>article</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
@@ -3858,40 +3838,60 @@
         </is>
       </c>
       <c r="K38" t="n">
-        <v>3475</v>
+        <v>9116</v>
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>Claude Sammut</t>
+          <t>Cynthia Rudin</t>
         </is>
       </c>
       <c r="M38" t="inlineStr"/>
       <c r="N38" t="inlineStr">
         <is>
-          <t>Claude Sammut, University Of New south Wales</t>
+          <t>Cynthia Rudin, Duke University;Cynthia Rudin, Duke University, Durham, NC, USA</t>
         </is>
       </c>
       <c r="O38" t="inlineStr"/>
-      <c r="P38" t="inlineStr"/>
+      <c r="P38" t="inlineStr">
+        <is>
+          <t>https://openalex.org/W1492170170; https://openalex.org/W1537462412; https://openalex.org/W1731081199; https://openalex.org/W1746506709; https://openalex.org/W1905782493; https://openalex.org/W1973682096; https://openalex.org/W1984314602; https://openalex.org/W1994407253; https://openalex.org/W2013587512; https://openalex.org/W2026905436; https://openalex.org/W2046945713; https://openalex.org/W2072136246; https://openalex.org/W2082262280; https://openalex.org/W2132166479; https://openalex.org/W2134598164; https://openalex.org/W2141097525; https://openalex.org/W2149033360; https://openalex.org/W2163598528; https://openalex.org/W2239135493; https://openalex.org/W2248060815; https://openalex.org/W2467510144; https://openalex.org/W2493343568; https://openalex.org/W2579555219; https://openalex.org/W2604231045; https://openalex.org/W2613140028; https://openalex.org/W2621305858; https://openalex.org/W2743731382; https://openalex.org/W2752988282; https://openalex.org/W2765813195; https://openalex.org/W2767442356; https://openalex.org/W2778670458; https://openalex.org/W2798857668; https://openalex.org/W2811104224; https://openalex.org/W2811374795; https://openalex.org/W2894881080; https://openalex.org/W2895051075; https://openalex.org/W2896176822; https://openalex.org/W2898694742; https://openalex.org/W2899360465; https://openalex.org/W2901939789; https://openalex.org/W2902991393; https://openalex.org/W2910705748; https://openalex.org/W2962689739; https://openalex.org/W2963125461; https://openalex.org/W2963533879; https://openalex.org/W2963816926; https://openalex.org/W2964134873; https://openalex.org/W2964180856; https://openalex.org/W3085162807; https://openalex.org/W3098636317; https://openalex.org/W3102221121; https://openalex.org/W3102834905; https://openalex.org/W3122175177; https://openalex.org/W4234008654; https://openalex.org/W6743543778</t>
+        </is>
+      </c>
       <c r="Q38" t="inlineStr">
         <is>
-          <t>Encyclopedia;Computer science;Artificial intelligence;Data science;Library science</t>
+          <t>Black box;Harm;Computer science;Key (lock);Criminal justice;Artificial intelligence;Economic Justice;Machine learning;Data science;Criminology;Psychology;Computer security;Political science;Social psychology;Law</t>
         </is>
       </c>
       <c r="R38" t="inlineStr"/>
       <c r="S38" t="inlineStr"/>
-      <c r="T38" t="inlineStr"/>
-      <c r="U38" t="inlineStr"/>
-      <c r="V38" t="inlineStr"/>
-      <c r="W38" t="inlineStr"/>
+      <c r="T38" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="U38" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="V38" t="inlineStr">
+        <is>
+          <t>206</t>
+        </is>
+      </c>
+      <c r="W38" t="inlineStr">
+        <is>
+          <t>215</t>
+        </is>
+      </c>
       <c r="X38" t="inlineStr">
         <is>
-          <t xml:space="preserve">Claude Sammut, 2010, </t>
+          <t>Cynthia Rudin, 2019, Nature Machine Intelligence</t>
         </is>
       </c>
       <c r="Y38" t="inlineStr">
         <is>
-          <t xml:space="preserve">Claude Sammut, 2010, </t>
+          <t>Cynthia Rudin, 2019, Nature Machine Intelligence</t>
         </is>
       </c>
     </row>
@@ -3941,7 +3941,7 @@
         </is>
       </c>
       <c r="K39" t="n">
-        <v>4242</v>
+        <v>4255</v>
       </c>
       <c r="L39" t="inlineStr">
         <is>
@@ -4048,7 +4048,7 @@
         </is>
       </c>
       <c r="K40" t="n">
-        <v>3431</v>
+        <v>3435</v>
       </c>
       <c r="L40" t="inlineStr">
         <is>
@@ -4155,7 +4155,7 @@
         </is>
       </c>
       <c r="K41" t="n">
-        <v>5153</v>
+        <v>5164</v>
       </c>
       <c r="L41" t="inlineStr">
         <is>
@@ -4374,24 +4374,36 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>https://openalex.org/W1873332500</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr"/>
+          <t>https://openalex.org/W4236362309</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1017/cbo9781107298019</t>
+        </is>
+      </c>
       <c r="D44" t="inlineStr"/>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Supervised Machine Learning: A Review of Classification Techniques</t>
-        </is>
-      </c>
-      <c r="F44" t="inlineStr"/>
-      <c r="G44" t="inlineStr"/>
+          <t>Understanding Machine Learning</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Cambridge University Press eBooks</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Cambridge University Press eBooks</t>
+        </is>
+      </c>
       <c r="H44" t="n">
-        <v>2007</v>
+        <v>2014</v>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>review</t>
+          <t>book</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
@@ -4400,60 +4412,44 @@
         </is>
       </c>
       <c r="K44" t="n">
-        <v>4147</v>
+        <v>2931</v>
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>Sotiris Kotsiantis</t>
+          <t>Shai Shalev‐Shwartz;Shai Ben-David</t>
         </is>
       </c>
       <c r="M44" t="inlineStr"/>
-      <c r="N44" t="inlineStr"/>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>Shai Shalev‐Shwartz, Hebrew University of Jerusalem;Shai Ben-David, University of Waterloo, Ontario</t>
+        </is>
+      </c>
       <c r="O44" t="inlineStr"/>
-      <c r="P44" t="inlineStr">
-        <is>
-          <t>https://openalex.org/W5472403; https://openalex.org/W135311109; https://openalex.org/W177590838; https://openalex.org/W203696055; https://openalex.org/W1007293483; https://openalex.org/W1497605902; https://openalex.org/W1506588750; https://openalex.org/W1515851193; https://openalex.org/W1520605446; https://openalex.org/W1522114398; https://openalex.org/W1528113134; https://openalex.org/W1537143578; https://openalex.org/W1538041071; https://openalex.org/W1547833367; https://openalex.org/W1554309553; https://openalex.org/W1560955742; https://openalex.org/W1562368284; https://openalex.org/W1563088657; https://openalex.org/W1567012231; https://openalex.org/W1570329253; https://openalex.org/W1570448133; https://openalex.org/W1570706771; https://openalex.org/W1587647246; https://openalex.org/W1588516554; https://openalex.org/W1594031697; https://openalex.org/W1594781927; https://openalex.org/W1602492977; https://openalex.org/W1605688901; https://openalex.org/W1605844890; https://openalex.org/W1637435380; https://openalex.org/W1670263352; https://openalex.org/W1671614046; https://openalex.org/W1746680969; https://openalex.org/W1780185704; https://openalex.org/W1808644423; https://openalex.org/W1813387235; https://openalex.org/W1817561967; https://openalex.org/W1827261456; https://openalex.org/W1904009171; https://openalex.org/W1935515061; https://openalex.org/W1973991804; https://openalex.org/W1974545290; https://openalex.org/W1979711143; https://openalex.org/W1983479840; https://openalex.org/W1983690667; https://openalex.org/W1986883011; https://openalex.org/W1992419399; https://openalex.org/W1993066733; https://openalex.org/W2006345381; https://openalex.org/W2011101028; https://openalex.org/W2016441117; https://openalex.org/W2022058268; https://openalex.org/W2026718556; https://openalex.org/W2037322594; https://openalex.org/W2046649434; https://openalex.org/W2050829396; https://openalex.org/W2063783806; https://openalex.org/W2074584355; https://openalex.org/W2075932270; https://openalex.org/W2093825590; https://openalex.org/W2096756482; https://openalex.org/W2104333211; https://openalex.org/W2110179049; https://openalex.org/W2119479037; https://openalex.org/W2120199131; https://openalex.org/W2122111042; https://openalex.org/W2122496402; https://openalex.org/W2123623606; https://openalex.org/W2125055259; https://openalex.org/W2126333738; https://openalex.org/W2128912745; https://openalex.org/W2133160781; https://openalex.org/W2133218851; https://openalex.org/W2133632100; https://openalex.org/W2136000097; https://openalex.org/W2136132422; https://openalex.org/W2137130182; https://openalex.org/W2139212933; https://openalex.org/W2140586694; https://openalex.org/W2140785063; https://openalex.org/W2142857211; https://openalex.org/W2143603257; https://openalex.org/W2144731007; https://openalex.org/W2145467382; https://openalex.org/W2145680191; https://openalex.org/W2150796457; https://openalex.org/W2151450140; https://openalex.org/W2156440942; https://openalex.org/W2156571267; https://openalex.org/W2156909104; https://openalex.org/W2157815868; https://openalex.org/W2158724449; https://openalex.org/W2159895197; https://openalex.org/W2161349318; https://openalex.org/W2161782846; https://openalex.org/W2161960932; https://openalex.org/W2164359548; https://openalex.org/W2166985738; https://openalex.org/W2167277498; https://openalex.org/W2167467747; https://openalex.org/W2168754135; https://openalex.org/W2171265988; https://openalex.org/W2172429451; https://openalex.org/W2322002063; https://openalex.org/W2488399954; https://openalex.org/W2603390332; https://openalex.org/W2766736793; https://openalex.org/W2911678770; https://openalex.org/W2912276539; https://openalex.org/W2912934387; https://openalex.org/W3015462599</t>
-        </is>
-      </c>
+      <c r="P44" t="inlineStr"/>
       <c r="Q44" t="inlineStr">
         <is>
-          <t>Machine learning;Artificial intelligence;Computer science;Classifier (UML);Supervised learning;One-class classification;Class (philosophy);Semi-supervised learning;Artificial neural network</t>
+          <t>Computer science;Artificial intelligence;Stability (learning theory);Algorithmic learning theory;Computational learning theory;Machine learning;Presentation (obstetrics);Stochastic gradient descent;Convexity;Online machine learning;Artificial neural network</t>
         </is>
       </c>
       <c r="R44" t="inlineStr"/>
       <c r="S44" t="inlineStr">
         <is>
-          <t>The goal of supervised learning is to build a concise model of the distribution of class labels in terms of predictor features. The resulting classifier is then used to assign class labels to the testing instances where the values of the predictor features are known, but the value of the class label is unknown. This paper describes various supervised machine learning classification techniques. Of course, a single chapter cannot be a complete review of all supervised machine learning classification algorithms (also known induction classification algorithms), yet we hope that the references cited will cover the major theoretical issues, guiding the researcher in interesting research directions and suggesting possible bias combinations that have yet to be explored.</t>
-        </is>
-      </c>
-      <c r="T44" t="inlineStr">
-        <is>
-          <t>160</t>
-        </is>
-      </c>
-      <c r="U44" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="V44" t="inlineStr">
-        <is>
-          <t>249</t>
-        </is>
-      </c>
-      <c r="W44" t="inlineStr">
-        <is>
-          <t>24</t>
-        </is>
-      </c>
+          <t>Machine learning is one of the fastest growing areas of computer science, with far-reaching applications. The aim of this textbook is to introduce machine learning, and the algorithmic paradigms it offers, in a principled way. The book provides a theoretical account of the fundamentals underlying machine learning and the mathematical derivations that transform these principles into practical algorithms. Following a presentation of the basics, the book covers a wide array of central topics unaddressed by previous textbooks. These include a discussion of the computational complexity of learning and the concepts of convexity and stability; important algorithmic paradigms including stochastic gradient descent, neural networks, and structured output learning; and emerging theoretical concepts such as the PAC-Bayes approach and compression-based bounds. Designed for advanced undergraduates or beginning graduates, the text makes the fundamentals and algorithms of machine learning accessible to students and non-expert readers in statistics, computer science, mathematics and engineering.</t>
+        </is>
+      </c>
+      <c r="T44" t="inlineStr"/>
+      <c r="U44" t="inlineStr"/>
+      <c r="V44" t="inlineStr"/>
+      <c r="W44" t="inlineStr"/>
       <c r="X44" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sotiris Kotsiantis, 2007, </t>
+          <t>Shai Shalev‐Shwartz, 2014, Cambridge University Press eBooks</t>
         </is>
       </c>
       <c r="Y44" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sotiris Kotsiantis, 2007, </t>
+          <t>Shai Shalev‐Shwartz, 2014, Cambridge University Press eBooks</t>
         </is>
       </c>
     </row>
@@ -4465,36 +4461,24 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>https://openalex.org/W4236362309</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.1017/cbo9781107298019</t>
-        </is>
-      </c>
+          <t>https://openalex.org/W1873332500</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr"/>
       <c r="D45" t="inlineStr"/>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Understanding Machine Learning</t>
-        </is>
-      </c>
-      <c r="F45" t="inlineStr">
-        <is>
-          <t>Cambridge University Press eBooks</t>
-        </is>
-      </c>
-      <c r="G45" t="inlineStr">
-        <is>
-          <t>Cambridge University Press eBooks</t>
-        </is>
-      </c>
+          <t>Supervised Machine Learning: A Review of Classification Techniques</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr"/>
+      <c r="G45" t="inlineStr"/>
       <c r="H45" t="n">
-        <v>2014</v>
+        <v>2007</v>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>book</t>
+          <t>review</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
@@ -4503,44 +4487,60 @@
         </is>
       </c>
       <c r="K45" t="n">
-        <v>2931</v>
+        <v>4147</v>
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>Shai Shalev‐Shwartz;Shai Ben-David</t>
+          <t>Sotiris Kotsiantis</t>
         </is>
       </c>
       <c r="M45" t="inlineStr"/>
-      <c r="N45" t="inlineStr">
-        <is>
-          <t>Shai Shalev‐Shwartz, Hebrew University of Jerusalem;Shai Ben-David, University of Waterloo, Ontario</t>
-        </is>
-      </c>
+      <c r="N45" t="inlineStr"/>
       <c r="O45" t="inlineStr"/>
-      <c r="P45" t="inlineStr"/>
+      <c r="P45" t="inlineStr">
+        <is>
+          <t>https://openalex.org/W5472403; https://openalex.org/W135311109; https://openalex.org/W177590838; https://openalex.org/W203696055; https://openalex.org/W1007293483; https://openalex.org/W1497605902; https://openalex.org/W1506588750; https://openalex.org/W1515851193; https://openalex.org/W1520605446; https://openalex.org/W1522114398; https://openalex.org/W1528113134; https://openalex.org/W1537143578; https://openalex.org/W1538041071; https://openalex.org/W1547833367; https://openalex.org/W1554309553; https://openalex.org/W1560955742; https://openalex.org/W1562368284; https://openalex.org/W1563088657; https://openalex.org/W1567012231; https://openalex.org/W1570329253; https://openalex.org/W1570448133; https://openalex.org/W1570706771; https://openalex.org/W1587647246; https://openalex.org/W1588516554; https://openalex.org/W1594031697; https://openalex.org/W1594781927; https://openalex.org/W1602492977; https://openalex.org/W1605688901; https://openalex.org/W1605844890; https://openalex.org/W1637435380; https://openalex.org/W1670263352; https://openalex.org/W1671614046; https://openalex.org/W1746680969; https://openalex.org/W1780185704; https://openalex.org/W1808644423; https://openalex.org/W1813387235; https://openalex.org/W1817561967; https://openalex.org/W1827261456; https://openalex.org/W1904009171; https://openalex.org/W1935515061; https://openalex.org/W1973991804; https://openalex.org/W1974545290; https://openalex.org/W1979711143; https://openalex.org/W1983479840; https://openalex.org/W1983690667; https://openalex.org/W1986883011; https://openalex.org/W1992419399; https://openalex.org/W1993066733; https://openalex.org/W2006345381; https://openalex.org/W2011101028; https://openalex.org/W2016441117; https://openalex.org/W2022058268; https://openalex.org/W2026718556; https://openalex.org/W2037322594; https://openalex.org/W2046649434; https://openalex.org/W2050829396; https://openalex.org/W2063783806; https://openalex.org/W2074584355; https://openalex.org/W2075932270; https://openalex.org/W2093825590; https://openalex.org/W2096756482; https://openalex.org/W2104333211; https://openalex.org/W2110179049; https://openalex.org/W2119479037; https://openalex.org/W2120199131; https://openalex.org/W2122111042; https://openalex.org/W2122496402; https://openalex.org/W2123623606; https://openalex.org/W2125055259; https://openalex.org/W2126333738; https://openalex.org/W2128912745; https://openalex.org/W2133160781; https://openalex.org/W2133218851; https://openalex.org/W2133632100; https://openalex.org/W2136000097; https://openalex.org/W2136132422; https://openalex.org/W2137130182; https://openalex.org/W2139212933; https://openalex.org/W2140586694; https://openalex.org/W2140785063; https://openalex.org/W2142857211; https://openalex.org/W2143603257; https://openalex.org/W2144731007; https://openalex.org/W2145467382; https://openalex.org/W2145680191; https://openalex.org/W2150796457; https://openalex.org/W2151450140; https://openalex.org/W2156440942; https://openalex.org/W2156571267; https://openalex.org/W2156909104; https://openalex.org/W2157815868; https://openalex.org/W2158724449; https://openalex.org/W2159895197; https://openalex.org/W2161349318; https://openalex.org/W2161782846; https://openalex.org/W2161960932; https://openalex.org/W2164359548; https://openalex.org/W2166985738; https://openalex.org/W2167277498; https://openalex.org/W2167467747; https://openalex.org/W2168754135; https://openalex.org/W2171265988; https://openalex.org/W2172429451; https://openalex.org/W2322002063; https://openalex.org/W2488399954; https://openalex.org/W2603390332; https://openalex.org/W2766736793; https://openalex.org/W2911678770; https://openalex.org/W2912276539; https://openalex.org/W2912934387; https://openalex.org/W3015462599</t>
+        </is>
+      </c>
       <c r="Q45" t="inlineStr">
         <is>
-          <t>Computer science;Artificial intelligence;Stability (learning theory);Algorithmic learning theory;Computational learning theory;Machine learning;Presentation (obstetrics);Stochastic gradient descent;Convexity;Online machine learning;Artificial neural network</t>
+          <t>Machine learning;Artificial intelligence;Computer science;Classifier (UML);Supervised learning;One-class classification;Class (philosophy);Semi-supervised learning;Artificial neural network</t>
         </is>
       </c>
       <c r="R45" t="inlineStr"/>
       <c r="S45" t="inlineStr">
         <is>
-          <t>Machine learning is one of the fastest growing areas of computer science, with far-reaching applications. The aim of this textbook is to introduce machine learning, and the algorithmic paradigms it offers, in a principled way. The book provides a theoretical account of the fundamentals underlying machine learning and the mathematical derivations that transform these principles into practical algorithms. Following a presentation of the basics, the book covers a wide array of central topics unaddressed by previous textbooks. These include a discussion of the computational complexity of learning and the concepts of convexity and stability; important algorithmic paradigms including stochastic gradient descent, neural networks, and structured output learning; and emerging theoretical concepts such as the PAC-Bayes approach and compression-based bounds. Designed for advanced undergraduates or beginning graduates, the text makes the fundamentals and algorithms of machine learning accessible to students and non-expert readers in statistics, computer science, mathematics and engineering.</t>
-        </is>
-      </c>
-      <c r="T45" t="inlineStr"/>
-      <c r="U45" t="inlineStr"/>
-      <c r="V45" t="inlineStr"/>
-      <c r="W45" t="inlineStr"/>
+          <t>The goal of supervised learning is to build a concise model of the distribution of class labels in terms of predictor features. The resulting classifier is then used to assign class labels to the testing instances where the values of the predictor features are known, but the value of the class label is unknown. This paper describes various supervised machine learning classification techniques. Of course, a single chapter cannot be a complete review of all supervised machine learning classification algorithms (also known induction classification algorithms), yet we hope that the references cited will cover the major theoretical issues, guiding the researcher in interesting research directions and suggesting possible bias combinations that have yet to be explored.</t>
+        </is>
+      </c>
+      <c r="T45" t="inlineStr">
+        <is>
+          <t>160</t>
+        </is>
+      </c>
+      <c r="U45" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="V45" t="inlineStr">
+        <is>
+          <t>249</t>
+        </is>
+      </c>
+      <c r="W45" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
       <c r="X45" t="inlineStr">
         <is>
-          <t>Shai Shalev‐Shwartz, 2014, Cambridge University Press eBooks</t>
+          <t xml:space="preserve">Sotiris Kotsiantis, 2007, </t>
         </is>
       </c>
       <c r="Y45" t="inlineStr">
         <is>
-          <t>Shai Shalev‐Shwartz, 2014, Cambridge University Press eBooks</t>
+          <t xml:space="preserve">Sotiris Kotsiantis, 2007, </t>
         </is>
       </c>
     </row>
@@ -4552,36 +4552,36 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>https://openalex.org/W3198350258</t>
+          <t>https://openalex.org/W2885770726</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1147/rd.33.0210</t>
+          <t>https://doi.org/10.3390/s18082674</t>
         </is>
       </c>
       <c r="D46" t="inlineStr"/>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Some Studies in Machine Learning Using the Game of Checkers</t>
+          <t>Machine Learning in Agriculture: A Review</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>IBM Journal of Research and Development</t>
+          <t>Sensors</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>IBM Journal of Research and Development</t>
+          <t>Sensors</t>
         </is>
       </c>
       <c r="H46" t="n">
-        <v>1959</v>
+        <v>2018</v>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>article</t>
+          <t>review</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
@@ -4590,56 +4590,64 @@
         </is>
       </c>
       <c r="K46" t="n">
-        <v>4367</v>
+        <v>3065</v>
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>Arthur L. Samuel</t>
+          <t>Κωνσταντίνος Λιάκος;Patrizia Busato;Dimitrios Moshou;Simon Pearson;Dionysis Bochtis</t>
         </is>
       </c>
       <c r="M46" t="inlineStr"/>
-      <c r="N46" t="inlineStr"/>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>Κωνσταντίνος Λιάκος, Institute for Bio-Economy and Agri-Technology (IBO), Centre of Research and Technology—Hellas (CERTH), 6th km Charilaou-Thermi Rd, GR 57001 Thessaloniki, Greece;Patrizia Busato, Department of Agriculture, Forestry and Food Sciences (DISAFA), Faculty of Agriculture, University of Turin, Largo Braccini 2, 10095 Grugliasco, Italy;Dimitrios Moshou, Agricultural Engineering Laboratory, Faculty of Agriculture, Aristotle University of Thessaloniki, 54124 Thessaloniki, Greece;Dimitrios Moshou, Institute for Bio-Economy and Agri-Technology (IBO), Centre of Research and Technology—Hellas (CERTH), 6th km Charilaou-Thermi Rd, GR 57001 Thessaloniki, Greece;Simon Pearson, Lincoln Institute for Agri-food Technology (LIAT), University of Lincoln, Brayford Way, Brayford Pool, Lincoln LN6 7TS, UK;Dionysis Bochtis, Institute for Bio-Economy and Agri-Technology (IBO), Centre of Research and Technology—Hellas (CERTH), 6th km Charilaou-Thermi Rd, GR 57001 Thessaloniki, Greece</t>
+        </is>
+      </c>
       <c r="O46" t="inlineStr"/>
-      <c r="P46" t="inlineStr"/>
+      <c r="P46" t="inlineStr">
+        <is>
+          <t>https://openalex.org/W94523489; https://openalex.org/W189596042; https://openalex.org/W1179140510; https://openalex.org/W1496317909; https://openalex.org/W1596717185; https://openalex.org/W1689445748; https://openalex.org/W1916445479; https://openalex.org/W1963579367; https://openalex.org/W1963790103; https://openalex.org/W1966124853; https://openalex.org/W1967320885; https://openalex.org/W1968452917; https://openalex.org/W1984530193; https://openalex.org/W1990517717; https://openalex.org/W1995341919; https://openalex.org/W1998871699; https://openalex.org/W2000972253; https://openalex.org/W2001619934; https://openalex.org/W2009986810; https://openalex.org/W2015263929; https://openalex.org/W2018435387; https://openalex.org/W2019207321; https://openalex.org/W2024081693; https://openalex.org/W2025279987; https://openalex.org/W2028606616; https://openalex.org/W2040104179; https://openalex.org/W2040870580; https://openalex.org/W2049633694; https://openalex.org/W2063304499; https://openalex.org/W2065165083; https://openalex.org/W2072680624; https://openalex.org/W2075320162; https://openalex.org/W2076857888; https://openalex.org/W2081544115; https://openalex.org/W2087877962; https://openalex.org/W2095727900; https://openalex.org/W2102201073; https://openalex.org/W2106855632; https://openalex.org/W2108703480; https://openalex.org/W2110642273; https://openalex.org/W2111072639; https://openalex.org/W2119821739; https://openalex.org/W2128084896; https://openalex.org/W2138178898; https://openalex.org/W2143908786; https://openalex.org/W2149723649; https://openalex.org/W2150593711; https://openalex.org/W2153476503; https://openalex.org/W2153635508; https://openalex.org/W2154350719; https://openalex.org/W2161673710; https://openalex.org/W2174918471; https://openalex.org/W2200121095; https://openalex.org/W2209382794; https://openalex.org/W2216013554; https://openalex.org/W2231576311; https://openalex.org/W2270460811; https://openalex.org/W2270641383; https://openalex.org/W2273322351; https://openalex.org/W2286091602; https://openalex.org/W2294798173; https://openalex.org/W2298521547; https://openalex.org/W2337945771; https://openalex.org/W2339447311; https://openalex.org/W2399675776; https://openalex.org/W2417395753; https://openalex.org/W2419137750; https://openalex.org/W2470803522; https://openalex.org/W2497210317; https://openalex.org/W2502044482; https://openalex.org/W2552660223; https://openalex.org/W2560811704; https://openalex.org/W2577148968; https://openalex.org/W2580808806; https://openalex.org/W2586821267; https://openalex.org/W2591104514; https://openalex.org/W2598645336; https://openalex.org/W2603364874; https://openalex.org/W2603417106; https://openalex.org/W2604196786; https://openalex.org/W2606244344; https://openalex.org/W2606916050; https://openalex.org/W2612828053; https://openalex.org/W2619390517; https://openalex.org/W2620473470; https://openalex.org/W2620542418; https://openalex.org/W2621525431; https://openalex.org/W2622758479; https://openalex.org/W2622999711; https://openalex.org/W2738911869; https://openalex.org/W2775111183; https://openalex.org/W2789255992; https://openalex.org/W2790639095; https://openalex.org/W2791690647; https://openalex.org/W2794415089; https://openalex.org/W2796501058; https://openalex.org/W2806779833; https://openalex.org/W2903950532; https://openalex.org/W2911964244; https://openalex.org/W2919115771; https://openalex.org/W3125807057; https://openalex.org/W4210451417; https://openalex.org/W4212883601; https://openalex.org/W4232670376; https://openalex.org/W4239510810; https://openalex.org/W4250143236; https://openalex.org/W4400360174; https://openalex.org/W6607775107; https://openalex.org/W6632223008; https://openalex.org/W6675321329; https://openalex.org/W6675436802; https://openalex.org/W6676769703</t>
+        </is>
+      </c>
       <c r="Q46" t="inlineStr">
         <is>
-          <t>Computer science;Artificial intelligence;Machine learning</t>
+          <t>Agriculture;Artificial intelligence;Precision agriculture;Computer science;Machine learning;Big data;Livestock;Decision support system;Data science;Data mining</t>
         </is>
       </c>
       <c r="R46" t="inlineStr"/>
       <c r="S46" t="inlineStr">
         <is>
-          <t>Two machine-learning procedures have been investigated in some detail using the game of checkers. Enough work has been done to verify the fact that a computer can be programmed so that it will learn to play a better game of checkers than can be played by the person who wrote the program. Furthermore, it can learn to do this in a remarkably short period of time (8 or 10 hours of machine-playing time) when given only the rules of the game, a sense of direction, and a redundant and incomplete list of parameters which are thought to have something to do with the game, but whose correct signs and relative weights are unknown and unspecified. The principles of machine learning verified by these experiments are, of course, applicable to many other situations.</t>
+          <t>Machine learning has emerged with big data technologies and high-performance computing to create new opportunities for data intensive science in the multi-disciplinary agri-technologies domain. In this paper, we present a comprehensive review of research dedicated to applications of machine learning in agricultural production systems. The works analyzed were categorized in (a) crop management, including applications on yield prediction, disease detection, weed detection crop quality, and species recognition; (b) livestock management, including applications on animal welfare and livestock production; (c) water management; and (d) soil management. The filtering and classification of the presented articles demonstrate how agriculture will benefit from machine learning technologies. By applying machine learning to sensor data, farm management systems are evolving into real time artificial intelligence enabled programs that provide rich recommendations and insights for farmer decision support and action.</t>
         </is>
       </c>
       <c r="T46" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>18</t>
         </is>
       </c>
       <c r="U46" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>8</t>
         </is>
       </c>
       <c r="V46" t="inlineStr">
         <is>
-          <t>210</t>
+          <t>2674</t>
         </is>
       </c>
       <c r="W46" t="inlineStr">
         <is>
-          <t>229</t>
+          <t>2674</t>
         </is>
       </c>
       <c r="X46" t="inlineStr">
         <is>
-          <t>Arthur L. Samuel, 1959, IBM Journal of Research and Development</t>
+          <t>Κωνσταντίνος Λιάκος, 2018, Sensors</t>
         </is>
       </c>
       <c r="Y46" t="inlineStr">
         <is>
-          <t>Arthur L. Samuel, 1959, IBM Journal of Research and Development</t>
+          <t>Κωνσταντίνος Λιάκος, 2018, Sensors</t>
         </is>
       </c>
     </row>
@@ -4651,36 +4659,36 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>https://openalex.org/W2885770726</t>
+          <t>https://openalex.org/W3198350258</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>https://doi.org/10.3390/s18082674</t>
+          <t>https://doi.org/10.1147/rd.33.0210</t>
         </is>
       </c>
       <c r="D47" t="inlineStr"/>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Machine Learning in Agriculture: A Review</t>
+          <t>Some Studies in Machine Learning Using the Game of Checkers</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Sensors</t>
+          <t>IBM Journal of Research and Development</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>Sensors</t>
+          <t>IBM Journal of Research and Development</t>
         </is>
       </c>
       <c r="H47" t="n">
-        <v>2018</v>
+        <v>1959</v>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>review</t>
+          <t>article</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
@@ -4689,64 +4697,56 @@
         </is>
       </c>
       <c r="K47" t="n">
-        <v>3057</v>
+        <v>4368</v>
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>Κωνσταντίνος Λιάκος;Patrizia Busato;Dimitrios Moshou;Simon Pearson;Dionysis Bochtis</t>
+          <t>Arthur L. Samuel</t>
         </is>
       </c>
       <c r="M47" t="inlineStr"/>
-      <c r="N47" t="inlineStr">
-        <is>
-          <t>Κωνσταντίνος Λιάκος, Institute for Bio-Economy and Agri-Technology (IBO), Centre of Research and Technology—Hellas (CERTH), 6th km Charilaou-Thermi Rd, GR 57001 Thessaloniki, Greece;Patrizia Busato, Department of Agriculture, Forestry and Food Sciences (DISAFA), Faculty of Agriculture, University of Turin, Largo Braccini 2, 10095 Grugliasco, Italy;Dimitrios Moshou, Agricultural Engineering Laboratory, Faculty of Agriculture, Aristotle University of Thessaloniki, 54124 Thessaloniki, Greece;Dimitrios Moshou, Institute for Bio-Economy and Agri-Technology (IBO), Centre of Research and Technology—Hellas (CERTH), 6th km Charilaou-Thermi Rd, GR 57001 Thessaloniki, Greece;Simon Pearson, Lincoln Institute for Agri-food Technology (LIAT), University of Lincoln, Brayford Way, Brayford Pool, Lincoln LN6 7TS, UK;Dionysis Bochtis, Institute for Bio-Economy and Agri-Technology (IBO), Centre of Research and Technology—Hellas (CERTH), 6th km Charilaou-Thermi Rd, GR 57001 Thessaloniki, Greece</t>
-        </is>
-      </c>
+      <c r="N47" t="inlineStr"/>
       <c r="O47" t="inlineStr"/>
-      <c r="P47" t="inlineStr">
-        <is>
-          <t>https://openalex.org/W94523489; https://openalex.org/W189596042; https://openalex.org/W1179140510; https://openalex.org/W1496317909; https://openalex.org/W1596717185; https://openalex.org/W1689445748; https://openalex.org/W1916445479; https://openalex.org/W1963579367; https://openalex.org/W1963790103; https://openalex.org/W1966124853; https://openalex.org/W1967320885; https://openalex.org/W1968452917; https://openalex.org/W1984530193; https://openalex.org/W1990517717; https://openalex.org/W1995341919; https://openalex.org/W1998871699; https://openalex.org/W2000972253; https://openalex.org/W2001619934; https://openalex.org/W2009986810; https://openalex.org/W2015263929; https://openalex.org/W2018435387; https://openalex.org/W2019207321; https://openalex.org/W2024081693; https://openalex.org/W2025279987; https://openalex.org/W2028606616; https://openalex.org/W2040104179; https://openalex.org/W2040870580; https://openalex.org/W2049633694; https://openalex.org/W2063304499; https://openalex.org/W2065165083; https://openalex.org/W2072680624; https://openalex.org/W2075320162; https://openalex.org/W2076857888; https://openalex.org/W2081544115; https://openalex.org/W2087877962; https://openalex.org/W2095727900; https://openalex.org/W2102201073; https://openalex.org/W2106855632; https://openalex.org/W2108703480; https://openalex.org/W2110642273; https://openalex.org/W2111072639; https://openalex.org/W2119821739; https://openalex.org/W2128084896; https://openalex.org/W2138178898; https://openalex.org/W2143908786; https://openalex.org/W2149723649; https://openalex.org/W2150593711; https://openalex.org/W2153476503; https://openalex.org/W2153635508; https://openalex.org/W2154350719; https://openalex.org/W2161673710; https://openalex.org/W2174918471; https://openalex.org/W2200121095; https://openalex.org/W2209382794; https://openalex.org/W2216013554; https://openalex.org/W2231576311; https://openalex.org/W2270460811; https://openalex.org/W2270641383; https://openalex.org/W2273322351; https://openalex.org/W2286091602; https://openalex.org/W2294798173; https://openalex.org/W2298521547; https://openalex.org/W2337945771; https://openalex.org/W2339447311; https://openalex.org/W2399675776; https://openalex.org/W2417395753; https://openalex.org/W2419137750; https://openalex.org/W2470803522; https://openalex.org/W2497210317; https://openalex.org/W2502044482; https://openalex.org/W2552660223; https://openalex.org/W2560811704; https://openalex.org/W2577148968; https://openalex.org/W2580808806; https://openalex.org/W2586821267; https://openalex.org/W2591104514; https://openalex.org/W2598645336; https://openalex.org/W2603364874; https://openalex.org/W2603417106; https://openalex.org/W2604196786; https://openalex.org/W2606244344; https://openalex.org/W2606916050; https://openalex.org/W2612828053; https://openalex.org/W2619390517; https://openalex.org/W2620473470; https://openalex.org/W2620542418; https://openalex.org/W2621525431; https://openalex.org/W2622758479; https://openalex.org/W2622999711; https://openalex.org/W2738911869; https://openalex.org/W2775111183; https://openalex.org/W2789255992; https://openalex.org/W2790639095; https://openalex.org/W2791690647; https://openalex.org/W2794415089; https://openalex.org/W2796501058; https://openalex.org/W2806779833; https://openalex.org/W2903950532; https://openalex.org/W2911964244; https://openalex.org/W2919115771; https://openalex.org/W3125807057; https://openalex.org/W4210451417; https://openalex.org/W4212883601; https://openalex.org/W4232670376; https://openalex.org/W4239510810; https://openalex.org/W4250143236; https://openalex.org/W4400360174; https://openalex.org/W6607775107; https://openalex.org/W6632223008; https://openalex.org/W6675321329; https://openalex.org/W6675436802; https://openalex.org/W6676769703</t>
-        </is>
-      </c>
+      <c r="P47" t="inlineStr"/>
       <c r="Q47" t="inlineStr">
         <is>
-          <t>Agriculture;Artificial intelligence;Precision agriculture;Computer science;Machine learning;Big data;Livestock;Decision support system;Data science;Data mining</t>
+          <t>Computer science;Artificial intelligence;Machine learning</t>
         </is>
       </c>
       <c r="R47" t="inlineStr"/>
       <c r="S47" t="inlineStr">
         <is>
-          <t>Machine learning has emerged with big data technologies and high-performance computing to create new opportunities for data intensive science in the multi-disciplinary agri-technologies domain. In this paper, we present a comprehensive review of research dedicated to applications of machine learning in agricultural production systems. The works analyzed were categorized in (a) crop management, including applications on yield prediction, disease detection, weed detection crop quality, and species recognition; (b) livestock management, including applications on animal welfare and livestock production; (c) water management; and (d) soil management. The filtering and classification of the presented articles demonstrate how agriculture will benefit from machine learning technologies. By applying machine learning to sensor data, farm management systems are evolving into real time artificial intelligence enabled programs that provide rich recommendations and insights for farmer decision support and action.</t>
+          <t>Two machine-learning procedures have been investigated in some detail using the game of checkers. Enough work has been done to verify the fact that a computer can be programmed so that it will learn to play a better game of checkers than can be played by the person who wrote the program. Furthermore, it can learn to do this in a remarkably short period of time (8 or 10 hours of machine-playing time) when given only the rules of the game, a sense of direction, and a redundant and incomplete list of parameters which are thought to have something to do with the game, but whose correct signs and relative weights are unknown and unspecified. The principles of machine learning verified by these experiments are, of course, applicable to many other situations.</t>
         </is>
       </c>
       <c r="T47" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>3</t>
         </is>
       </c>
       <c r="U47" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>3</t>
         </is>
       </c>
       <c r="V47" t="inlineStr">
         <is>
-          <t>2674</t>
+          <t>210</t>
         </is>
       </c>
       <c r="W47" t="inlineStr">
         <is>
-          <t>2674</t>
+          <t>229</t>
         </is>
       </c>
       <c r="X47" t="inlineStr">
         <is>
-          <t>Κωνσταντίνος Λιάκος, 2018, Sensors</t>
+          <t>Arthur L. Samuel, 1959, IBM Journal of Research and Development</t>
         </is>
       </c>
       <c r="Y47" t="inlineStr">
         <is>
-          <t>Κωνσταντίνος Λιάκος, 2018, Sensors</t>
+          <t>Arthur L. Samuel, 1959, IBM Journal of Research and Development</t>
         </is>
       </c>
     </row>
@@ -4796,7 +4796,7 @@
         </is>
       </c>
       <c r="K48" t="n">
-        <v>4374</v>
+        <v>4375</v>
       </c>
       <c r="L48" t="inlineStr">
         <is>
@@ -4883,7 +4883,7 @@
         </is>
       </c>
       <c r="K49" t="n">
-        <v>4234</v>
+        <v>4239</v>
       </c>
       <c r="L49" t="inlineStr">
         <is>
@@ -4982,7 +4982,7 @@
         </is>
       </c>
       <c r="K50" t="n">
-        <v>4682</v>
+        <v>4692</v>
       </c>
       <c r="L50" t="inlineStr">
         <is>
@@ -5089,7 +5089,7 @@
         </is>
       </c>
       <c r="K51" t="n">
-        <v>2494</v>
+        <v>2499</v>
       </c>
       <c r="L51" t="inlineStr">
         <is>
@@ -5271,7 +5271,7 @@
         </is>
       </c>
       <c r="K53" t="n">
-        <v>2957</v>
+        <v>2963</v>
       </c>
       <c r="L53" t="inlineStr">
         <is>
@@ -5378,7 +5378,7 @@
         </is>
       </c>
       <c r="K54" t="n">
-        <v>3154</v>
+        <v>3157</v>
       </c>
       <c r="L54" t="inlineStr">
         <is>
@@ -5568,7 +5568,7 @@
         </is>
       </c>
       <c r="K56" t="n">
-        <v>4630</v>
+        <v>4633</v>
       </c>
       <c r="L56" t="inlineStr">
         <is>
@@ -5853,7 +5853,7 @@
         </is>
       </c>
       <c r="K59" t="n">
-        <v>2639</v>
+        <v>2653</v>
       </c>
       <c r="L59" t="inlineStr">
         <is>
@@ -5960,7 +5960,7 @@
         </is>
       </c>
       <c r="K60" t="n">
-        <v>2464</v>
+        <v>2467</v>
       </c>
       <c r="L60" t="inlineStr">
         <is>
@@ -6063,7 +6063,7 @@
         </is>
       </c>
       <c r="K61" t="n">
-        <v>2964</v>
+        <v>2973</v>
       </c>
       <c r="L61" t="inlineStr">
         <is>
@@ -6166,7 +6166,7 @@
         </is>
       </c>
       <c r="K62" t="n">
-        <v>3625</v>
+        <v>3633</v>
       </c>
       <c r="L62" t="inlineStr">
         <is>
@@ -6269,7 +6269,7 @@
         </is>
       </c>
       <c r="K63" t="n">
-        <v>3032</v>
+        <v>3033</v>
       </c>
       <c r="L63" t="inlineStr">
         <is>
@@ -6372,7 +6372,7 @@
         </is>
       </c>
       <c r="K64" t="n">
-        <v>3151</v>
+        <v>3152</v>
       </c>
       <c r="L64" t="inlineStr">
         <is>
@@ -6471,7 +6471,7 @@
         </is>
       </c>
       <c r="K65" t="n">
-        <v>2645</v>
+        <v>2652</v>
       </c>
       <c r="L65" t="inlineStr">
         <is>
@@ -6536,36 +6536,36 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>https://openalex.org/W2111547563</t>
+          <t>https://openalex.org/W2161336914</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1016/j.csbj.2014.11.005</t>
+          <t>https://doi.org/10.1145/2347736.2347755</t>
         </is>
       </c>
       <c r="D66" t="inlineStr"/>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Machine learning applications in cancer prognosis and prediction</t>
+          <t>A few useful things to know about machine learning</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>Computational and Structural Biotechnology Journal</t>
+          <t>Communications of the ACM</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>Computational and Structural Biotechnology Journal</t>
+          <t>Communications of the ACM</t>
         </is>
       </c>
       <c r="H66" t="n">
-        <v>2014</v>
+        <v>2012</v>
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>review</t>
+          <t>article</t>
         </is>
       </c>
       <c r="J66" t="inlineStr">
@@ -6574,60 +6574,64 @@
         </is>
       </c>
       <c r="K66" t="n">
-        <v>3302</v>
+        <v>3254</v>
       </c>
       <c r="L66" t="inlineStr">
         <is>
-          <t>Κωνσταντίνα Κούρου;Themis P. Exarchos;Konstantinos Exarchos;Michalis V. Karamouzis;Dimitrios I. Fotiadis</t>
+          <t>Pedro Domingos</t>
         </is>
       </c>
       <c r="M66" t="inlineStr"/>
       <c r="N66" t="inlineStr">
         <is>
-          <t>Κωνσταντίνα Κούρου, Unit of Medical Technology and Intelligent Information Systems, Dept. of Materials Science and Engineering, University of Ioannina, Ioannina, Greece;Themis P. Exarchos, IMBB — FORTH, Dept. of Biomedical Research, Ioannina, Greece;Themis P. Exarchos, Unit of Medical Technology and Intelligent Information Systems, Dept. of Materials Science and Engineering, University of Ioannina, Ioannina, Greece;Konstantinos Exarchos, Unit of Medical Technology and Intelligent Information Systems, Dept. of Materials Science and Engineering, University of Ioannina, Ioannina, Greece;Michalis V. Karamouzis, Molecular Oncology Unit, Department of Biological Chemistry, Medical School, University of Athens, Athens, Greece;Dimitrios I. Fotiadis, IMBB — FORTH, Dept. of Biomedical Research, Ioannina, Greece;Dimitrios I. Fotiadis, Unit of Medical Technology and Intelligent Information Systems, Dept. of Materials Science and Engineering, University of Ioannina, Ioannina, Greece</t>
+          <t>Pedro Domingos, University of Washington, Seattle</t>
         </is>
       </c>
       <c r="O66" t="inlineStr"/>
       <c r="P66" t="inlineStr">
         <is>
-          <t>https://openalex.org/W1491953704; https://openalex.org/W1500572886; https://openalex.org/W1517879388; https://openalex.org/W1519433744; https://openalex.org/W1565377632; https://openalex.org/W1570448133; https://openalex.org/W1591717158; https://openalex.org/W1651586605; https://openalex.org/W1663973292; https://openalex.org/W1960669649; https://openalex.org/W1971005400; https://openalex.org/W1978761216; https://openalex.org/W1983024255; https://openalex.org/W1985663400; https://openalex.org/W1987776395; https://openalex.org/W1989628460; https://openalex.org/W1992297816; https://openalex.org/W1993628165; https://openalex.org/W1995199599; https://openalex.org/W2007265575; https://openalex.org/W2011021469; https://openalex.org/W2014510428; https://openalex.org/W2017337590; https://openalex.org/W2020402396; https://openalex.org/W2021100122; https://openalex.org/W2025060250; https://openalex.org/W2025738103; https://openalex.org/W2036839465; https://openalex.org/W2041652340; https://openalex.org/W2048701123; https://openalex.org/W2053522428; https://openalex.org/W2058089746; https://openalex.org/W2062364738; https://openalex.org/W2083780116; https://openalex.org/W2088338744; https://openalex.org/W2089927030; https://openalex.org/W2091947792; https://openalex.org/W2097554668; https://openalex.org/W2105882193; https://openalex.org/W2109103446; https://openalex.org/W2109896839; https://openalex.org/W2111461407; https://openalex.org/W2116841457; https://openalex.org/W2117692326; https://openalex.org/W2118366842; https://openalex.org/W2119782683; https://openalex.org/W2122227569; https://openalex.org/W2123696692; https://openalex.org/W2126009609; https://openalex.org/W2128767954; https://openalex.org/W2130338776; https://openalex.org/W2132619562; https://openalex.org/W2133601033; https://openalex.org/W2140218006; https://openalex.org/W2148078825; https://openalex.org/W2152121590; https://openalex.org/W2154362705; https://openalex.org/W2155461561; https://openalex.org/W2156483112; https://openalex.org/W2157132621; https://openalex.org/W2157239837; https://openalex.org/W2163042952; https://openalex.org/W2167645795; https://openalex.org/W2167769381; https://openalex.org/W2170379523; https://openalex.org/W2324845196; https://openalex.org/W2431164060; https://openalex.org/W2476253186; https://openalex.org/W2977661550; https://openalex.org/W4205774955; https://openalex.org/W4255865525; https://openalex.org/W4296886862; https://openalex.org/W6660969321; https://openalex.org/W6663876547</t>
+          <t>https://openalex.org/W1486658274; https://openalex.org/W1494137514; https://openalex.org/W1504694836; https://openalex.org/W1521062204; https://openalex.org/W1570448133; https://openalex.org/W1583837637; https://openalex.org/W1585009072; https://openalex.org/W1761022139; https://openalex.org/W1977970897; https://openalex.org/W2001141328; https://openalex.org/W2039683780; https://openalex.org/W2063961549; https://openalex.org/W2070902649; https://openalex.org/W2072128103; https://openalex.org/W2089624555; https://openalex.org/W2100483895; https://openalex.org/W2110065044; https://openalex.org/W2110228583; https://openalex.org/W2125055259; https://openalex.org/W2140785063; https://openalex.org/W2143891888; https://openalex.org/W2152761983; https://openalex.org/W2156909104; https://openalex.org/W2400138769; https://openalex.org/W2966207845; https://openalex.org/W3133236490; https://openalex.org/W3135029803; https://openalex.org/W4231109964; https://openalex.org/W4232632925; https://openalex.org/W4299515571; https://openalex.org/W6791387550</t>
         </is>
       </c>
       <c r="Q66" t="inlineStr">
         <is>
-          <t>Machine learning;Artificial intelligence;Computer science;Support vector machine;Cancer;Artificial neural network;Bayesian network;Clinical Practice;Variety (cybernetics);Field (mathematics);Predictive modelling;Medicine;Mathematics</t>
+          <t>Computer science;Need to know;Artificial intelligence;Machine learning;Computer security</t>
         </is>
       </c>
       <c r="R66" t="inlineStr"/>
       <c r="S66" t="inlineStr">
         <is>
-          <t>Cancer has been characterized as a heterogeneous disease consisting of many different subtypes. The early diagnosis and prognosis of a cancer type have become a necessity in cancer research, as it can facilitate the subsequent clinical management of patients. The importance of classifying cancer patients into high or low risk groups has led many research teams, from the biomedical and the bioinformatics field, to study the application of machine learning (ML) methods. Therefore, these techniques have been utilized as an aim to model the progression and treatment of cancerous conditions. In addition, the ability of ML tools to detect key features from complex datasets reveals their importance. A variety of these techniques, including Artificial Neural Networks (ANNs), Bayesian Networks (BNs), Support Vector Machines (SVMs) and Decision Trees (DTs) have been widely applied in cancer research for the development of predictive models, resulting in effective and accurate decision making. Even though it is evident that the use of ML methods can improve our understanding of cancer progression, an appropriate level of validation is needed in order for these methods to be considered in the everyday clinical practice. In this work, we present a review of recent ML approaches employed in the modeling of cancer progression. The predictive models discussed here are based on various supervised ML techniques as well as on different input features and data samples. Given the growing trend on the application of ML methods in cancer research, we present here the most recent publications that employ these techniques as an aim to model cancer risk or patient outcomes.</t>
+          <t>Tapping into the "folk knowledge" needed to advance machine learning applications.</t>
         </is>
       </c>
       <c r="T66" t="inlineStr">
         <is>
-          <t>13</t>
-        </is>
-      </c>
-      <c r="U66" t="inlineStr"/>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="U66" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
       <c r="V66" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>78</t>
         </is>
       </c>
       <c r="W66" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>87</t>
         </is>
       </c>
       <c r="X66" t="inlineStr">
         <is>
-          <t>Κωνσταντίνα Κούρου, 2014, Computational and Structural Biotechnology Journal</t>
+          <t>Pedro Domingos, 2012, Communications of the ACM</t>
         </is>
       </c>
       <c r="Y66" t="inlineStr">
         <is>
-          <t>Κωνσταντίνα Κούρου, 2014, Computational and Structural Biotechnology Journal</t>
+          <t>Pedro Domingos, 2012, Communications of the ACM</t>
         </is>
       </c>
     </row>
@@ -6639,32 +6643,32 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>https://openalex.org/W2161336914</t>
+          <t>https://openalex.org/W2135194391</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1145/2347736.2347755</t>
+          <t>https://doi.org/10.1023/a:1020281327116</t>
         </is>
       </c>
       <c r="D67" t="inlineStr"/>
       <c r="E67" t="inlineStr">
         <is>
-          <t>A few useful things to know about machine learning</t>
+          <t>An Introduction to MCMC for Machine Learning</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>Communications of the ACM</t>
+          <t>Machine Learning</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>Communications of the ACM</t>
+          <t>Machine Learning</t>
         </is>
       </c>
       <c r="H67" t="n">
-        <v>2012</v>
+        <v>2003</v>
       </c>
       <c r="I67" t="inlineStr">
         <is>
@@ -6677,64 +6681,60 @@
         </is>
       </c>
       <c r="K67" t="n">
-        <v>3253</v>
+        <v>2421</v>
       </c>
       <c r="L67" t="inlineStr">
         <is>
-          <t>Pedro Domingos</t>
+          <t>Christophe Andrieu;Nando de Freitas;Arnaud Doucet;Michael I. Jordan</t>
         </is>
       </c>
       <c r="M67" t="inlineStr"/>
       <c r="N67" t="inlineStr">
         <is>
-          <t>Pedro Domingos, University of Washington, Seattle</t>
+          <t>Christophe Andrieu, Department of Mathematics, Statistics Group, University of Bristol, University Walk, Bristol, BS8 1TW, UK;Christophe Andrieu, Department of Mathematics, Statistics Group, University of Bristol, University Walk, UK;Nando de Freitas, Department of Computer Science, University of British Columbia, 2366 Main Mall, Vancouver, BC, V6T 1Z4, Canada;Nando de Freitas, Department of Computer Science,  University of British Columbia,  Vancouver, Canada;Arnaud Doucet, Department of Electrical and Electronic Engineering, University of Melbourne, Parkville, Victoria, 3052, Australia;Arnaud Doucet, [Department of Electrical and Electronic Engineering, University of Melbourne, Parkville, Australia];Michael I. Jordan, Departments of Computer Science and Statistics, University of California at Berkeley, 387 Soda Hall, Berkeley, CA, 94720-1776, USA;Michael I. Jordan, Departments of Computer Science and Statistics, University of California at Berkeley, Berkeley, USA</t>
         </is>
       </c>
       <c r="O67" t="inlineStr"/>
       <c r="P67" t="inlineStr">
         <is>
-          <t>https://openalex.org/W1486658274; https://openalex.org/W1494137514; https://openalex.org/W1504694836; https://openalex.org/W1521062204; https://openalex.org/W1570448133; https://openalex.org/W1583837637; https://openalex.org/W1585009072; https://openalex.org/W1761022139; https://openalex.org/W1977970897; https://openalex.org/W2001141328; https://openalex.org/W2039683780; https://openalex.org/W2063961549; https://openalex.org/W2070902649; https://openalex.org/W2072128103; https://openalex.org/W2089624555; https://openalex.org/W2100483895; https://openalex.org/W2110065044; https://openalex.org/W2110228583; https://openalex.org/W2125055259; https://openalex.org/W2140785063; https://openalex.org/W2143891888; https://openalex.org/W2152761983; https://openalex.org/W2156909104; https://openalex.org/W2400138769; https://openalex.org/W2966207845; https://openalex.org/W3133236490; https://openalex.org/W3135029803; https://openalex.org/W4231109964; https://openalex.org/W4232632925; https://openalex.org/W4299515571; https://openalex.org/W6791387550</t>
+          <t>https://openalex.org/W23879647; https://openalex.org/W37728405; https://openalex.org/W69190551; https://openalex.org/W156498718; https://openalex.org/W195465510; https://openalex.org/W1481420047; https://openalex.org/W1483307070; https://openalex.org/W1486315527; https://openalex.org/W1493490444; https://openalex.org/W1494582337; https://openalex.org/W1506487567; https://openalex.org/W1509183771; https://openalex.org/W1509783656; https://openalex.org/W1510634602; https://openalex.org/W1515591979; https://openalex.org/W1528056001; https://openalex.org/W1530042113; https://openalex.org/W1548782607; https://openalex.org/W1561837455; https://openalex.org/W1565864173; https://openalex.org/W1567512734; https://openalex.org/W1571444101; https://openalex.org/W1578685895; https://openalex.org/W1582801283; https://openalex.org/W1587957970; https://openalex.org/W1600266325; https://openalex.org/W1606274310; https://openalex.org/W1607251184; https://openalex.org/W1824745232; https://openalex.org/W1829096983; https://openalex.org/W1854214752; https://openalex.org/W1880189740; https://openalex.org/W1894704206; https://openalex.org/W1966017656; https://openalex.org/W1969466749; https://openalex.org/W1973594349; https://openalex.org/W1974600023; https://openalex.org/W1978304080; https://openalex.org/W1984862890; https://openalex.org/W1985093013; https://openalex.org/W1986045245; https://openalex.org/W1988684120; https://openalex.org/W1990313671; https://openalex.org/W1990757250; https://openalex.org/W1994693590; https://openalex.org/W1994823593; https://openalex.org/W1995713768; https://openalex.org/W2002067385; https://openalex.org/W2004258534; https://openalex.org/W2008197960; https://openalex.org/W2008693968; https://openalex.org/W2015399216; https://openalex.org/W2017488093; https://openalex.org/W2019473674; https://openalex.org/W2020999234; https://openalex.org/W2024060531; https://openalex.org/W2024315245; https://openalex.org/W2037139490; https://openalex.org/W2038885294; https://openalex.org/W2042217732; https://openalex.org/W2047834101; https://openalex.org/W2049633694; https://openalex.org/W2051203581; https://openalex.org/W2056674749; https://openalex.org/W2056760934; https://openalex.org/W2057565703; https://openalex.org/W2059171997; https://openalex.org/W2059448777; https://openalex.org/W2063168839; https://openalex.org/W2063342497; https://openalex.org/W2066749736; https://openalex.org/W2069691149; https://openalex.org/W2069739265; https://openalex.org/W2071988465; https://openalex.org/W2072634211; https://openalex.org/W2076092328; https://openalex.org/W2080577297; https://openalex.org/W2082630584; https://openalex.org/W2082856185; https://openalex.org/W2083875149; https://openalex.org/W2084495102; https://openalex.org/W2086699924; https://openalex.org/W2087978636; https://openalex.org/W2089657469; https://openalex.org/W2090361527; https://openalex.org/W2091797506; https://openalex.org/W2093976733; https://openalex.org/W2094436494; https://openalex.org/W2096878708; https://openalex.org/W2098613108; https://openalex.org/W2103569423; https://openalex.org/W2106110775; https://openalex.org/W2106706098; https://openalex.org/W2108306139; https://openalex.org/W2113889826; https://openalex.org/W2116800676; https://openalex.org/W2117838564; https://openalex.org/W2118460912; https://openalex.org/W2121448470; https://openalex.org/W2121810339; https://openalex.org/W2122146783; https://openalex.org/W2122891730; https://openalex.org/W2123256163; https://openalex.org/W2124156864; https://openalex.org/W2126736494; https://openalex.org/W2127182131; https://openalex.org/W2128909582; https://openalex.org/W2128981260; https://openalex.org/W2130105580; https://openalex.org/W2130416410; https://openalex.org/W2131034613; https://openalex.org/W2131598171; https://openalex.org/W2132317470; https://openalex.org/W2134043769; https://openalex.org/W2134356662; https://openalex.org/W2136796925; https://openalex.org/W2138309709; https://openalex.org/W2140014834; https://openalex.org/W2143358994; https://openalex.org/W2147632348; https://openalex.org/W2149020252; https://openalex.org/W2150344704; https://openalex.org/W2152917223; https://openalex.org/W2152977846; https://openalex.org/W2154085356; https://openalex.org/W2154941050; https://openalex.org/W2158071659; https://openalex.org/W2161335636; https://openalex.org/W2163230106; https://openalex.org/W2163682810; https://openalex.org/W2171166780; https://openalex.org/W2171776966; https://openalex.org/W2322211931; https://openalex.org/W2322240213; https://openalex.org/W2341726179; https://openalex.org/W2343427443; https://openalex.org/W2582449852; https://openalex.org/W2613849015; https://openalex.org/W2914470628; https://openalex.org/W2950350592; https://openalex.org/W2950783152; https://openalex.org/W3006625324; https://openalex.org/W3037265734; https://openalex.org/W3105307699; https://openalex.org/W3121762057; https://openalex.org/W3143893444; https://openalex.org/W3160881378; https://openalex.org/W4213170070; https://openalex.org/W4229575850; https://openalex.org/W4230306435; https://openalex.org/W4230550322; https://openalex.org/W4232991410; https://openalex.org/W4233358567; https://openalex.org/W4235686993; https://openalex.org/W4241275264; https://openalex.org/W4241385190; https://openalex.org/W4241641375; https://openalex.org/W4244486013; https://openalex.org/W4245655784; https://openalex.org/W4245883374; https://openalex.org/W4246169471; https://openalex.org/W4246464108; https://openalex.org/W4247403446; https://openalex.org/W4247477375; https://openalex.org/W4247985008; https://openalex.org/W4247999480; https://openalex.org/W4248373945; https://openalex.org/W4249120700; https://openalex.org/W4252244571; https://openalex.org/W4254147434; https://openalex.org/W4285719527; https://openalex.org/W4292403327; https://openalex.org/W4302422232; https://openalex.org/W4302434451; https://openalex.org/W4302617909; https://openalex.org/W4387173443; https://openalex.org/W4388085068; https://openalex.org/W6601363074; https://openalex.org/W6629456519; https://openalex.org/W6629702432; https://openalex.org/W6631580585; https://openalex.org/W6634021638; https://openalex.org/W6634113456; https://openalex.org/W6635206105; https://openalex.org/W6638589003; https://openalex.org/W6639055396; https://openalex.org/W6647454992; https://openalex.org/W6652751995; https://openalex.org/W6656727730; https://openalex.org/W6668080254; https://openalex.org/W6677279966; https://openalex.org/W6678392814; https://openalex.org/W6679417241; https://openalex.org/W6683899899; https://openalex.org/W6828034933; https://openalex.org/W6998813755</t>
         </is>
       </c>
       <c r="Q67" t="inlineStr">
         <is>
-          <t>Computer science;Need to know;Artificial intelligence;Machine learning;Computer security</t>
+          <t>Computer science;Markov chain Monte Carlo;Monte Carlo method;Probabilistic logic;Artificial intelligence;Machine learning;Bayesian probability;Mathematics;Statistics</t>
         </is>
       </c>
       <c r="R67" t="inlineStr"/>
-      <c r="S67" t="inlineStr">
-        <is>
-          <t>Tapping into the "folk knowledge" needed to advance machine learning applications.</t>
-        </is>
-      </c>
+      <c r="S67" t="inlineStr"/>
       <c r="T67" t="inlineStr">
         <is>
-          <t>55</t>
+          <t>50</t>
         </is>
       </c>
       <c r="U67" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>1-2</t>
         </is>
       </c>
       <c r="V67" t="inlineStr">
         <is>
-          <t>78</t>
+          <t>5</t>
         </is>
       </c>
       <c r="W67" t="inlineStr">
         <is>
-          <t>87</t>
+          <t>43</t>
         </is>
       </c>
       <c r="X67" t="inlineStr">
         <is>
-          <t>Pedro Domingos, 2012, Communications of the ACM</t>
+          <t>Christophe Andrieu, 2003, Machine Learning</t>
         </is>
       </c>
       <c r="Y67" t="inlineStr">
         <is>
-          <t>Pedro Domingos, 2012, Communications of the ACM</t>
+          <t>Christophe Andrieu, 2003, Machine Learning</t>
         </is>
       </c>
     </row>
@@ -6784,7 +6784,7 @@
         </is>
       </c>
       <c r="K68" t="n">
-        <v>2440</v>
+        <v>2443</v>
       </c>
       <c r="L68" t="inlineStr">
         <is>
@@ -6845,36 +6845,36 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>https://openalex.org/W2135194391</t>
+          <t>https://openalex.org/W2111547563</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1023/a:1020281327116</t>
+          <t>https://doi.org/10.1016/j.csbj.2014.11.005</t>
         </is>
       </c>
       <c r="D69" t="inlineStr"/>
       <c r="E69" t="inlineStr">
         <is>
-          <t>An Introduction to MCMC for Machine Learning</t>
+          <t>Machine learning applications in cancer prognosis and prediction</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>Machine Learning</t>
+          <t>Computational and Structural Biotechnology Journal</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>Machine Learning</t>
+          <t>Computational and Structural Biotechnology Journal</t>
         </is>
       </c>
       <c r="H69" t="n">
-        <v>2003</v>
+        <v>2014</v>
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>article</t>
+          <t>review</t>
         </is>
       </c>
       <c r="J69" t="inlineStr">
@@ -6883,60 +6883,60 @@
         </is>
       </c>
       <c r="K69" t="n">
-        <v>2418</v>
+        <v>3307</v>
       </c>
       <c r="L69" t="inlineStr">
         <is>
-          <t>Christophe Andrieu;Nando de Freitas;Arnaud Doucet;Michael I. Jordan</t>
+          <t>Κωνσταντίνα Κούρου;Themis P. Exarchos;Konstantinos Exarchos;Michalis V. Karamouzis;Dimitrios I. Fotiadis</t>
         </is>
       </c>
       <c r="M69" t="inlineStr"/>
       <c r="N69" t="inlineStr">
         <is>
-          <t>Christophe Andrieu, Department of Mathematics, Statistics Group, University of Bristol, University Walk, Bristol, BS8 1TW, UK;Christophe Andrieu, Department of Mathematics, Statistics Group, University of Bristol, University Walk, UK;Nando de Freitas, Department of Computer Science, University of British Columbia, 2366 Main Mall, Vancouver, BC, V6T 1Z4, Canada;Nando de Freitas, Department of Computer Science,  University of British Columbia,  Vancouver, Canada;Arnaud Doucet, Department of Electrical and Electronic Engineering, University of Melbourne, Parkville, Victoria, 3052, Australia;Arnaud Doucet, [Department of Electrical and Electronic Engineering, University of Melbourne, Parkville, Australia];Michael I. Jordan, Departments of Computer Science and Statistics, University of California at Berkeley, 387 Soda Hall, Berkeley, CA, 94720-1776, USA;Michael I. Jordan, Departments of Computer Science and Statistics, University of California at Berkeley, Berkeley, USA</t>
+          <t>Κωνσταντίνα Κούρου, Unit of Medical Technology and Intelligent Information Systems, Dept. of Materials Science and Engineering, University of Ioannina, Ioannina, Greece;Themis P. Exarchos, IMBB — FORTH, Dept. of Biomedical Research, Ioannina, Greece;Themis P. Exarchos, Unit of Medical Technology and Intelligent Information Systems, Dept. of Materials Science and Engineering, University of Ioannina, Ioannina, Greece;Konstantinos Exarchos, Unit of Medical Technology and Intelligent Information Systems, Dept. of Materials Science and Engineering, University of Ioannina, Ioannina, Greece;Michalis V. Karamouzis, Molecular Oncology Unit, Department of Biological Chemistry, Medical School, University of Athens, Athens, Greece;Dimitrios I. Fotiadis, IMBB — FORTH, Dept. of Biomedical Research, Ioannina, Greece;Dimitrios I. Fotiadis, Unit of Medical Technology and Intelligent Information Systems, Dept. of Materials Science and Engineering, University of Ioannina, Ioannina, Greece</t>
         </is>
       </c>
       <c r="O69" t="inlineStr"/>
       <c r="P69" t="inlineStr">
         <is>
-          <t>https://openalex.org/W23879647; https://openalex.org/W37728405; https://openalex.org/W69190551; https://openalex.org/W156498718; https://openalex.org/W195465510; https://openalex.org/W1481420047; https://openalex.org/W1483307070; https://openalex.org/W1486315527; https://openalex.org/W1493490444; https://openalex.org/W1494582337; https://openalex.org/W1506487567; https://openalex.org/W1509183771; https://openalex.org/W1509783656; https://openalex.org/W1510634602; https://openalex.org/W1515591979; https://openalex.org/W1528056001; https://openalex.org/W1530042113; https://openalex.org/W1548782607; https://openalex.org/W1561837455; https://openalex.org/W1565864173; https://openalex.org/W1567512734; https://openalex.org/W1571444101; https://openalex.org/W1578685895; https://openalex.org/W1582801283; https://openalex.org/W1587957970; https://openalex.org/W1600266325; https://openalex.org/W1606274310; https://openalex.org/W1607251184; https://openalex.org/W1824745232; https://openalex.org/W1829096983; https://openalex.org/W1854214752; https://openalex.org/W1880189740; https://openalex.org/W1894704206; https://openalex.org/W1966017656; https://openalex.org/W1969466749; https://openalex.org/W1973594349; https://openalex.org/W1974600023; https://openalex.org/W1978304080; https://openalex.org/W1984862890; https://openalex.org/W1985093013; https://openalex.org/W1986045245; https://openalex.org/W1988684120; https://openalex.org/W1990313671; https://openalex.org/W1990757250; https://openalex.org/W1994693590; https://openalex.org/W1994823593; https://openalex.org/W1995713768; https://openalex.org/W2002067385; https://openalex.org/W2004258534; https://openalex.org/W2008197960; https://openalex.org/W2008693968; https://openalex.org/W2015399216; https://openalex.org/W2017488093; https://openalex.org/W2019473674; https://openalex.org/W2020999234; https://openalex.org/W2024060531; https://openalex.org/W2024315245; https://openalex.org/W2037139490; https://openalex.org/W2038885294; https://openalex.org/W2042217732; https://openalex.org/W2047834101; https://openalex.org/W2049633694; https://openalex.org/W2051203581; https://openalex.org/W2056674749; https://openalex.org/W2056760934; https://openalex.org/W2057565703; https://openalex.org/W2059171997; https://openalex.org/W2059448777; https://openalex.org/W2063168839; https://openalex.org/W2063342497; https://openalex.org/W2066749736; https://openalex.org/W2069691149; https://openalex.org/W2069739265; https://openalex.org/W2071988465; https://openalex.org/W2072634211; https://openalex.org/W2076092328; https://openalex.org/W2080577297; https://openalex.org/W2082630584; https://openalex.org/W2082856185; https://openalex.org/W2083875149; https://openalex.org/W2084495102; https://openalex.org/W2086699924; https://openalex.org/W2087978636; https://openalex.org/W2089657469; https://openalex.org/W2090361527; https://openalex.org/W2091797506; https://openalex.org/W2093976733; https://openalex.org/W2094436494; https://openalex.org/W2096878708; https://openalex.org/W2098613108; https://openalex.org/W2103569423; https://openalex.org/W2106110775; https://openalex.org/W2106706098; https://openalex.org/W2108306139; https://openalex.org/W2113889826; https://openalex.org/W2116800676; https://openalex.org/W2117838564; https://openalex.org/W2118460912; https://openalex.org/W2121448470; https://openalex.org/W2121810339; https://openalex.org/W2122146783; https://openalex.org/W2122891730; https://openalex.org/W2123256163; https://openalex.org/W2124156864; https://openalex.org/W2126736494; https://openalex.org/W2127182131; https://openalex.org/W2128909582; https://openalex.org/W2128981260; https://openalex.org/W2130105580; https://openalex.org/W2130416410; https://openalex.org/W2131034613; https://openalex.org/W2131598171; https://openalex.org/W2132317470; https://openalex.org/W2134043769; https://openalex.org/W2134356662; https://openalex.org/W2136796925; https://openalex.org/W2138309709; https://openalex.org/W2140014834; https://openalex.org/W2143358994; https://openalex.org/W2147632348; https://openalex.org/W2149020252; https://openalex.org/W2150344704; https://openalex.org/W2152917223; https://openalex.org/W2152977846; https://openalex.org/W2154085356; https://openalex.org/W2154941050; https://openalex.org/W2158071659; https://openalex.org/W2161335636; https://openalex.org/W2163230106; https://openalex.org/W2163682810; https://openalex.org/W2171166780; https://openalex.org/W2171776966; https://openalex.org/W2322211931; https://openalex.org/W2322240213; https://openalex.org/W2341726179; https://openalex.org/W2343427443; https://openalex.org/W2582449852; https://openalex.org/W2613849015; https://openalex.org/W2914470628; https://openalex.org/W2950350592; https://openalex.org/W2950783152; https://openalex.org/W3006625324; https://openalex.org/W3037265734; https://openalex.org/W3105307699; https://openalex.org/W3121762057; https://openalex.org/W3143893444; https://openalex.org/W3160881378; https://openalex.org/W4213170070; https://openalex.org/W4229575850; https://openalex.org/W4230306435; https://openalex.org/W4230550322; https://openalex.org/W4232991410; https://openalex.org/W4233358567; https://openalex.org/W4235686993; https://openalex.org/W4241275264; https://openalex.org/W4241385190; https://openalex.org/W4241641375; https://openalex.org/W4244486013; https://openalex.org/W4245655784; https://openalex.org/W4245883374; https://openalex.org/W4246169471; https://openalex.org/W4246464108; https://openalex.org/W4247403446; https://openalex.org/W4247477375; https://openalex.org/W4247985008; https://openalex.org/W4247999480; https://openalex.org/W4248373945; https://openalex.org/W4249120700; https://openalex.org/W4252244571; https://openalex.org/W4254147434; https://openalex.org/W4285719527; https://openalex.org/W4292403327; https://openalex.org/W4302422232; https://openalex.org/W4302434451; https://openalex.org/W4302617909; https://openalex.org/W4387173443; https://openalex.org/W4388085068; https://openalex.org/W6601363074; https://openalex.org/W6629456519; https://openalex.org/W6629702432; https://openalex.org/W6631580585; https://openalex.org/W6634021638; https://openalex.org/W6634113456; https://openalex.org/W6635206105; https://openalex.org/W6638589003; https://openalex.org/W6639055396; https://openalex.org/W6647454992; https://openalex.org/W6652751995; https://openalex.org/W6656727730; https://openalex.org/W6668080254; https://openalex.org/W6677279966; https://openalex.org/W6678392814; https://openalex.org/W6679417241; https://openalex.org/W6683899899; https://openalex.org/W6828034933; https://openalex.org/W6998813755</t>
+          <t>https://openalex.org/W1491953704; https://openalex.org/W1500572886; https://openalex.org/W1517879388; https://openalex.org/W1519433744; https://openalex.org/W1565377632; https://openalex.org/W1570448133; https://openalex.org/W1591717158; https://openalex.org/W1651586605; https://openalex.org/W1663973292; https://openalex.org/W1960669649; https://openalex.org/W1971005400; https://openalex.org/W1978761216; https://openalex.org/W1983024255; https://openalex.org/W1985663400; https://openalex.org/W1987776395; https://openalex.org/W1989628460; https://openalex.org/W1992297816; https://openalex.org/W1993628165; https://openalex.org/W1995199599; https://openalex.org/W2007265575; https://openalex.org/W2011021469; https://openalex.org/W2014510428; https://openalex.org/W2017337590; https://openalex.org/W2020402396; https://openalex.org/W2021100122; https://openalex.org/W2025060250; https://openalex.org/W2025738103; https://openalex.org/W2036839465; https://openalex.org/W2041652340; https://openalex.org/W2048701123; https://openalex.org/W2053522428; https://openalex.org/W2058089746; https://openalex.org/W2062364738; https://openalex.org/W2083780116; https://openalex.org/W2088338744; https://openalex.org/W2089927030; https://openalex.org/W2091947792; https://openalex.org/W2097554668; https://openalex.org/W2105882193; https://openalex.org/W2109103446; https://openalex.org/W2109896839; https://openalex.org/W2111461407; https://openalex.org/W2116841457; https://openalex.org/W2117692326; https://openalex.org/W2118366842; https://openalex.org/W2119782683; https://openalex.org/W2122227569; https://openalex.org/W2123696692; https://openalex.org/W2126009609; https://openalex.org/W2128767954; https://openalex.org/W2130338776; https://openalex.org/W2132619562; https://openalex.org/W2133601033; https://openalex.org/W2140218006; https://openalex.org/W2148078825; https://openalex.org/W2152121590; https://openalex.org/W2154362705; https://openalex.org/W2155461561; https://openalex.org/W2156483112; https://openalex.org/W2157132621; https://openalex.org/W2157239837; https://openalex.org/W2163042952; https://openalex.org/W2167645795; https://openalex.org/W2167769381; https://openalex.org/W2170379523; https://openalex.org/W2324845196; https://openalex.org/W2431164060; https://openalex.org/W2476253186; https://openalex.org/W2977661550; https://openalex.org/W4205774955; https://openalex.org/W4255865525; https://openalex.org/W4296886862; https://openalex.org/W6660969321; https://openalex.org/W6663876547</t>
         </is>
       </c>
       <c r="Q69" t="inlineStr">
         <is>
-          <t>Computer science;Markov chain Monte Carlo;Monte Carlo method;Probabilistic logic;Artificial intelligence;Machine learning;Bayesian probability;Mathematics;Statistics</t>
+          <t>Machine learning;Artificial intelligence;Computer science;Support vector machine;Cancer;Artificial neural network;Bayesian network;Clinical Practice;Variety (cybernetics);Field (mathematics);Predictive modelling;Medicine;Mathematics</t>
         </is>
       </c>
       <c r="R69" t="inlineStr"/>
-      <c r="S69" t="inlineStr"/>
+      <c r="S69" t="inlineStr">
+        <is>
+          <t>Cancer has been characterized as a heterogeneous disease consisting of many different subtypes. The early diagnosis and prognosis of a cancer type have become a necessity in cancer research, as it can facilitate the subsequent clinical management of patients. The importance of classifying cancer patients into high or low risk groups has led many research teams, from the biomedical and the bioinformatics field, to study the application of machine learning (ML) methods. Therefore, these techniques have been utilized as an aim to model the progression and treatment of cancerous conditions. In addition, the ability of ML tools to detect key features from complex datasets reveals their importance. A variety of these techniques, including Artificial Neural Networks (ANNs), Bayesian Networks (BNs), Support Vector Machines (SVMs) and Decision Trees (DTs) have been widely applied in cancer research for the development of predictive models, resulting in effective and accurate decision making. Even though it is evident that the use of ML methods can improve our understanding of cancer progression, an appropriate level of validation is needed in order for these methods to be considered in the everyday clinical practice. In this work, we present a review of recent ML approaches employed in the modeling of cancer progression. The predictive models discussed here are based on various supervised ML techniques as well as on different input features and data samples. Given the growing trend on the application of ML methods in cancer research, we present here the most recent publications that employ these techniques as an aim to model cancer risk or patient outcomes.</t>
+        </is>
+      </c>
       <c r="T69" t="inlineStr">
         <is>
-          <t>50</t>
-        </is>
-      </c>
-      <c r="U69" t="inlineStr">
-        <is>
-          <t>1-2</t>
-        </is>
-      </c>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="U69" t="inlineStr"/>
       <c r="V69" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>8</t>
         </is>
       </c>
       <c r="W69" t="inlineStr">
         <is>
-          <t>43</t>
+          <t>17</t>
         </is>
       </c>
       <c r="X69" t="inlineStr">
         <is>
-          <t>Christophe Andrieu, 2003, Machine Learning</t>
+          <t>Κωνσταντίνα Κούρου, 2014, Computational and Structural Biotechnology Journal</t>
         </is>
       </c>
       <c r="Y69" t="inlineStr">
         <is>
-          <t>Christophe Andrieu, 2003, Machine Learning</t>
+          <t>Κωνσταντίνα Κούρου, 2014, Computational and Structural Biotechnology Journal</t>
         </is>
       </c>
     </row>
@@ -6986,7 +6986,7 @@
         </is>
       </c>
       <c r="K70" t="n">
-        <v>3515</v>
+        <v>3520</v>
       </c>
       <c r="L70" t="inlineStr">
         <is>
@@ -7085,7 +7085,7 @@
         </is>
       </c>
       <c r="K71" t="n">
-        <v>3486</v>
+        <v>3488</v>
       </c>
       <c r="L71" t="inlineStr">
         <is>
@@ -7176,7 +7176,7 @@
         </is>
       </c>
       <c r="K72" t="n">
-        <v>24483</v>
+        <v>24503</v>
       </c>
       <c r="L72" t="inlineStr">
         <is>
@@ -7275,7 +7275,7 @@
         </is>
       </c>
       <c r="K73" t="n">
-        <v>13888</v>
+        <v>13889</v>
       </c>
       <c r="L73" t="inlineStr">
         <is>
@@ -7362,7 +7362,7 @@
         </is>
       </c>
       <c r="K74" t="n">
-        <v>2080</v>
+        <v>2084</v>
       </c>
       <c r="L74" t="inlineStr">
         <is>
@@ -7498,36 +7498,36 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>https://openalex.org/W3116286104</t>
+          <t>https://openalex.org/W2594639291</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>https://doi.org/10.3390/e23010018</t>
+          <t>https://doi.org/10.5860/choice.44-5091</t>
         </is>
       </c>
       <c r="D76" t="inlineStr"/>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Explainable AI: A Review of Machine Learning Interpretability Methods</t>
+          <t>Pattern recognition and machine learning</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>Entropy</t>
+          <t>Choice Reviews Online</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>Entropy</t>
+          <t>Choice Reviews Online</t>
         </is>
       </c>
       <c r="H76" t="n">
-        <v>2020</v>
+        <v>2007</v>
       </c>
       <c r="I76" t="inlineStr">
         <is>
-          <t>review</t>
+          <t>article</t>
         </is>
       </c>
       <c r="J76" t="inlineStr">
@@ -7536,64 +7536,48 @@
         </is>
       </c>
       <c r="K76" t="n">
-        <v>2760</v>
-      </c>
-      <c r="L76" t="inlineStr">
-        <is>
-          <t>Pantelis Linardatos;Vasilis Papastefanopoulos;Sotiris Kotsiantis</t>
-        </is>
-      </c>
+        <v>2688</v>
+      </c>
+      <c r="L76" t="inlineStr"/>
       <c r="M76" t="inlineStr"/>
-      <c r="N76" t="inlineStr">
-        <is>
-          <t>Pantelis Linardatos, Department of Mathematics, University of Patras, 26504 Patras, Greece;Vasilis Papastefanopoulos, Department of Mathematics, University of Patras, 26504 Patras, Greece;Sotiris Kotsiantis, Department of Mathematics, University of Patras, 26504 Patras, Greece</t>
-        </is>
-      </c>
+      <c r="N76" t="inlineStr"/>
       <c r="O76" t="inlineStr"/>
-      <c r="P76" t="inlineStr">
-        <is>
-          <t>https://openalex.org/W100464641; https://openalex.org/W273955616; https://openalex.org/W999207820; https://openalex.org/W1678356000; https://openalex.org/W1787224781; https://openalex.org/W1825675169; https://openalex.org/W1849277567; https://openalex.org/W1901616594; https://openalex.org/W1942214758; https://openalex.org/W1945616565; https://openalex.org/W1961345416; https://openalex.org/W1979362125; https://openalex.org/W1979769549; https://openalex.org/W1994080277; https://openalex.org/W1996796871; https://openalex.org/W2014352947; https://openalex.org/W2029767409; https://openalex.org/W2035363534; https://openalex.org/W2044639673; https://openalex.org/W2046945713; https://openalex.org/W2066238228; https://openalex.org/W2088765131; https://openalex.org/W2097246321; https://openalex.org/W2100960835; https://openalex.org/W2101589741; https://openalex.org/W2102636708; https://openalex.org/W2116572416; https://openalex.org/W2116666691; https://openalex.org/W2116984840; https://openalex.org/W2123045220; https://openalex.org/W2125283600; https://openalex.org/W2125847307; https://openalex.org/W2128272608; https://openalex.org/W2141200610; https://openalex.org/W2141755357; https://openalex.org/W2151868609; https://openalex.org/W2157928966; https://openalex.org/W2163605009; https://openalex.org/W2164878629; https://openalex.org/W2180612164; https://openalex.org/W2195388612; https://openalex.org/W2243397390; https://openalex.org/W2282821441; https://openalex.org/W2295107390; https://openalex.org/W2295598076; https://openalex.org/W2336525064; https://openalex.org/W2396394641; https://openalex.org/W2440159969; https://openalex.org/W2483215953; https://openalex.org/W2484189903; https://openalex.org/W2492294785; https://openalex.org/W2535873859; https://openalex.org/W2543927648; https://openalex.org/W2551974706; https://openalex.org/W2556096924; https://openalex.org/W2570685808; https://openalex.org/W2594475271; https://openalex.org/W2597603852; https://openalex.org/W2603766943; https://openalex.org/W2605409611; https://openalex.org/W2609368435; https://openalex.org/W2618851150; https://openalex.org/W2626639386; https://openalex.org/W2732560823; https://openalex.org/W2734421735; https://openalex.org/W2739220786; https://openalex.org/W2745565856; https://openalex.org/W2746600820; https://openalex.org/W2755655609; https://openalex.org/W2765424254; https://openalex.org/W2765793020; https://openalex.org/W2768894107; https://openalex.org/W2770312844; https://openalex.org/W2773022113; https://openalex.org/W2773497437; https://openalex.org/W2774644650; https://openalex.org/W2785699986; https://openalex.org/W2787955716; https://openalex.org/W2788199784; https://openalex.org/W2788403449; https://openalex.org/W2789160704; https://openalex.org/W2792942633; https://openalex.org/W2796215194; https://openalex.org/W2796885425; https://openalex.org/W2798312813; https://openalex.org/W2799194071; https://openalex.org/W2803831897; https://openalex.org/W2809136100; https://openalex.org/W2887252986; https://openalex.org/W2888078780; https://openalex.org/W2888421747; https://openalex.org/W2889210204; https://openalex.org/W2889252776; https://openalex.org/W2891503716; https://openalex.org/W2905526464; https://openalex.org/W2905810301; https://openalex.org/W2909878761; https://openalex.org/W2910705748; https://openalex.org/W2914598080; https://openalex.org/W2919115771; https://openalex.org/W2943646750; https://openalex.org/W2949128310; https://openalex.org/W2949197630; https://openalex.org/W2949200088; https://openalex.org/W2953911539; https://openalex.org/W2954503794; https://openalex.org/W2955782190; https://openalex.org/W2962718684; https://openalex.org/W2962772482; https://openalex.org/W2962790223; https://openalex.org/W2962816513; https://openalex.org/W2962818281; https://openalex.org/W2962858109; https://openalex.org/W2963095307; https://openalex.org/W2963100392; https://openalex.org/W2963116854; https://openalex.org/W2963125461; https://openalex.org/W2963126845; https://openalex.org/W2963165363; https://openalex.org/W2963233086; https://openalex.org/W2963382180; https://openalex.org/W2963483561; https://openalex.org/W2963615251; https://openalex.org/W2963847595; https://openalex.org/W2963857521; https://openalex.org/W2963859254; https://openalex.org/W2963969878; https://openalex.org/W2964082701; https://openalex.org/W2965749257; https://openalex.org/W2966149470; https://openalex.org/W2971970905; https://openalex.org/W2981731882; https://openalex.org/W2988194011; https://openalex.org/W2998277219; https://openalex.org/W3000208741; https://openalex.org/W3003420231; https://openalex.org/W3013371788; https://openalex.org/W3015625436; https://openalex.org/W3023553115; https://openalex.org/W3027870051; https://openalex.org/W3035517615; https://openalex.org/W3035736465; https://openalex.org/W3037881545; https://openalex.org/W3098276446; https://openalex.org/W3098278632; https://openalex.org/W3099126561; https://openalex.org/W3101449015; https://openalex.org/W3102476541; https://openalex.org/W3103557498; https://openalex.org/W3104423855; https://openalex.org/W3104570147; https://openalex.org/W3106412272; https://openalex.org/W3121410165; https://openalex.org/W3121588992; https://openalex.org/W3138819813; https://openalex.org/W4238293282; https://openalex.org/W4241793634; https://openalex.org/W4251708881; https://openalex.org/W4288625073; https://openalex.org/W4289258088; https://openalex.org/W4300337452; https://openalex.org/W6610017368; https://openalex.org/W6637162671; https://openalex.org/W6684072790; https://openalex.org/W6703326205; https://openalex.org/W6719080892; https://openalex.org/W6728551298; https://openalex.org/W6733049761; https://openalex.org/W6734194636; https://openalex.org/W6739575509; https://openalex.org/W6740085662; https://openalex.org/W6744110554; https://openalex.org/W6745730051; https://openalex.org/W6747473890; https://openalex.org/W6748377460; https://openalex.org/W6750628419; https://openalex.org/W6750829902; https://openalex.org/W6751569023; https://openalex.org/W6751776086; https://openalex.org/W6752083044; https://openalex.org/W6755768460; https://openalex.org/W6762840784; https://openalex.org/W6765646913; https://openalex.org/W7014198846</t>
-        </is>
-      </c>
+      <c r="P76" t="inlineStr"/>
       <c r="Q76" t="inlineStr">
         <is>
-          <t>Interpretability;Artificial intelligence;Computer science;Machine learning;Ambiguity;Field (mathematics);Implementation;Black box;Management science;Data science;Software engineering;Engineering</t>
+          <t>Artificial intelligence;Computer science;Pattern recognition (psychology);Psychology</t>
         </is>
       </c>
       <c r="R76" t="inlineStr"/>
-      <c r="S76" t="inlineStr">
-        <is>
-          <t>Recent advances in artificial intelligence (AI) have led to its widespread industrial adoption, with machine learning systems demonstrating superhuman performance in a significant number of tasks. However, this surge in performance, has often been achieved through increased model complexity, turning such systems into "black box" approaches and causing uncertainty regarding the way they operate and, ultimately, the way that they come to decisions. This ambiguity has made it problematic for machine learning systems to be adopted in sensitive yet critical domains, where their value could be immense, such as healthcare. As a result, scientific interest in the field of Explainable Artificial Intelligence (XAI), a field that is concerned with the development of new methods that explain and interpret machine learning models, has been tremendously reignited over recent years. This study focuses on machine learning interpretability methods; more specifically, a literature review and taxonomy of these methods are presented, as well as links to their programming implementations, in the hope that this survey would serve as a reference point for both theorists and practitioners.</t>
-        </is>
-      </c>
+      <c r="S76" t="inlineStr"/>
       <c r="T76" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>44</t>
         </is>
       </c>
       <c r="U76" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>09</t>
         </is>
       </c>
       <c r="V76" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>44</t>
         </is>
       </c>
       <c r="W76" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>5091</t>
         </is>
       </c>
       <c r="X76" t="inlineStr">
         <is>
-          <t>Pantelis Linardatos, 2020, Entropy</t>
+          <t>NA, 2007, Choice Reviews Online</t>
         </is>
       </c>
       <c r="Y76" t="inlineStr">
         <is>
-          <t>Pantelis Linardatos, 2020, Entropy</t>
+          <t>NA, 2007, Choice Reviews Online</t>
         </is>
       </c>
     </row>
@@ -7605,36 +7589,36 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>https://openalex.org/W2594639291</t>
+          <t>https://openalex.org/W3116286104</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>https://doi.org/10.5860/choice.44-5091</t>
+          <t>https://doi.org/10.3390/e23010018</t>
         </is>
       </c>
       <c r="D77" t="inlineStr"/>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Pattern recognition and machine learning</t>
+          <t>Explainable AI: A Review of Machine Learning Interpretability Methods</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>Choice Reviews Online</t>
+          <t>Entropy</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>Choice Reviews Online</t>
+          <t>Entropy</t>
         </is>
       </c>
       <c r="H77" t="n">
-        <v>2007</v>
+        <v>2020</v>
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>article</t>
+          <t>review</t>
         </is>
       </c>
       <c r="J77" t="inlineStr">
@@ -7643,48 +7627,64 @@
         </is>
       </c>
       <c r="K77" t="n">
-        <v>2688</v>
-      </c>
-      <c r="L77" t="inlineStr"/>
+        <v>2764</v>
+      </c>
+      <c r="L77" t="inlineStr">
+        <is>
+          <t>Pantelis Linardatos;Vasilis Papastefanopoulos;Sotiris Kotsiantis</t>
+        </is>
+      </c>
       <c r="M77" t="inlineStr"/>
-      <c r="N77" t="inlineStr"/>
+      <c r="N77" t="inlineStr">
+        <is>
+          <t>Pantelis Linardatos, Department of Mathematics, University of Patras, 26504 Patras, Greece;Vasilis Papastefanopoulos, Department of Mathematics, University of Patras, 26504 Patras, Greece;Sotiris Kotsiantis, Department of Mathematics, University of Patras, 26504 Patras, Greece</t>
+        </is>
+      </c>
       <c r="O77" t="inlineStr"/>
-      <c r="P77" t="inlineStr"/>
+      <c r="P77" t="inlineStr">
+        <is>
+          <t>https://openalex.org/W100464641; https://openalex.org/W273955616; https://openalex.org/W999207820; https://openalex.org/W1678356000; https://openalex.org/W1787224781; https://openalex.org/W1825675169; https://openalex.org/W1849277567; https://openalex.org/W1901616594; https://openalex.org/W1942214758; https://openalex.org/W1945616565; https://openalex.org/W1961345416; https://openalex.org/W1979362125; https://openalex.org/W1979769549; https://openalex.org/W1994080277; https://openalex.org/W1996796871; https://openalex.org/W2014352947; https://openalex.org/W2029767409; https://openalex.org/W2035363534; https://openalex.org/W2044639673; https://openalex.org/W2046945713; https://openalex.org/W2066238228; https://openalex.org/W2088765131; https://openalex.org/W2097246321; https://openalex.org/W2100960835; https://openalex.org/W2101589741; https://openalex.org/W2102636708; https://openalex.org/W2116572416; https://openalex.org/W2116666691; https://openalex.org/W2116984840; https://openalex.org/W2123045220; https://openalex.org/W2125283600; https://openalex.org/W2125847307; https://openalex.org/W2128272608; https://openalex.org/W2141200610; https://openalex.org/W2141755357; https://openalex.org/W2151868609; https://openalex.org/W2157928966; https://openalex.org/W2163605009; https://openalex.org/W2164878629; https://openalex.org/W2180612164; https://openalex.org/W2195388612; https://openalex.org/W2243397390; https://openalex.org/W2282821441; https://openalex.org/W2295107390; https://openalex.org/W2295598076; https://openalex.org/W2336525064; https://openalex.org/W2396394641; https://openalex.org/W2440159969; https://openalex.org/W2483215953; https://openalex.org/W2484189903; https://openalex.org/W2492294785; https://openalex.org/W2535873859; https://openalex.org/W2543927648; https://openalex.org/W2551974706; https://openalex.org/W2556096924; https://openalex.org/W2570685808; https://openalex.org/W2594475271; https://openalex.org/W2597603852; https://openalex.org/W2603766943; https://openalex.org/W2605409611; https://openalex.org/W2609368435; https://openalex.org/W2618851150; https://openalex.org/W2626639386; https://openalex.org/W2732560823; https://openalex.org/W2734421735; https://openalex.org/W2739220786; https://openalex.org/W2745565856; https://openalex.org/W2746600820; https://openalex.org/W2755655609; https://openalex.org/W2765424254; https://openalex.org/W2765793020; https://openalex.org/W2768894107; https://openalex.org/W2770312844; https://openalex.org/W2773022113; https://openalex.org/W2773497437; https://openalex.org/W2774644650; https://openalex.org/W2785699986; https://openalex.org/W2787955716; https://openalex.org/W2788199784; https://openalex.org/W2788403449; https://openalex.org/W2789160704; https://openalex.org/W2792942633; https://openalex.org/W2796215194; https://openalex.org/W2796885425; https://openalex.org/W2798312813; https://openalex.org/W2799194071; https://openalex.org/W2803831897; https://openalex.org/W2809136100; https://openalex.org/W2887252986; https://openalex.org/W2888078780; https://openalex.org/W2888421747; https://openalex.org/W2889210204; https://openalex.org/W2889252776; https://openalex.org/W2891503716; https://openalex.org/W2905526464; https://openalex.org/W2905810301; https://openalex.org/W2909878761; https://openalex.org/W2910705748; https://openalex.org/W2914598080; https://openalex.org/W2919115771; https://openalex.org/W2943646750; https://openalex.org/W2949128310; https://openalex.org/W2949197630; https://openalex.org/W2949200088; https://openalex.org/W2953911539; https://openalex.org/W2954503794; https://openalex.org/W2955782190; https://openalex.org/W2962718684; https://openalex.org/W2962772482; https://openalex.org/W2962790223; https://openalex.org/W2962816513; https://openalex.org/W2962818281; https://openalex.org/W2962858109; https://openalex.org/W2963095307; https://openalex.org/W2963100392; https://openalex.org/W2963116854; https://openalex.org/W2963125461; https://openalex.org/W2963126845; https://openalex.org/W2963165363; https://openalex.org/W2963233086; https://openalex.org/W2963382180; https://openalex.org/W2963483561; https://openalex.org/W2963615251; https://openalex.org/W2963847595; https://openalex.org/W2963857521; https://openalex.org/W2963859254; https://openalex.org/W2963969878; https://openalex.org/W2964082701; https://openalex.org/W2965749257; https://openalex.org/W2966149470; https://openalex.org/W2971970905; https://openalex.org/W2981731882; https://openalex.org/W2988194011; https://openalex.org/W2998277219; https://openalex.org/W3000208741; https://openalex.org/W3003420231; https://openalex.org/W3013371788; https://openalex.org/W3015625436; https://openalex.org/W3023553115; https://openalex.org/W3027870051; https://openalex.org/W3035517615; https://openalex.org/W3035736465; https://openalex.org/W3037881545; https://openalex.org/W3098276446; https://openalex.org/W3098278632; https://openalex.org/W3099126561; https://openalex.org/W3101449015; https://openalex.org/W3102476541; https://openalex.org/W3103557498; https://openalex.org/W3104423855; https://openalex.org/W3104570147; https://openalex.org/W3106412272; https://openalex.org/W3121410165; https://openalex.org/W3121588992; https://openalex.org/W3138819813; https://openalex.org/W4238293282; https://openalex.org/W4241793634; https://openalex.org/W4251708881; https://openalex.org/W4288625073; https://openalex.org/W4289258088; https://openalex.org/W4300337452; https://openalex.org/W6610017368; https://openalex.org/W6637162671; https://openalex.org/W6684072790; https://openalex.org/W6703326205; https://openalex.org/W6719080892; https://openalex.org/W6728551298; https://openalex.org/W6733049761; https://openalex.org/W6734194636; https://openalex.org/W6739575509; https://openalex.org/W6740085662; https://openalex.org/W6744110554; https://openalex.org/W6745730051; https://openalex.org/W6747473890; https://openalex.org/W6748377460; https://openalex.org/W6750628419; https://openalex.org/W6750829902; https://openalex.org/W6751569023; https://openalex.org/W6751776086; https://openalex.org/W6752083044; https://openalex.org/W6755768460; https://openalex.org/W6762840784; https://openalex.org/W6765646913; https://openalex.org/W7014198846</t>
+        </is>
+      </c>
       <c r="Q77" t="inlineStr">
         <is>
-          <t>Artificial intelligence;Computer science;Pattern recognition (psychology);Psychology</t>
+          <t>Interpretability;Artificial intelligence;Computer science;Machine learning;Ambiguity;Field (mathematics);Implementation;Black box;Management science;Data science;Software engineering;Engineering</t>
         </is>
       </c>
       <c r="R77" t="inlineStr"/>
-      <c r="S77" t="inlineStr"/>
+      <c r="S77" t="inlineStr">
+        <is>
+          <t>Recent advances in artificial intelligence (AI) have led to its widespread industrial adoption, with machine learning systems demonstrating superhuman performance in a significant number of tasks. However, this surge in performance, has often been achieved through increased model complexity, turning such systems into "black box" approaches and causing uncertainty regarding the way they operate and, ultimately, the way that they come to decisions. This ambiguity has made it problematic for machine learning systems to be adopted in sensitive yet critical domains, where their value could be immense, such as healthcare. As a result, scientific interest in the field of Explainable Artificial Intelligence (XAI), a field that is concerned with the development of new methods that explain and interpret machine learning models, has been tremendously reignited over recent years. This study focuses on machine learning interpretability methods; more specifically, a literature review and taxonomy of these methods are presented, as well as links to their programming implementations, in the hope that this survey would serve as a reference point for both theorists and practitioners.</t>
+        </is>
+      </c>
       <c r="T77" t="inlineStr">
         <is>
-          <t>44</t>
+          <t>23</t>
         </is>
       </c>
       <c r="U77" t="inlineStr">
         <is>
-          <t>09</t>
+          <t>1</t>
         </is>
       </c>
       <c r="V77" t="inlineStr">
         <is>
-          <t>44</t>
+          <t>18</t>
         </is>
       </c>
       <c r="W77" t="inlineStr">
         <is>
-          <t>5091</t>
+          <t>18</t>
         </is>
       </c>
       <c r="X77" t="inlineStr">
         <is>
-          <t>NA, 2007, Choice Reviews Online</t>
+          <t>Pantelis Linardatos, 2020, Entropy</t>
         </is>
       </c>
       <c r="Y77" t="inlineStr">
         <is>
-          <t>NA, 2007, Choice Reviews Online</t>
+          <t>Pantelis Linardatos, 2020, Entropy</t>
         </is>
       </c>
     </row>
@@ -7928,7 +7928,7 @@
         </is>
       </c>
       <c r="K80" t="n">
-        <v>13182</v>
+        <v>13187</v>
       </c>
       <c r="L80" t="inlineStr">
         <is>
@@ -7993,36 +7993,28 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>https://openalex.org/W2751318774</t>
+          <t>https://openalex.org/W2767079719</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1142/9789811201967_0001</t>
+          <t>https://doi.org/10.1145/3133956.3133982</t>
         </is>
       </c>
       <c r="D81" t="inlineStr"/>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Introduction to Machine Learning</t>
-        </is>
-      </c>
-      <c r="F81" t="inlineStr">
-        <is>
-          <t>Series in machine perception and artificial intelligence</t>
-        </is>
-      </c>
-      <c r="G81" t="inlineStr">
-        <is>
-          <t>Series in machine perception and artificial intelligence</t>
-        </is>
-      </c>
+          <t>Practical Secure Aggregation for Privacy-Preserving Machine Learning</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr"/>
+      <c r="G81" t="inlineStr"/>
       <c r="H81" t="n">
-        <v>2019</v>
+        <v>2017</v>
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>book-chapter</t>
+          <t>article</t>
         </is>
       </c>
       <c r="J81" t="inlineStr">
@@ -8031,44 +8023,56 @@
         </is>
       </c>
       <c r="K81" t="n">
-        <v>1659</v>
-      </c>
-      <c r="L81" t="inlineStr"/>
+        <v>3461</v>
+      </c>
+      <c r="L81" t="inlineStr">
+        <is>
+          <t>Keith Bonawitz;Vladimir Ivanov;Ben Kreuter;Antonio Marcedone;H. Brendan McMahan;Sarvar Patel;Daniel Ramage;Aaron Segal;Karn Seth</t>
+        </is>
+      </c>
       <c r="M81" t="inlineStr"/>
-      <c r="N81" t="inlineStr"/>
+      <c r="N81" t="inlineStr">
+        <is>
+          <t>Keith Bonawitz, Google Inc., Mountain View, CA, USA;Vladimir Ivanov, Google Inc., Mountain View, CA, USA;Ben Kreuter, Google Inc., Mountain View, CA, USA;Antonio Marcedone, Cornell Tech &amp;amp;Google Inc., New York, NY, USA;H. Brendan McMahan, Google Inc., Mountain View, CA, USA;Sarvar Patel, Google Inc., Mountain View, CA, USA;Daniel Ramage, Google Inc., Mountain View, CA, USA;Aaron Segal, Google Inc., Mountain View, CA, USA;Karn Seth, Google Inc., Mountain View, CA, USA</t>
+        </is>
+      </c>
       <c r="O81" t="inlineStr"/>
-      <c r="P81" t="inlineStr"/>
+      <c r="P81" t="inlineStr">
+        <is>
+          <t>https://openalex.org/W25045116; https://openalex.org/W95608104; https://openalex.org/W1071368427; https://openalex.org/W1493407996; https://openalex.org/W1519947574; https://openalex.org/W1557833142; https://openalex.org/W1595357546; https://openalex.org/W1656028867; https://openalex.org/W1836711297; https://openalex.org/W1952161176; https://openalex.org/W1952958290; https://openalex.org/W1981029888; https://openalex.org/W2006453614; https://openalex.org/W2027471022; https://openalex.org/W2027595342; https://openalex.org/W2033974828; https://openalex.org/W2051267297; https://openalex.org/W2053637704; https://openalex.org/W2053801139; https://openalex.org/W2058648304; https://openalex.org/W2061106457; https://openalex.org/W2069657084; https://openalex.org/W2087811006; https://openalex.org/W2104803737; https://openalex.org/W2128865076; https://openalex.org/W2135930857; https://openalex.org/W2141420453; https://openalex.org/W2146673169; https://openalex.org/W2149093588; https://openalex.org/W2152768255; https://openalex.org/W2156186849; https://openalex.org/W2163481970; https://openalex.org/W2164284862; https://openalex.org/W2200869402; https://openalex.org/W2232997092; https://openalex.org/W2267098117; https://openalex.org/W2295522738; https://openalex.org/W2336650964; https://openalex.org/W2400777838; https://openalex.org/W2402235285; https://openalex.org/W2413533038; https://openalex.org/W2473418344; https://openalex.org/W2525846285; https://openalex.org/W2535690855; https://openalex.org/W2536058570; https://openalex.org/W2538520193; https://openalex.org/W2541884796; https://openalex.org/W2557283755; https://openalex.org/W2568821124; https://openalex.org/W2599930814; https://openalex.org/W2911978475; https://openalex.org/W2951114885; https://openalex.org/W3031847131; https://openalex.org/W3102407811; https://openalex.org/W3141405531; https://openalex.org/W3150645827</t>
+        </is>
+      </c>
       <c r="Q81" t="inlineStr">
         <is>
-          <t>Computer science;Artificial intelligence</t>
+          <t>Computer science;Overhead (engineering);Protocol (science);Universal composability;Adversary;Computer network;Aggregate (composite);Cryptographic protocol;Distributed computing;Theoretical computer science;Cryptography;Computer security;Operating system</t>
         </is>
       </c>
       <c r="R81" t="inlineStr"/>
       <c r="S81" t="inlineStr">
         <is>
-          <t>The goal of machine learning is to program computers to use example data or past experience to solve a given problem. Many successful applications of machine learning exist already, including systems that analyze past sales data to predict customer behavior, optimize robot behavior so that a task can be completed using minimum resources, and extract knowledge from bioinformatics data. Introduction to Machine Learning is a comprehensive textbook on the subject, covering a broad array of topics not usually included in introductory machine learning texts. In order to present a unified treatment of machine learning problems and solutions, it discusses many methods from different fields, including statistics, pattern recognition, neural networks, artificial intelligence, signal processing, control, and data mining. All learning algorithms are explained so that the student can easily move from the equations in the book to a computer program. The text covers such topics as supervised learning, Bayesian decision theory, parametric methods, multivariate methods, multilayer perceptrons, local models, hidden Markov models, assessing and comparing classification algorithms, and reinforcement learning. New to the second edition are chapters on kernel machines, graphical models, and Bayesian estimation; expanded coverage of statistical tests in a chapter on design and analysis of machine learning experiments; case studies available on the Web (with downloadable results for instructors); and many additional exercises. All chapters have been revised and updated. Introduction to Machine Learning can be used by advanced undergraduates and graduate students who have completed courses in computer programming, probability, calculus, and linear algebra. It will also be of interest to engineers in the field who are concerned with the application of machine learning methods. Adaptive Computation and Machine Learning series</t>
+          <t>We design a novel, communication-efficient, failure-robust protocol for secure aggregation of high-dimensional data. Our protocol allows a server to compute the sum of large, user-held data vectors from mobile devices in a secure manner (i.e. without learning each user's individual contribution), and can be used, for example, in a federated learning setting, to aggregate user-provided model updates for a deep neural network. We prove the security of our protocol in the honest-but-curious and active adversary settings, and show that security is maintained even if an arbitrarily chosen subset of users drop out at any time. We evaluate the efficiency of our protocol and show, by complexity analysis and a concrete implementation, that its runtime and communication overhead remain low even on large data sets and client pools. For 16-bit input values, our protocol offers $1.73 x communication expansion for 210 users and 220-dimensional vectors, and 1.98 x expansion for 214 users and 224-dimensional vectors over sending data in the clear.</t>
         </is>
       </c>
       <c r="T81" t="inlineStr"/>
       <c r="U81" t="inlineStr"/>
       <c r="V81" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>1175</t>
         </is>
       </c>
       <c r="W81" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>1191</t>
         </is>
       </c>
       <c r="X81" t="inlineStr">
         <is>
-          <t>NA, 2019, Series in machine perception and artificial intelligence</t>
+          <t xml:space="preserve">Keith Bonawitz, 2017, </t>
         </is>
       </c>
       <c r="Y81" t="inlineStr">
         <is>
-          <t>NA, 2019, Series in machine perception and artificial intelligence</t>
+          <t xml:space="preserve">Keith Bonawitz, 2017, </t>
         </is>
       </c>
     </row>
@@ -8080,36 +8084,36 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>https://openalex.org/W3122548859</t>
+          <t>https://openalex.org/W2751318774</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1177/2053951715622512</t>
+          <t>https://doi.org/10.1142/9789811201967_0001</t>
         </is>
       </c>
       <c r="D82" t="inlineStr"/>
       <c r="E82" t="inlineStr">
         <is>
-          <t>How the machine ‘thinks’: Understanding opacity in machine learning algorithms</t>
+          <t>Introduction to Machine Learning</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>Big Data &amp; Society</t>
+          <t>Series in machine perception and artificial intelligence</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>Big Data &amp; Society</t>
+          <t>Series in machine perception and artificial intelligence</t>
         </is>
       </c>
       <c r="H82" t="n">
-        <v>2016</v>
+        <v>2019</v>
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>article</t>
+          <t>book-chapter</t>
         </is>
       </c>
       <c r="J82" t="inlineStr">
@@ -8118,56 +8122,44 @@
         </is>
       </c>
       <c r="K82" t="n">
-        <v>2508</v>
-      </c>
-      <c r="L82" t="inlineStr">
-        <is>
-          <t>Jenna Burrell</t>
-        </is>
-      </c>
+        <v>1659</v>
+      </c>
+      <c r="L82" t="inlineStr"/>
       <c r="M82" t="inlineStr"/>
-      <c r="N82" t="inlineStr">
-        <is>
-          <t>Jenna Burrell, School of Information, UC-Berkeley, Berkeley, CA, USA</t>
-        </is>
-      </c>
+      <c r="N82" t="inlineStr"/>
       <c r="O82" t="inlineStr"/>
-      <c r="P82" t="inlineStr">
-        <is>
-          <t>https://openalex.org/W202799293; https://openalex.org/W606820417; https://openalex.org/W1540016313; https://openalex.org/W1648303880; https://openalex.org/W1990060255; https://openalex.org/W2021362544; https://openalex.org/W2048315072; https://openalex.org/W2065240211; https://openalex.org/W2066384602; https://openalex.org/W2074057591; https://openalex.org/W2078620351; https://openalex.org/W2100960835; https://openalex.org/W2158604749; https://openalex.org/W2161336914; https://openalex.org/W2163284576; https://openalex.org/W2186089794; https://openalex.org/W2339183141; https://openalex.org/W2556704061; https://openalex.org/W2566747599; https://openalex.org/W2735886174; https://openalex.org/W2799929805; https://openalex.org/W2951240445; https://openalex.org/W3123374861; https://openalex.org/W3157172840; https://openalex.org/W4233093336; https://openalex.org/W4233551533; https://openalex.org/W4238428424; https://openalex.org/W4239941956; https://openalex.org/W4242887383; https://openalex.org/W4244021162; https://openalex.org/W4285719527</t>
-        </is>
-      </c>
+      <c r="P82" t="inlineStr"/>
       <c r="Q82" t="inlineStr">
         <is>
-          <t>Machine learning;Computer science;Artificial intelligence;Credit card fraud;Algorithm;Audit;Opacity;Credit card;Economics;World Wide Web</t>
+          <t>Computer science;Artificial intelligence</t>
         </is>
       </c>
       <c r="R82" t="inlineStr"/>
       <c r="S82" t="inlineStr">
         <is>
-          <t>This article considers the issue of opacity as a problem for socially consequential mechanisms of classification and ranking, such as spam filters, credit card fraud detection, search engines, news trends, market segmentation and advertising, insurance or loan qualification, and credit scoring. These mechanisms of classification all frequently rely on computational algorithms, and in many cases on machine learning algorithms to do this work. In this article, I draw a distinction between three forms of opacity: (1) opacity as intentional corporate or state secrecy, (2) opacity as technical illiteracy, and (3) an opacity that arises from the characteristics of machine learning algorithms and the scale required to apply them usefully. The analysis in this article gets inside the algorithms themselves. I cite existing literatures in computer science, known industry practices (as they are publicly presented), and do some testing and manipulation of code as a form of lightweight code audit. I argue that recognizing the distinct forms of opacity that may be coming into play in a given application is a key to determining which of a variety of technical and non-technical solutions could help to prevent harm.</t>
-        </is>
-      </c>
-      <c r="T82" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="U82" t="inlineStr">
+          <t>The goal of machine learning is to program computers to use example data or past experience to solve a given problem. Many successful applications of machine learning exist already, including systems that analyze past sales data to predict customer behavior, optimize robot behavior so that a task can be completed using minimum resources, and extract knowledge from bioinformatics data. Introduction to Machine Learning is a comprehensive textbook on the subject, covering a broad array of topics not usually included in introductory machine learning texts. In order to present a unified treatment of machine learning problems and solutions, it discusses many methods from different fields, including statistics, pattern recognition, neural networks, artificial intelligence, signal processing, control, and data mining. All learning algorithms are explained so that the student can easily move from the equations in the book to a computer program. The text covers such topics as supervised learning, Bayesian decision theory, parametric methods, multivariate methods, multilayer perceptrons, local models, hidden Markov models, assessing and comparing classification algorithms, and reinforcement learning. New to the second edition are chapters on kernel machines, graphical models, and Bayesian estimation; expanded coverage of statistical tests in a chapter on design and analysis of machine learning experiments; case studies available on the Web (with downloadable results for instructors); and many additional exercises. All chapters have been revised and updated. Introduction to Machine Learning can be used by advanced undergraduates and graduate students who have completed courses in computer programming, probability, calculus, and linear algebra. It will also be of interest to engineers in the field who are concerned with the application of machine learning methods. Adaptive Computation and Machine Learning series</t>
+        </is>
+      </c>
+      <c r="T82" t="inlineStr"/>
+      <c r="U82" t="inlineStr"/>
+      <c r="V82" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="V82" t="inlineStr"/>
-      <c r="W82" t="inlineStr"/>
+      <c r="W82" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
       <c r="X82" t="inlineStr">
         <is>
-          <t>Jenna Burrell, 2016, Big Data &amp; Society</t>
+          <t>NA, 2019, Series in machine perception and artificial intelligence</t>
         </is>
       </c>
       <c r="Y82" t="inlineStr">
         <is>
-          <t>Jenna Burrell, 2016, Big Data &amp; Society</t>
+          <t>NA, 2019, Series in machine perception and artificial intelligence</t>
         </is>
       </c>
     </row>
@@ -8217,7 +8209,7 @@
         </is>
       </c>
       <c r="K83" t="n">
-        <v>2052</v>
+        <v>2055</v>
       </c>
       <c r="L83" t="inlineStr">
         <is>
@@ -8282,32 +8274,32 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>https://openalex.org/W1993220166</t>
+          <t>https://openalex.org/W3122548859</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1145/1007730.1007735</t>
+          <t>https://doi.org/10.1177/2053951715622512</t>
         </is>
       </c>
       <c r="D84" t="inlineStr"/>
       <c r="E84" t="inlineStr">
         <is>
-          <t>A study of the behavior of several methods for balancing machine learning training data</t>
+          <t>How the machine ‘thinks’: Understanding opacity in machine learning algorithms</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>ACM SIGKDD Explorations Newsletter</t>
+          <t>Big Data &amp; Society</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>ACM SIGKDD Explorations Newsletter</t>
+          <t>Big Data &amp; Society</t>
         </is>
       </c>
       <c r="H84" t="n">
-        <v>2004</v>
+        <v>2016</v>
       </c>
       <c r="I84" t="inlineStr">
         <is>
@@ -8320,39 +8312,39 @@
         </is>
       </c>
       <c r="K84" t="n">
-        <v>4136</v>
+        <v>2521</v>
       </c>
       <c r="L84" t="inlineStr">
         <is>
-          <t>Gustavo E. A. P. A. Batista;Ronaldo C. Prati;Maria Carolina Monard</t>
+          <t>Jenna Burrell</t>
         </is>
       </c>
       <c r="M84" t="inlineStr"/>
       <c r="N84" t="inlineStr">
         <is>
-          <t>Gustavo E. A. P. A. Batista, Instituto de Ciências Matemáticas e de Computação, São Carlos - SP, Brazil;Ronaldo C. Prati, Instituto de Ciências Matemáticas e de Computação, São Carlos - SP, Brazil;Maria Carolina Monard, Instituto de Ciências Matemáticas e de Computação, São Carlos - SP, Brazil</t>
+          <t>Jenna Burrell, School of Information, UC-Berkeley, Berkeley, CA, USA</t>
         </is>
       </c>
       <c r="O84" t="inlineStr"/>
       <c r="P84" t="inlineStr">
         <is>
-          <t>https://openalex.org/W85350352; https://openalex.org/W102369970; https://openalex.org/W142793689; https://openalex.org/W1499467920; https://openalex.org/W1504694836; https://openalex.org/W1576442155; https://openalex.org/W1591261915; https://openalex.org/W1941659294; https://openalex.org/W1977245551; https://openalex.org/W1994410331; https://openalex.org/W2004131797; https://openalex.org/W2058732827; https://openalex.org/W2084812512; https://openalex.org/W2107686700; https://openalex.org/W2114968414; https://openalex.org/W2122496402; https://openalex.org/W2125055259; https://openalex.org/W2136903812; https://openalex.org/W2137029138; https://openalex.org/W2147169507; https://openalex.org/W2148143831; https://openalex.org/W2152761983; https://openalex.org/W2157092487; https://openalex.org/W2170913656; https://openalex.org/W2797114046; https://openalex.org/W4285719527</t>
+          <t>https://openalex.org/W202799293; https://openalex.org/W606820417; https://openalex.org/W1540016313; https://openalex.org/W1648303880; https://openalex.org/W1990060255; https://openalex.org/W2021362544; https://openalex.org/W2048315072; https://openalex.org/W2065240211; https://openalex.org/W2066384602; https://openalex.org/W2074057591; https://openalex.org/W2078620351; https://openalex.org/W2100960835; https://openalex.org/W2158604749; https://openalex.org/W2161336914; https://openalex.org/W2163284576; https://openalex.org/W2186089794; https://openalex.org/W2339183141; https://openalex.org/W2556704061; https://openalex.org/W2566747599; https://openalex.org/W2735886174; https://openalex.org/W2799929805; https://openalex.org/W2951240445; https://openalex.org/W3123374861; https://openalex.org/W3157172840; https://openalex.org/W4233093336; https://openalex.org/W4233551533; https://openalex.org/W4238428424; https://openalex.org/W4239941956; https://openalex.org/W4242887383; https://openalex.org/W4244021162; https://openalex.org/W4285719527</t>
         </is>
       </c>
       <c r="Q84" t="inlineStr">
         <is>
-          <t>Computer science;Class (philosophy);Machine learning;Artificial intelligence;Sampling (signal processing);Simple random sample;Event (particle physics);Data mining;Simple (philosophy)</t>
+          <t>Machine learning;Computer science;Artificial intelligence;Credit card fraud;Algorithm;Audit;Opacity;Credit card;Economics;World Wide Web</t>
         </is>
       </c>
       <c r="R84" t="inlineStr"/>
       <c r="S84" t="inlineStr">
         <is>
-          <t>There are several aspects that might influence the performance achieved by existing learning systems. It has been reported that one of these aspects is related to class imbalance in which examples in training data belonging to one class heavily outnumber the examples in the other class. In this situation, which is found in real world data describing an infrequent but important event, the learning system may have difficulties to learn the concept related to the minority class. In this work we perform a broad experimental evaluation involving ten methods, three of them proposed by the authors, to deal with the class imbalance problem in thirteen UCI data sets. Our experiments provide evidence that class imbalance does not systematically hinder the performance of learning systems. In fact, the problem seems to be related to learning with too few minority class examples in the presence of other complicating factors, such as class overlapping. Two of our proposed methods deal with these conditions directly, allying a known over-sampling method with data cleaning methods in order to produce better-defined class clusters. Our comparative experiments show that, in general, over-sampling methods provide more accurate results than under-sampling methods considering the area under the ROC curve (AUC). This result seems to contradict results previously published in the literature. Two of our proposed methods, Smote + Tomek and Smote + ENN, presented very good results for data sets with a small number of positive examples. Moreover, Random over-sampling, a very simple over-sampling method, is very competitive to more complex over-sampling methods. Since the over-sampling methods provided very good performance results, we also measured the syntactic complexity of the decision trees induced from over-sampled data. Our results show that these trees are usually more complex then the ones induced from original data. Random over-sampling usually produced the smallest increase in the mean number of induced rules and Smote + ENN the smallest increase in the mean number of conditions per rule, when compared among the investigated over-sampling methods.</t>
+          <t>This article considers the issue of opacity as a problem for socially consequential mechanisms of classification and ranking, such as spam filters, credit card fraud detection, search engines, news trends, market segmentation and advertising, insurance or loan qualification, and credit scoring. These mechanisms of classification all frequently rely on computational algorithms, and in many cases on machine learning algorithms to do this work. In this article, I draw a distinction between three forms of opacity: (1) opacity as intentional corporate or state secrecy, (2) opacity as technical illiteracy, and (3) an opacity that arises from the characteristics of machine learning algorithms and the scale required to apply them usefully. The analysis in this article gets inside the algorithms themselves. I cite existing literatures in computer science, known industry practices (as they are publicly presented), and do some testing and manipulation of code as a form of lightweight code audit. I argue that recognizing the distinct forms of opacity that may be coming into play in a given application is a key to determining which of a variety of technical and non-technical solutions could help to prevent harm.</t>
         </is>
       </c>
       <c r="T84" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>3</t>
         </is>
       </c>
       <c r="U84" t="inlineStr">
@@ -8360,24 +8352,16 @@
           <t>1</t>
         </is>
       </c>
-      <c r="V84" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="W84" t="inlineStr">
-        <is>
-          <t>29</t>
-        </is>
-      </c>
+      <c r="V84" t="inlineStr"/>
+      <c r="W84" t="inlineStr"/>
       <c r="X84" t="inlineStr">
         <is>
-          <t>Gustavo E. A. P. A. Batista, 2004, ACM SIGKDD Explorations Newsletter</t>
+          <t>Jenna Burrell, 2016, Big Data &amp; Society</t>
         </is>
       </c>
       <c r="Y84" t="inlineStr">
         <is>
-          <t>Gustavo E. A. P. A. Batista, 2004, ACM SIGKDD Explorations Newsletter</t>
+          <t>Jenna Burrell, 2016, Big Data &amp; Society</t>
         </is>
       </c>
     </row>
@@ -8389,28 +8373,36 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>https://openalex.org/W2767079719</t>
+          <t>https://openalex.org/W3145506661</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1145/3133956.3133982</t>
+          <t>https://doi.org/10.1007/978-3-030-10546-4_1</t>
         </is>
       </c>
       <c r="D85" t="inlineStr"/>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Practical Secure Aggregation for Privacy-Preserving Machine Learning</t>
-        </is>
-      </c>
-      <c r="F85" t="inlineStr"/>
-      <c r="G85" t="inlineStr"/>
+          <t>Introduction to Machine Learning</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>Springer briefs in electrical and computer engineering</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>Springer briefs in electrical and computer engineering</t>
+        </is>
+      </c>
       <c r="H85" t="n">
-        <v>2017</v>
+        <v>2019</v>
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>article</t>
+          <t>book-chapter</t>
         </is>
       </c>
       <c r="J85" t="inlineStr">
@@ -8419,56 +8411,52 @@
         </is>
       </c>
       <c r="K85" t="n">
-        <v>3455</v>
+        <v>1620</v>
       </c>
       <c r="L85" t="inlineStr">
         <is>
-          <t>Keith Bonawitz;Vladimir Ivanov;Ben Kreuter;Antonio Marcedone;H. Brendan McMahan;Sarvar Patel;Daniel Ramage;Aaron Segal;Karn Seth</t>
+          <t>F. Richard Yu;Ying He</t>
         </is>
       </c>
       <c r="M85" t="inlineStr"/>
       <c r="N85" t="inlineStr">
         <is>
-          <t>Keith Bonawitz, Google Inc., Mountain View, CA, USA;Vladimir Ivanov, Google Inc., Mountain View, CA, USA;Ben Kreuter, Google Inc., Mountain View, CA, USA;Antonio Marcedone, Cornell Tech &amp;amp;Google Inc., New York, NY, USA;H. Brendan McMahan, Google Inc., Mountain View, CA, USA;Sarvar Patel, Google Inc., Mountain View, CA, USA;Daniel Ramage, Google Inc., Mountain View, CA, USA;Aaron Segal, Google Inc., Mountain View, CA, USA;Karn Seth, Google Inc., Mountain View, CA, USA</t>
+          <t>F. Richard Yu, Carleton University, Ottawa, ON, Canada;Ying He, Carleton University, Ottawa, ON, Canada</t>
         </is>
       </c>
       <c r="O85" t="inlineStr"/>
       <c r="P85" t="inlineStr">
         <is>
-          <t>https://openalex.org/W25045116; https://openalex.org/W95608104; https://openalex.org/W1071368427; https://openalex.org/W1493407996; https://openalex.org/W1519947574; https://openalex.org/W1557833142; https://openalex.org/W1595357546; https://openalex.org/W1656028867; https://openalex.org/W1836711297; https://openalex.org/W1952161176; https://openalex.org/W1952958290; https://openalex.org/W1981029888; https://openalex.org/W2006453614; https://openalex.org/W2027471022; https://openalex.org/W2027595342; https://openalex.org/W2033974828; https://openalex.org/W2051267297; https://openalex.org/W2053637704; https://openalex.org/W2053801139; https://openalex.org/W2058648304; https://openalex.org/W2061106457; https://openalex.org/W2069657084; https://openalex.org/W2087811006; https://openalex.org/W2104803737; https://openalex.org/W2128865076; https://openalex.org/W2135930857; https://openalex.org/W2141420453; https://openalex.org/W2146673169; https://openalex.org/W2149093588; https://openalex.org/W2152768255; https://openalex.org/W2156186849; https://openalex.org/W2163481970; https://openalex.org/W2164284862; https://openalex.org/W2200869402; https://openalex.org/W2232997092; https://openalex.org/W2267098117; https://openalex.org/W2295522738; https://openalex.org/W2336650964; https://openalex.org/W2400777838; https://openalex.org/W2402235285; https://openalex.org/W2413533038; https://openalex.org/W2473418344; https://openalex.org/W2525846285; https://openalex.org/W2535690855; https://openalex.org/W2536058570; https://openalex.org/W2538520193; https://openalex.org/W2541884796; https://openalex.org/W2557283755; https://openalex.org/W2568821124; https://openalex.org/W2599930814; https://openalex.org/W2911978475; https://openalex.org/W2951114885; https://openalex.org/W3031847131; https://openalex.org/W3102407811; https://openalex.org/W3141405531; https://openalex.org/W3150645827</t>
+          <t>https://openalex.org/W79158146; https://openalex.org/W332743987; https://openalex.org/W1480376833; https://openalex.org/W1571801203; https://openalex.org/W1615454278; https://openalex.org/W1698155719; https://openalex.org/W1755360231; https://openalex.org/W1817561967; https://openalex.org/W1873332500; https://openalex.org/W1967903496; https://openalex.org/W1970653610; https://openalex.org/W1983320747; https://openalex.org/W1983405239; https://openalex.org/W1989241020; https://openalex.org/W2002011878; https://openalex.org/W2027645392; https://openalex.org/W2033213616; https://openalex.org/W2036950464; https://openalex.org/W2040678502; https://openalex.org/W2045377245; https://openalex.org/W2046079134; https://openalex.org/W2064675550; https://openalex.org/W2076063813; https://openalex.org/W2105993120; https://openalex.org/W2119615570; https://openalex.org/W2122111042; https://openalex.org/W2124776405; https://openalex.org/W2125838338; https://openalex.org/W2140190241; https://openalex.org/W2148603752; https://openalex.org/W2149520764; https://openalex.org/W2149706766; https://openalex.org/W2156273867; https://openalex.org/W2161160262; https://openalex.org/W2163605009; https://openalex.org/W2171265988; https://openalex.org/W2171928131; https://openalex.org/W2293634267; https://openalex.org/W2523431972; https://openalex.org/W2755588949; https://openalex.org/W2763049519; https://openalex.org/W2768975974; https://openalex.org/W2783146946; https://openalex.org/W2911964244; https://openalex.org/W2919115771; https://openalex.org/W3085162807; https://openalex.org/W4210979681; https://openalex.org/W4234721591; https://openalex.org/W4391374765; https://openalex.org/W6603212874; https://openalex.org/W6636455871; https://openalex.org/W6680140577; https://openalex.org/W6817491142</t>
         </is>
       </c>
       <c r="Q85" t="inlineStr">
         <is>
-          <t>Computer science;Overhead (engineering);Protocol (science);Universal composability;Adversary;Computer network;Aggregate (composite);Cryptographic protocol;Distributed computing;Theoretical computer science;Cryptography;Computer security;Operating system</t>
+          <t>Computer science;Artificial intelligence</t>
         </is>
       </c>
       <c r="R85" t="inlineStr"/>
-      <c r="S85" t="inlineStr">
-        <is>
-          <t>We design a novel, communication-efficient, failure-robust protocol for secure aggregation of high-dimensional data. Our protocol allows a server to compute the sum of large, user-held data vectors from mobile devices in a secure manner (i.e. without learning each user's individual contribution), and can be used, for example, in a federated learning setting, to aggregate user-provided model updates for a deep neural network. We prove the security of our protocol in the honest-but-curious and active adversary settings, and show that security is maintained even if an arbitrarily chosen subset of users drop out at any time. We evaluate the efficiency of our protocol and show, by complexity analysis and a concrete implementation, that its runtime and communication overhead remain low even on large data sets and client pools. For 16-bit input values, our protocol offers $1.73 x communication expansion for 210 users and 220-dimensional vectors, and 1.98 x expansion for 214 users and 224-dimensional vectors over sending data in the clear.</t>
-        </is>
-      </c>
+      <c r="S85" t="inlineStr"/>
       <c r="T85" t="inlineStr"/>
       <c r="U85" t="inlineStr"/>
       <c r="V85" t="inlineStr">
         <is>
-          <t>1175</t>
+          <t>1</t>
         </is>
       </c>
       <c r="W85" t="inlineStr">
         <is>
-          <t>1191</t>
+          <t>13</t>
         </is>
       </c>
       <c r="X85" t="inlineStr">
         <is>
-          <t xml:space="preserve">Keith Bonawitz, 2017, </t>
+          <t>F. Richard Yu, 2019, Springer briefs in electrical and computer engineering</t>
         </is>
       </c>
       <c r="Y85" t="inlineStr">
         <is>
-          <t xml:space="preserve">Keith Bonawitz, 2017, </t>
+          <t>F. Richard Yu, 2019, Springer briefs in electrical and computer engineering</t>
         </is>
       </c>
     </row>
@@ -8480,32 +8468,32 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>https://openalex.org/W4205539948</t>
+          <t>https://openalex.org/W1993220166</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1093/rfs/hhaa009</t>
+          <t>https://doi.org/10.1145/1007730.1007735</t>
         </is>
       </c>
       <c r="D86" t="inlineStr"/>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Empirical Asset Pricing via Machine Learning</t>
+          <t>A study of the behavior of several methods for balancing machine learning training data</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>Review of Financial Studies</t>
+          <t>ACM SIGKDD Explorations Newsletter</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>Review of Financial Studies</t>
+          <t>ACM SIGKDD Explorations Newsletter</t>
         </is>
       </c>
       <c r="H86" t="n">
-        <v>2020</v>
+        <v>2004</v>
       </c>
       <c r="I86" t="inlineStr">
         <is>
@@ -8518,64 +8506,64 @@
         </is>
       </c>
       <c r="K86" t="n">
-        <v>2241</v>
+        <v>4143</v>
       </c>
       <c r="L86" t="inlineStr">
         <is>
-          <t>Shihao Gu;Bryan Kelly;Dacheng Xiu</t>
+          <t>Gustavo E. A. P. A. Batista;Ronaldo C. Prati;Maria Carolina Monard</t>
         </is>
       </c>
       <c r="M86" t="inlineStr"/>
       <c r="N86" t="inlineStr">
         <is>
-          <t>Shihao Gu, Booth School of Business, University of Chicago;Bryan Kelly, Yale University, AQR Capital Management, and NBER;Dacheng Xiu, Booth School of Business, University of Chicago</t>
+          <t>Gustavo E. A. P. A. Batista, Instituto de Ciências Matemáticas e de Computação, São Carlos - SP, Brazil;Ronaldo C. Prati, Instituto de Ciências Matemáticas e de Computação, São Carlos - SP, Brazil;Maria Carolina Monard, Instituto de Ciências Matemáticas e de Computação, São Carlos - SP, Brazil</t>
         </is>
       </c>
       <c r="O86" t="inlineStr"/>
       <c r="P86" t="inlineStr">
         <is>
-          <t>https://openalex.org/W608042232; https://openalex.org/W1503022246; https://openalex.org/W1522301498; https://openalex.org/W1533618852; https://openalex.org/W1534477342; https://openalex.org/W1594031697; https://openalex.org/W1678356000; https://openalex.org/W1789808336; https://openalex.org/W1969404656; https://openalex.org/W1971217947; https://openalex.org/W1976251851; https://openalex.org/W1995834279; https://openalex.org/W2007694684; https://openalex.org/W2024046085; https://openalex.org/W2046033161; https://openalex.org/W2048662624; https://openalex.org/W2063730763; https://openalex.org/W2070534370; https://openalex.org/W2103496339; https://openalex.org/W2135293965; https://openalex.org/W2136922672; https://openalex.org/W2137983211; https://openalex.org/W2139753118; https://openalex.org/W2144570112; https://openalex.org/W2154987621; https://openalex.org/W2194775991; https://openalex.org/W2265274622; https://openalex.org/W2291108100; https://openalex.org/W2319405822; https://openalex.org/W2338469198; https://openalex.org/W2503100348; https://openalex.org/W2546302380; https://openalex.org/W2560674852; https://openalex.org/W2741371467; https://openalex.org/W2787894218; https://openalex.org/W2799643291; https://openalex.org/W2911964244; https://openalex.org/W2938815980; https://openalex.org/W2967005703; https://openalex.org/W3001826040; https://openalex.org/W3004050393; https://openalex.org/W3004732066; https://openalex.org/W3018089439; https://openalex.org/W3121274430; https://openalex.org/W3121588992; https://openalex.org/W3122020290; https://openalex.org/W3122118888; https://openalex.org/W3123267500; https://openalex.org/W3123752263; https://openalex.org/W3124436545; https://openalex.org/W3125696988; https://openalex.org/W3125950889; https://openalex.org/W3126032681; https://openalex.org/W3126136988; https://openalex.org/W3131102529; https://openalex.org/W4211170237; https://openalex.org/W4237239309; https://openalex.org/W4242067316; https://openalex.org/W4297853882; https://openalex.org/W4388297464; https://openalex.org/W6637242042; https://openalex.org/W6637404493; https://openalex.org/W6638667902; https://openalex.org/W6660794422; https://openalex.org/W6682889407; https://openalex.org/W6684409620; https://openalex.org/W6691187937; https://openalex.org/W6694527737; https://openalex.org/W6736719330; https://openalex.org/W6781003217</t>
+          <t>https://openalex.org/W85350352; https://openalex.org/W102369970; https://openalex.org/W142793689; https://openalex.org/W1499467920; https://openalex.org/W1504694836; https://openalex.org/W1576442155; https://openalex.org/W1591261915; https://openalex.org/W1941659294; https://openalex.org/W1977245551; https://openalex.org/W1994410331; https://openalex.org/W2004131797; https://openalex.org/W2058732827; https://openalex.org/W2084812512; https://openalex.org/W2107686700; https://openalex.org/W2114968414; https://openalex.org/W2122496402; https://openalex.org/W2125055259; https://openalex.org/W2136903812; https://openalex.org/W2137029138; https://openalex.org/W2147169507; https://openalex.org/W2148143831; https://openalex.org/W2152761983; https://openalex.org/W2157092487; https://openalex.org/W2170913656; https://openalex.org/W2797114046; https://openalex.org/W4285719527</t>
         </is>
       </c>
       <c r="Q86" t="inlineStr">
         <is>
-          <t>Capital asset pricing model;Machine learning;Computer science;Artificial intelligence;Artificial neural network;Volatility (finance);Market liquidity;Econometrics;Asset (computer security);TRACE (psycholinguistics);Set (abstract data type);Economics;Finance</t>
+          <t>Computer science;Class (philosophy);Machine learning;Artificial intelligence;Sampling (signal processing);Simple random sample;Event (particle physics);Data mining;Simple (philosophy)</t>
         </is>
       </c>
       <c r="R86" t="inlineStr"/>
       <c r="S86" t="inlineStr">
         <is>
-          <t>Abstract We perform a comparative analysis of machine learning methods for the canonical problem of empirical asset pricing: measuring asset risk premiums. We demonstrate large economic gains to investors using machine learning forecasts, in some cases doubling the performance of leading regression-based strategies from the literature. We identify the best-performing methods (trees and neural networks) and trace their predictive gains to allowing nonlinear predictor interactions missed by other methods. All methods agree on the same set of dominant predictive signals, a set that includes variations on momentum, liquidity, and volatility. Authors have furnished an Internet Appendix, which is available on the Oxford University Press Web site next to the link to the final published paper online.</t>
+          <t>There are several aspects that might influence the performance achieved by existing learning systems. It has been reported that one of these aspects is related to class imbalance in which examples in training data belonging to one class heavily outnumber the examples in the other class. In this situation, which is found in real world data describing an infrequent but important event, the learning system may have difficulties to learn the concept related to the minority class. In this work we perform a broad experimental evaluation involving ten methods, three of them proposed by the authors, to deal with the class imbalance problem in thirteen UCI data sets. Our experiments provide evidence that class imbalance does not systematically hinder the performance of learning systems. In fact, the problem seems to be related to learning with too few minority class examples in the presence of other complicating factors, such as class overlapping. Two of our proposed methods deal with these conditions directly, allying a known over-sampling method with data cleaning methods in order to produce better-defined class clusters. Our comparative experiments show that, in general, over-sampling methods provide more accurate results than under-sampling methods considering the area under the ROC curve (AUC). This result seems to contradict results previously published in the literature. Two of our proposed methods, Smote + Tomek and Smote + ENN, presented very good results for data sets with a small number of positive examples. Moreover, Random over-sampling, a very simple over-sampling method, is very competitive to more complex over-sampling methods. Since the over-sampling methods provided very good performance results, we also measured the syntactic complexity of the decision trees induced from over-sampled data. Our results show that these trees are usually more complex then the ones induced from original data. Random over-sampling usually produced the smallest increase in the mean number of induced rules and Smote + ENN the smallest increase in the mean number of conditions per rule, when compared among the investigated over-sampling methods.</t>
         </is>
       </c>
       <c r="T86" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>6</t>
         </is>
       </c>
       <c r="U86" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="V86" t="inlineStr">
         <is>
-          <t>2223</t>
+          <t>20</t>
         </is>
       </c>
       <c r="W86" t="inlineStr">
         <is>
-          <t>2273</t>
+          <t>29</t>
         </is>
       </c>
       <c r="X86" t="inlineStr">
         <is>
-          <t>Shihao Gu, 2020, Review of Financial Studies</t>
+          <t>Gustavo E. A. P. A. Batista, 2004, ACM SIGKDD Explorations Newsletter</t>
         </is>
       </c>
       <c r="Y86" t="inlineStr">
         <is>
-          <t>Shihao Gu, 2020, Review of Financial Studies</t>
+          <t>Gustavo E. A. P. A. Batista, 2004, ACM SIGKDD Explorations Newsletter</t>
         </is>
       </c>
     </row>
@@ -8654,36 +8642,36 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>https://openalex.org/W3145506661</t>
+          <t>https://openalex.org/W4205539948</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1007/978-3-030-10546-4_1</t>
+          <t>https://doi.org/10.1093/rfs/hhaa009</t>
         </is>
       </c>
       <c r="D88" t="inlineStr"/>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Introduction to Machine Learning</t>
+          <t>Empirical Asset Pricing via Machine Learning</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>Springer briefs in electrical and computer engineering</t>
+          <t>Review of Financial Studies</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>Springer briefs in electrical and computer engineering</t>
+          <t>Review of Financial Studies</t>
         </is>
       </c>
       <c r="H88" t="n">
-        <v>2019</v>
+        <v>2020</v>
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>book-chapter</t>
+          <t>article</t>
         </is>
       </c>
       <c r="J88" t="inlineStr">
@@ -8692,52 +8680,64 @@
         </is>
       </c>
       <c r="K88" t="n">
-        <v>1620</v>
+        <v>2254</v>
       </c>
       <c r="L88" t="inlineStr">
         <is>
-          <t>F. Richard Yu;Ying He</t>
+          <t>Shihao Gu;Bryan Kelly;Dacheng Xiu</t>
         </is>
       </c>
       <c r="M88" t="inlineStr"/>
       <c r="N88" t="inlineStr">
         <is>
-          <t>F. Richard Yu, Carleton University, Ottawa, ON, Canada;Ying He, Carleton University, Ottawa, ON, Canada</t>
+          <t>Shihao Gu, Booth School of Business, University of Chicago;Bryan Kelly, Yale University, AQR Capital Management, and NBER;Dacheng Xiu, Booth School of Business, University of Chicago</t>
         </is>
       </c>
       <c r="O88" t="inlineStr"/>
       <c r="P88" t="inlineStr">
         <is>
-          <t>https://openalex.org/W79158146; https://openalex.org/W332743987; https://openalex.org/W1480376833; https://openalex.org/W1571801203; https://openalex.org/W1615454278; https://openalex.org/W1698155719; https://openalex.org/W1755360231; https://openalex.org/W1817561967; https://openalex.org/W1873332500; https://openalex.org/W1967903496; https://openalex.org/W1970653610; https://openalex.org/W1983320747; https://openalex.org/W1983405239; https://openalex.org/W1989241020; https://openalex.org/W2002011878; https://openalex.org/W2027645392; https://openalex.org/W2033213616; https://openalex.org/W2036950464; https://openalex.org/W2040678502; https://openalex.org/W2045377245; https://openalex.org/W2046079134; https://openalex.org/W2064675550; https://openalex.org/W2076063813; https://openalex.org/W2105993120; https://openalex.org/W2119615570; https://openalex.org/W2122111042; https://openalex.org/W2124776405; https://openalex.org/W2125838338; https://openalex.org/W2140190241; https://openalex.org/W2148603752; https://openalex.org/W2149520764; https://openalex.org/W2149706766; https://openalex.org/W2156273867; https://openalex.org/W2161160262; https://openalex.org/W2163605009; https://openalex.org/W2171265988; https://openalex.org/W2171928131; https://openalex.org/W2293634267; https://openalex.org/W2523431972; https://openalex.org/W2755588949; https://openalex.org/W2763049519; https://openalex.org/W2768975974; https://openalex.org/W2783146946; https://openalex.org/W2911964244; https://openalex.org/W2919115771; https://openalex.org/W3085162807; https://openalex.org/W4210979681; https://openalex.org/W4234721591; https://openalex.org/W4391374765; https://openalex.org/W6603212874; https://openalex.org/W6636455871; https://openalex.org/W6680140577; https://openalex.org/W6817491142</t>
+          <t>https://openalex.org/W608042232; https://openalex.org/W1503022246; https://openalex.org/W1522301498; https://openalex.org/W1533618852; https://openalex.org/W1534477342; https://openalex.org/W1594031697; https://openalex.org/W1678356000; https://openalex.org/W1789808336; https://openalex.org/W1969404656; https://openalex.org/W1971217947; https://openalex.org/W1976251851; https://openalex.org/W1995834279; https://openalex.org/W2007694684; https://openalex.org/W2024046085; https://openalex.org/W2046033161; https://openalex.org/W2048662624; https://openalex.org/W2063730763; https://openalex.org/W2070534370; https://openalex.org/W2103496339; https://openalex.org/W2135293965; https://openalex.org/W2136922672; https://openalex.org/W2137983211; https://openalex.org/W2139753118; https://openalex.org/W2144570112; https://openalex.org/W2154987621; https://openalex.org/W2194775991; https://openalex.org/W2265274622; https://openalex.org/W2291108100; https://openalex.org/W2319405822; https://openalex.org/W2338469198; https://openalex.org/W2503100348; https://openalex.org/W2546302380; https://openalex.org/W2560674852; https://openalex.org/W2741371467; https://openalex.org/W2787894218; https://openalex.org/W2799643291; https://openalex.org/W2911964244; https://openalex.org/W2938815980; https://openalex.org/W2967005703; https://openalex.org/W3001826040; https://openalex.org/W3004050393; https://openalex.org/W3004732066; https://openalex.org/W3018089439; https://openalex.org/W3121274430; https://openalex.org/W3121588992; https://openalex.org/W3122020290; https://openalex.org/W3122118888; https://openalex.org/W3123267500; https://openalex.org/W3123752263; https://openalex.org/W3124436545; https://openalex.org/W3125696988; https://openalex.org/W3125950889; https://openalex.org/W3126032681; https://openalex.org/W3126136988; https://openalex.org/W3131102529; https://openalex.org/W4211170237; https://openalex.org/W4237239309; https://openalex.org/W4242067316; https://openalex.org/W4297853882; https://openalex.org/W4388297464; https://openalex.org/W6637242042; https://openalex.org/W6637404493; https://openalex.org/W6638667902; https://openalex.org/W6660794422; https://openalex.org/W6682889407; https://openalex.org/W6684409620; https://openalex.org/W6691187937; https://openalex.org/W6694527737; https://openalex.org/W6736719330; https://openalex.org/W6781003217</t>
         </is>
       </c>
       <c r="Q88" t="inlineStr">
         <is>
-          <t>Computer science;Artificial intelligence</t>
+          <t>Capital asset pricing model;Machine learning;Computer science;Artificial intelligence;Artificial neural network;Volatility (finance);Market liquidity;Econometrics;Asset (computer security);TRACE (psycholinguistics);Set (abstract data type);Economics;Finance</t>
         </is>
       </c>
       <c r="R88" t="inlineStr"/>
-      <c r="S88" t="inlineStr"/>
-      <c r="T88" t="inlineStr"/>
-      <c r="U88" t="inlineStr"/>
+      <c r="S88" t="inlineStr">
+        <is>
+          <t>Abstract We perform a comparative analysis of machine learning methods for the canonical problem of empirical asset pricing: measuring asset risk premiums. We demonstrate large economic gains to investors using machine learning forecasts, in some cases doubling the performance of leading regression-based strategies from the literature. We identify the best-performing methods (trees and neural networks) and trace their predictive gains to allowing nonlinear predictor interactions missed by other methods. All methods agree on the same set of dominant predictive signals, a set that includes variations on momentum, liquidity, and volatility. Authors have furnished an Internet Appendix, which is available on the Oxford University Press Web site next to the link to the final published paper online.</t>
+        </is>
+      </c>
+      <c r="T88" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="U88" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
       <c r="V88" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2223</t>
         </is>
       </c>
       <c r="W88" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>2273</t>
         </is>
       </c>
       <c r="X88" t="inlineStr">
         <is>
-          <t>F. Richard Yu, 2019, Springer briefs in electrical and computer engineering</t>
+          <t>Shihao Gu, 2020, Review of Financial Studies</t>
         </is>
       </c>
       <c r="Y88" t="inlineStr">
         <is>
-          <t>F. Richard Yu, 2019, Springer briefs in electrical and computer engineering</t>
+          <t>Shihao Gu, 2020, Review of Financial Studies</t>
         </is>
       </c>
     </row>
@@ -8953,7 +8953,7 @@
         </is>
       </c>
       <c r="K91" t="n">
-        <v>1891</v>
+        <v>1893</v>
       </c>
       <c r="L91" t="inlineStr">
         <is>
@@ -9060,7 +9060,7 @@
         </is>
       </c>
       <c r="K92" t="n">
-        <v>1987</v>
+        <v>1989</v>
       </c>
       <c r="L92" t="inlineStr">
         <is>
@@ -9163,7 +9163,7 @@
         </is>
       </c>
       <c r="K93" t="n">
-        <v>2708</v>
+        <v>2715</v>
       </c>
       <c r="L93" t="inlineStr">
         <is>
@@ -9224,36 +9224,36 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>https://openalex.org/W2919115771</t>
+          <t>https://openalex.org/W2791315675</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1038/nature14539</t>
+          <t>https://doi.org/10.1016/j.neucom.2017.11.077</t>
         </is>
       </c>
       <c r="D94" t="inlineStr"/>
       <c r="E94" t="inlineStr">
         <is>
-          <t>Deep learning</t>
+          <t>Feature selection in machine learning: A new perspective</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>Nature</t>
+          <t>Neurocomputing</t>
         </is>
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>Nature</t>
+          <t>Neurocomputing</t>
         </is>
       </c>
       <c r="H94" t="n">
-        <v>2015</v>
+        <v>2018</v>
       </c>
       <c r="I94" t="inlineStr">
         <is>
-          <t>review</t>
+          <t>article</t>
         </is>
       </c>
       <c r="J94" t="inlineStr">
@@ -9262,60 +9262,56 @@
         </is>
       </c>
       <c r="K94" t="n">
-        <v>81801</v>
+        <v>2059</v>
       </c>
       <c r="L94" t="inlineStr">
         <is>
-          <t>Yann LeCun;Yoshua Bengio;Geoffrey E. Hinton</t>
+          <t>Jie Cai;Jiawei Luo;Shulin Wang;Sheng Yang</t>
         </is>
       </c>
       <c r="M94" t="inlineStr"/>
       <c r="N94" t="inlineStr">
         <is>
-          <t>Yann LeCun, 1] Facebook AI Research, 770 Broadway, New York, New York 10003 USA. [2] New York University, 715 Broadway, New York, New York 10003, USA;Yann LeCun, Facebook AI Research, 770 Broadway, New York, 10003, New York, USA;Yann LeCun, New York University, 715 Broadway, New York, 10003, New York, USA;Yoshua Bengio, Department of Computer Science and Operations Research Université de Montréal, Pavillon André-Aisenstadt, PO Box 6128 Centre-Ville STN Montréal, Quebec H3C 3J7, Canada;Yoshua Bengio, Department of Computer Science and Operations Research Université de Montréal, Pavillon André-Aisenstadt, PO Box 6128 Centre-Ville STN, Montréal, H3C 3J7, Quebec, Canada;Geoffrey E. Hinton, 1] Google, 1600 Amphitheatre Parkway, Mountain View, California 94043, USA. [2] Department of Computer Science, University of Toronto, 6 King's College Road, Toronto, Ontario M5S 3G4, Canada;Geoffrey E. Hinton, Google, 1600 Amphitheatre Parkway, Mountain View, 94043, California, USA;Geoffrey E. Hinton, Department of Computer Science, University of Toronto, 6 King's College Road, Toronto, M5S 3G4, Ontario, Canada</t>
+          <t>Jie Cai, College of Computer Science and Electronic Engineering, Hunan University, Changsha, Hunan, China;Jiawei Luo, College of Computer Science and Electronic Engineering, Hunan University, Changsha, Hunan, China;Shulin Wang, College of Computer Science and Electronic Engineering, Hunan University, Changsha, Hunan, China;Sheng Yang, College of Computer Science and Electronic Engineering, Hunan University, Changsha, Hunan, China</t>
         </is>
       </c>
       <c r="O94" t="inlineStr"/>
       <c r="P94" t="inlineStr">
         <is>
-          <t>https://openalex.org/W146900863; https://openalex.org/W170811313; https://openalex.org/W1487583988; https://openalex.org/W1498436455; https://openalex.org/W1514535095; https://openalex.org/W1573503290; https://openalex.org/W1752712236; https://openalex.org/W1970689298; https://openalex.org/W1978592082; https://openalex.org/W1993845689; https://openalex.org/W1993882792; https://openalex.org/W1999497791; https://openalex.org/W1999798000; https://openalex.org/W2022508996; https://openalex.org/W2025768430; https://openalex.org/W2064675550; https://openalex.org/W2072128103; https://openalex.org/W2074551195; https://openalex.org/W2085989895; https://openalex.org/W2088338354; https://openalex.org/W2091987367; https://openalex.org/W2095739681; https://openalex.org/W2098580305; https://openalex.org/W2100495367; https://openalex.org/W2107878631; https://openalex.org/W2108069432; https://openalex.org/W2111304802; https://openalex.org/W2112796928; https://openalex.org/W2116360511; https://openalex.org/W2117671523; https://openalex.org/W2120284346; https://openalex.org/W2120432001; https://openalex.org/W2121289914; https://openalex.org/W2136922672; https://openalex.org/W2144015117; https://openalex.org/W2144354855; https://openalex.org/W2145339207; https://openalex.org/W2146989110; https://openalex.org/W2157331557; https://openalex.org/W2158778629; https://openalex.org/W2160815625; https://openalex.org/W2163922914; https://openalex.org/W2166206801; https://openalex.org/W2169488311; https://openalex.org/W2169805405; https://openalex.org/W2800394774; https://openalex.org/W3139812727; https://openalex.org/W4232280717; https://openalex.org/W4249882522; https://openalex.org/W6630820455; https://openalex.org/W6674914833; https://openalex.org/W6683738474; https://openalex.org/W6743198006</t>
+          <t>https://openalex.org/W62404953; https://openalex.org/W110173923; https://openalex.org/W129457532; https://openalex.org/W137065004; https://openalex.org/W140777655; https://openalex.org/W146732357; https://openalex.org/W175909076; https://openalex.org/W204835077; https://openalex.org/W323404752; https://openalex.org/W1253096047; https://openalex.org/W1480716458; https://openalex.org/W1541321639; https://openalex.org/W1543715688; https://openalex.org/W1546113605; https://openalex.org/W1554275123; https://openalex.org/W1554663460; https://openalex.org/W1555244713; https://openalex.org/W1560107318; https://openalex.org/W1570713908; https://openalex.org/W1581426664; https://openalex.org/W1583700199; https://openalex.org/W1583837637; https://openalex.org/W1585743408; https://openalex.org/W1590246454; https://openalex.org/W1608549042; https://openalex.org/W1761159547; https://openalex.org/W1804170020; https://openalex.org/W1808644423; https://openalex.org/W1887132526; https://openalex.org/W1898334332; https://openalex.org/W1949281989; https://openalex.org/W1958291604; https://openalex.org/W1964042173; https://openalex.org/W1964137961; https://openalex.org/W1967643968; https://openalex.org/W1970594742; https://openalex.org/W1977496278; https://openalex.org/W1978962787; https://openalex.org/W1980945904; https://openalex.org/W1982635318; https://openalex.org/W1983150145; https://openalex.org/W1983380373; https://openalex.org/W1987888496; https://openalex.org/W1987984266; https://openalex.org/W1994451802; https://openalex.org/W1995925293; https://openalex.org/W2002613604; https://openalex.org/W2003179529; https://openalex.org/W2004039783; https://openalex.org/W2006260073; https://openalex.org/W2012352340; https://openalex.org/W2012674856; https://openalex.org/W2014102731; https://openalex.org/W2014464762; https://openalex.org/W2016070752; https://openalex.org/W2017396468; https://openalex.org/W2020925091; https://openalex.org/W2022892346; https://openalex.org/W2025357764; https://openalex.org/W2025640367; https://openalex.org/W2027902860; https://openalex.org/W2028504354; https://openalex.org/W2030363461; https://openalex.org/W2031795937; https://openalex.org/W2040015143; https://openalex.org/W2040884411; https://openalex.org/W2043420811; https://openalex.org/W2044289181; https://openalex.org/W2048178552; https://openalex.org/W2050431484; https://openalex.org/W2051680981; https://openalex.org/W2056517460; https://openalex.org/W2058232500; https://openalex.org/W2060542593; https://openalex.org/W2061692200; https://openalex.org/W2063341754; https://openalex.org/W2063978378; https://openalex.org/W2066944227; https://openalex.org/W2070996757; https://openalex.org/W2076384720; https://openalex.org/W2076542102; https://openalex.org/W2077959816; https://openalex.org/W2079709766; https://openalex.org/W2081028792; https://openalex.org/W2083272186; https://openalex.org/W2086424613; https://openalex.org/W2087973052; https://openalex.org/W2089137303; https://openalex.org/W2089898582; https://openalex.org/W2090123586; https://openalex.org/W2093045504; https://openalex.org/W2094397139; https://openalex.org/W2099322651; https://openalex.org/W2102207582; https://openalex.org/W2102413177; https://openalex.org/W2102708620; https://openalex.org/W2102831150; https://openalex.org/W2104766538; https://openalex.org/W2105875820; https://openalex.org/W2107979498; https://openalex.org/W2109155353; https://openalex.org/W2113242816; https://openalex.org/W2115412314; https://openalex.org/W2117004913; https://openalex.org/W2118561568; https://openalex.org/W2119689447; https://openalex.org/W2122499709; https://openalex.org/W2122825543; https://openalex.org/W2125055259; https://openalex.org/W2126185804; https://openalex.org/W2126611570; https://openalex.org/W2130302054; https://openalex.org/W2131101925; https://openalex.org/W2133143568; https://openalex.org/W2134208464; https://openalex.org/W2134544888; https://openalex.org/W2135046866; https://openalex.org/W2138570191; https://openalex.org/W2140190241; https://openalex.org/W2143426320; https://openalex.org/W2143539328; https://openalex.org/W2145955247; https://openalex.org/W2147339185; https://openalex.org/W2147345348; https://openalex.org/W2148730406; https://openalex.org/W2149043691; https://openalex.org/W2149454242; https://openalex.org/W2149620660; https://openalex.org/W2149772057; https://openalex.org/W2150102617; https://openalex.org/W2150248355; https://openalex.org/W2150747245; https://openalex.org/W2153338628; https://openalex.org/W2153377299; https://openalex.org/W2154053567; https://openalex.org/W2154706222; https://openalex.org/W2155344811; https://openalex.org/W2155461849; https://openalex.org/W2155648952; https://openalex.org/W2156571267; https://openalex.org/W2156758690; https://openalex.org/W2157317320; https://openalex.org/W2158012006; https://openalex.org/W2158469157; https://openalex.org/W2160164899; https://openalex.org/W2160488076; https://openalex.org/W2161182256; https://openalex.org/W2163264097; https://openalex.org/W2165250079; https://openalex.org/W2165835468; https://openalex.org/W2166267715; https://openalex.org/W2167776024; https://openalex.org/W2184364778; https://openalex.org/W2319669445; https://openalex.org/W2344681634; https://openalex.org/W2379509210; https://openalex.org/W2398336627; https://openalex.org/W2478358886; https://openalex.org/W2488133945; https://openalex.org/W2516294100; https://openalex.org/W2516938563; https://openalex.org/W2531563875; https://openalex.org/W2533318895; https://openalex.org/W2550999023; https://openalex.org/W2554446914; https://openalex.org/W2560674852; https://openalex.org/W2566313994; https://openalex.org/W2578238698; https://openalex.org/W2586696233; https://openalex.org/W2590286530; https://openalex.org/W2596799992; https://openalex.org/W2599276638; https://openalex.org/W2741543704; https://openalex.org/W2800106282; https://openalex.org/W2911640577; https://openalex.org/W2911681169; https://openalex.org/W2911964244; https://openalex.org/W2912467488; https://openalex.org/W2950901611; https://openalex.org/W2997674406; https://openalex.org/W2998216295; https://openalex.org/W3003734944; https://openalex.org/W3105524694; https://openalex.org/W3139732350; https://openalex.org/W3144008936; https://openalex.org/W4213245422; https://openalex.org/W4214740783; https://openalex.org/W4233164864; https://openalex.org/W4235838756; https://openalex.org/W4239666910; https://openalex.org/W4244877265; https://openalex.org/W4248003669; https://openalex.org/W4252566574; https://openalex.org/W4254300870; https://openalex.org/W4285719527; https://openalex.org/W4297873013; https://openalex.org/W4300101671; https://openalex.org/W6602507595; https://openalex.org/W6604434393; https://openalex.org/W6605134655; https://openalex.org/W6605578906; https://openalex.org/W6605960250; https://openalex.org/W6607161487; https://openalex.org/W6608247899; https://openalex.org/W6628796916; https://openalex.org/W6632582745; https://openalex.org/W6633167049; https://openalex.org/W6633497745; https://openalex.org/W6634692335; https://openalex.org/W6635046684; https://openalex.org/W6636336243; https://openalex.org/W6638201858; https://openalex.org/W6638249342; https://openalex.org/W6639167513; https://openalex.org/W6639817432; https://openalex.org/W6640718358; https://openalex.org/W6642023902; https://openalex.org/W6645174655; https://openalex.org/W6645634710; https://openalex.org/W6645712975; https://openalex.org/W6645986874; https://openalex.org/W6649353885; https://openalex.org/W6651118512; https://openalex.org/W6654415589; https://openalex.org/W6660318337; https://openalex.org/W6663537612; https://openalex.org/W6668178708; https://openalex.org/W6671241806; https://openalex.org/W6672508006; https://openalex.org/W6674946015; https://openalex.org/W6674952872; https://openalex.org/W6675935835; https://openalex.org/W6676563591; https://openalex.org/W6677786031; https://openalex.org/W6678522416; https://openalex.org/W6678932631; https://openalex.org/W6679144653; https://openalex.org/W6679384483; https://openalex.org/W6680095430; https://openalex.org/W6680765659; https://openalex.org/W6681822384; https://openalex.org/W6681875376; https://openalex.org/W6681923237; https://openalex.org/W6681948290; https://openalex.org/W6682496738; https://openalex.org/W6682744373; https://openalex.org/W6682904970; https://openalex.org/W6682926446; https://openalex.org/W6683024897; https://openalex.org/W6683561382; https://openalex.org/W6683942726; https://openalex.org/W6683993829; https://openalex.org/W6685046167; https://openalex.org/W6686231358; https://openalex.org/W6721249974; https://openalex.org/W6729106673; https://openalex.org/W6729685833; https://openalex.org/W6731561570; https://openalex.org/W6732256179; https://openalex.org/W6735148111; https://openalex.org/W6742166947; https://openalex.org/W6758972637; https://openalex.org/W7055425972; https://openalex.org/W7066667914</t>
         </is>
       </c>
       <c r="Q94" t="inlineStr">
         <is>
-          <t>Computer science;Deep learning;Artificial intelligence;Abstraction;Representation (politics);Layer (electronics);Object (grammar);Backpropagation;Convolutional neural network;Feature learning;Pattern recognition (psychology);Speech recognition;Artificial neural network</t>
+          <t>Feature selection;Machine learning;Computer science;Artificial intelligence;Cluster analysis;Feature (linguistics);Perspective (graphical);Selection (genetic algorithm);Unsupervised learning;Supervised learning;Feature learning;Data mining;Artificial neural network</t>
         </is>
       </c>
       <c r="R94" t="inlineStr"/>
       <c r="S94" t="inlineStr"/>
       <c r="T94" t="inlineStr">
         <is>
-          <t>521</t>
-        </is>
-      </c>
-      <c r="U94" t="inlineStr">
-        <is>
-          <t>7553</t>
-        </is>
-      </c>
+          <t>300</t>
+        </is>
+      </c>
+      <c r="U94" t="inlineStr"/>
       <c r="V94" t="inlineStr">
         <is>
-          <t>436</t>
+          <t>70</t>
         </is>
       </c>
       <c r="W94" t="inlineStr">
         <is>
-          <t>444</t>
+          <t>79</t>
         </is>
       </c>
       <c r="X94" t="inlineStr">
         <is>
-          <t>Yann LeCun, 2015, Nature</t>
+          <t>Jie Cai, 2018, Neurocomputing</t>
         </is>
       </c>
       <c r="Y94" t="inlineStr">
         <is>
-          <t>Yann LeCun, 2015, Nature</t>
+          <t>Jie Cai, 2018, Neurocomputing</t>
         </is>
       </c>
     </row>
@@ -9327,36 +9323,36 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>https://openalex.org/W2791315675</t>
+          <t>https://openalex.org/W2919115771</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1016/j.neucom.2017.11.077</t>
+          <t>https://doi.org/10.1038/nature14539</t>
         </is>
       </c>
       <c r="D95" t="inlineStr"/>
       <c r="E95" t="inlineStr">
         <is>
-          <t>Feature selection in machine learning: A new perspective</t>
+          <t>Deep learning</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>Neurocomputing</t>
+          <t>Nature</t>
         </is>
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>Neurocomputing</t>
+          <t>Nature</t>
         </is>
       </c>
       <c r="H95" t="n">
-        <v>2018</v>
+        <v>2015</v>
       </c>
       <c r="I95" t="inlineStr">
         <is>
-          <t>article</t>
+          <t>review</t>
         </is>
       </c>
       <c r="J95" t="inlineStr">
@@ -9365,56 +9361,60 @@
         </is>
       </c>
       <c r="K95" t="n">
-        <v>2059</v>
+        <v>81904</v>
       </c>
       <c r="L95" t="inlineStr">
         <is>
-          <t>Jie Cai;Jiawei Luo;Shulin Wang;Sheng Yang</t>
+          <t>Yann LeCun;Yoshua Bengio;Geoffrey E. Hinton</t>
         </is>
       </c>
       <c r="M95" t="inlineStr"/>
       <c r="N95" t="inlineStr">
         <is>
-          <t>Jie Cai, College of Computer Science and Electronic Engineering, Hunan University, Changsha, Hunan, China;Jiawei Luo, College of Computer Science and Electronic Engineering, Hunan University, Changsha, Hunan, China;Shulin Wang, College of Computer Science and Electronic Engineering, Hunan University, Changsha, Hunan, China;Sheng Yang, College of Computer Science and Electronic Engineering, Hunan University, Changsha, Hunan, China</t>
+          <t>Yann LeCun, 1] Facebook AI Research, 770 Broadway, New York, New York 10003 USA. [2] New York University, 715 Broadway, New York, New York 10003, USA;Yann LeCun, Facebook AI Research, 770 Broadway, New York, 10003, New York, USA;Yann LeCun, New York University, 715 Broadway, New York, 10003, New York, USA;Yoshua Bengio, Department of Computer Science and Operations Research Université de Montréal, Pavillon André-Aisenstadt, PO Box 6128 Centre-Ville STN Montréal, Quebec H3C 3J7, Canada;Yoshua Bengio, Department of Computer Science and Operations Research Université de Montréal, Pavillon André-Aisenstadt, PO Box 6128 Centre-Ville STN, Montréal, H3C 3J7, Quebec, Canada;Geoffrey E. Hinton, 1] Google, 1600 Amphitheatre Parkway, Mountain View, California 94043, USA. [2] Department of Computer Science, University of Toronto, 6 King's College Road, Toronto, Ontario M5S 3G4, Canada;Geoffrey E. Hinton, Google, 1600 Amphitheatre Parkway, Mountain View, 94043, California, USA;Geoffrey E. Hinton, Department of Computer Science, University of Toronto, 6 King's College Road, Toronto, M5S 3G4, Ontario, Canada</t>
         </is>
       </c>
       <c r="O95" t="inlineStr"/>
       <c r="P95" t="inlineStr">
         <is>
-          <t>https://openalex.org/W62404953; https://openalex.org/W110173923; https://openalex.org/W129457532; https://openalex.org/W137065004; https://openalex.org/W140777655; https://openalex.org/W146732357; https://openalex.org/W175909076; https://openalex.org/W204835077; https://openalex.org/W323404752; https://openalex.org/W1253096047; https://openalex.org/W1480716458; https://openalex.org/W1541321639; https://openalex.org/W1543715688; https://openalex.org/W1546113605; https://openalex.org/W1554275123; https://openalex.org/W1554663460; https://openalex.org/W1555244713; https://openalex.org/W1560107318; https://openalex.org/W1570713908; https://openalex.org/W1581426664; https://openalex.org/W1583700199; https://openalex.org/W1583837637; https://openalex.org/W1585743408; https://openalex.org/W1590246454; https://openalex.org/W1608549042; https://openalex.org/W1761159547; https://openalex.org/W1804170020; https://openalex.org/W1808644423; https://openalex.org/W1887132526; https://openalex.org/W1898334332; https://openalex.org/W1949281989; https://openalex.org/W1958291604; https://openalex.org/W1964042173; https://openalex.org/W1964137961; https://openalex.org/W1967643968; https://openalex.org/W1970594742; https://openalex.org/W1977496278; https://openalex.org/W1978962787; https://openalex.org/W1980945904; https://openalex.org/W1982635318; https://openalex.org/W1983150145; https://openalex.org/W1983380373; https://openalex.org/W1987888496; https://openalex.org/W1987984266; https://openalex.org/W1994451802; https://openalex.org/W1995925293; https://openalex.org/W2002613604; https://openalex.org/W2003179529; https://openalex.org/W2004039783; https://openalex.org/W2006260073; https://openalex.org/W2012352340; https://openalex.org/W2012674856; https://openalex.org/W2014102731; https://openalex.org/W2014464762; https://openalex.org/W2016070752; https://openalex.org/W2017396468; https://openalex.org/W2020925091; https://openalex.org/W2022892346; https://openalex.org/W2025357764; https://openalex.org/W2025640367; https://openalex.org/W2027902860; https://openalex.org/W2028504354; https://openalex.org/W2030363461; https://openalex.org/W2031795937; https://openalex.org/W2040015143; https://openalex.org/W2040884411; https://openalex.org/W2043420811; https://openalex.org/W2044289181; https://openalex.org/W2048178552; https://openalex.org/W2050431484; https://openalex.org/W2051680981; https://openalex.org/W2056517460; https://openalex.org/W2058232500; https://openalex.org/W2060542593; https://openalex.org/W2061692200; https://openalex.org/W2063341754; https://openalex.org/W2063978378; https://openalex.org/W2066944227; https://openalex.org/W2070996757; https://openalex.org/W2076384720; https://openalex.org/W2076542102; https://openalex.org/W2077959816; https://openalex.org/W2079709766; https://openalex.org/W2081028792; https://openalex.org/W2083272186; https://openalex.org/W2086424613; https://openalex.org/W2087973052; https://openalex.org/W2089137303; https://openalex.org/W2089898582; https://openalex.org/W2090123586; https://openalex.org/W2093045504; https://openalex.org/W2094397139; https://openalex.org/W2099322651; https://openalex.org/W2102207582; https://openalex.org/W2102413177; https://openalex.org/W2102708620; https://openalex.org/W2102831150; https://openalex.org/W2104766538; https://openalex.org/W2105875820; https://openalex.org/W2107979498; https://openalex.org/W2109155353; https://openalex.org/W2113242816; https://openalex.org/W2115412314; https://openalex.org/W2117004913; https://openalex.org/W2118561568; https://openalex.org/W2119689447; https://openalex.org/W2122499709; https://openalex.org/W2122825543; https://openalex.org/W2125055259; https://openalex.org/W2126185804; https://openalex.org/W2126611570; https://openalex.org/W2130302054; https://openalex.org/W2131101925; https://openalex.org/W2133143568; https://openalex.org/W2134208464; https://openalex.org/W2134544888; https://openalex.org/W2135046866; https://openalex.org/W2138570191; https://openalex.org/W2140190241; https://openalex.org/W2143426320; https://openalex.org/W2143539328; https://openalex.org/W2145955247; https://openalex.org/W2147339185; https://openalex.org/W2147345348; https://openalex.org/W2148730406; https://openalex.org/W2149043691; https://openalex.org/W2149454242; https://openalex.org/W2149620660; https://openalex.org/W2149772057; https://openalex.org/W2150102617; https://openalex.org/W2150248355; https://openalex.org/W2150747245; https://openalex.org/W2153338628; https://openalex.org/W2153377299; https://openalex.org/W2154053567; https://openalex.org/W2154706222; https://openalex.org/W2155344811; https://openalex.org/W2155461849; https://openalex.org/W2155648952; https://openalex.org/W2156571267; https://openalex.org/W2156758690; https://openalex.org/W2157317320; https://openalex.org/W2158012006; https://openalex.org/W2158469157; https://openalex.org/W2160164899; https://openalex.org/W2160488076; https://openalex.org/W2161182256; https://openalex.org/W2163264097; https://openalex.org/W2165250079; https://openalex.org/W2165835468; https://openalex.org/W2166267715; https://openalex.org/W2167776024; https://openalex.org/W2184364778; https://openalex.org/W2319669445; https://openalex.org/W2344681634; https://openalex.org/W2379509210; https://openalex.org/W2398336627; https://openalex.org/W2478358886; https://openalex.org/W2488133945; https://openalex.org/W2516294100; https://openalex.org/W2516938563; https://openalex.org/W2531563875; https://openalex.org/W2533318895; https://openalex.org/W2550999023; https://openalex.org/W2554446914; https://openalex.org/W2560674852; https://openalex.org/W2566313994; https://openalex.org/W2578238698; https://openalex.org/W2586696233; https://openalex.org/W2590286530; https://openalex.org/W2596799992; https://openalex.org/W2599276638; https://openalex.org/W2741543704; https://openalex.org/W2800106282; https://openalex.org/W2911640577; https://openalex.org/W2911681169; https://openalex.org/W2911964244; https://openalex.org/W2912467488; https://openalex.org/W2950901611; https://openalex.org/W2997674406; https://openalex.org/W2998216295; https://openalex.org/W3003734944; https://openalex.org/W3105524694; https://openalex.org/W3139732350; https://openalex.org/W3144008936; https://openalex.org/W4213245422; https://openalex.org/W4214740783; https://openalex.org/W4233164864; https://openalex.org/W4235838756; https://openalex.org/W4239666910; https://openalex.org/W4244877265; https://openalex.org/W4248003669; https://openalex.org/W4252566574; https://openalex.org/W4254300870; https://openalex.org/W4285719527; https://openalex.org/W4297873013; https://openalex.org/W4300101671; https://openalex.org/W6602507595; https://openalex.org/W6604434393; https://openalex.org/W6605134655; https://openalex.org/W6605578906; https://openalex.org/W6605960250; https://openalex.org/W6607161487; https://openalex.org/W6608247899; https://openalex.org/W6628796916; https://openalex.org/W6632582745; https://openalex.org/W6633167049; https://openalex.org/W6633497745; https://openalex.org/W6634692335; https://openalex.org/W6635046684; https://openalex.org/W6636336243; https://openalex.org/W6638201858; https://openalex.org/W6638249342; https://openalex.org/W6639167513; https://openalex.org/W6639817432; https://openalex.org/W6640718358; https://openalex.org/W6642023902; https://openalex.org/W6645174655; https://openalex.org/W6645634710; https://openalex.org/W6645712975; https://openalex.org/W6645986874; https://openalex.org/W6649353885; https://openalex.org/W6651118512; https://openalex.org/W6654415589; https://openalex.org/W6660318337; https://openalex.org/W6663537612; https://openalex.org/W6668178708; https://openalex.org/W6671241806; https://openalex.org/W6672508006; https://openalex.org/W6674946015; https://openalex.org/W6674952872; https://openalex.org/W6675935835; https://openalex.org/W6676563591; https://openalex.org/W6677786031; https://openalex.org/W6678522416; https://openalex.org/W6678932631; https://openalex.org/W6679144653; https://openalex.org/W6679384483; https://openalex.org/W6680095430; https://openalex.org/W6680765659; https://openalex.org/W6681822384; https://openalex.org/W6681875376; https://openalex.org/W6681923237; https://openalex.org/W6681948290; https://openalex.org/W6682496738; https://openalex.org/W6682744373; https://openalex.org/W6682904970; https://openalex.org/W6682926446; https://openalex.org/W6683024897; https://openalex.org/W6683561382; https://openalex.org/W6683942726; https://openalex.org/W6683993829; https://openalex.org/W6685046167; https://openalex.org/W6686231358; https://openalex.org/W6721249974; https://openalex.org/W6729106673; https://openalex.org/W6729685833; https://openalex.org/W6731561570; https://openalex.org/W6732256179; https://openalex.org/W6735148111; https://openalex.org/W6742166947; https://openalex.org/W6758972637; https://openalex.org/W7055425972; https://openalex.org/W7066667914</t>
+          <t>https://openalex.org/W146900863; https://openalex.org/W170811313; https://openalex.org/W1487583988; https://openalex.org/W1498436455; https://openalex.org/W1514535095; https://openalex.org/W1573503290; https://openalex.org/W1752712236; https://openalex.org/W1970689298; https://openalex.org/W1978592082; https://openalex.org/W1993845689; https://openalex.org/W1993882792; https://openalex.org/W1999497791; https://openalex.org/W1999798000; https://openalex.org/W2022508996; https://openalex.org/W2025768430; https://openalex.org/W2064675550; https://openalex.org/W2072128103; https://openalex.org/W2074551195; https://openalex.org/W2085989895; https://openalex.org/W2088338354; https://openalex.org/W2091987367; https://openalex.org/W2095739681; https://openalex.org/W2098580305; https://openalex.org/W2100495367; https://openalex.org/W2107878631; https://openalex.org/W2108069432; https://openalex.org/W2111304802; https://openalex.org/W2112796928; https://openalex.org/W2116360511; https://openalex.org/W2117671523; https://openalex.org/W2120284346; https://openalex.org/W2120432001; https://openalex.org/W2121289914; https://openalex.org/W2136922672; https://openalex.org/W2144015117; https://openalex.org/W2144354855; https://openalex.org/W2145339207; https://openalex.org/W2146989110; https://openalex.org/W2157331557; https://openalex.org/W2158778629; https://openalex.org/W2160815625; https://openalex.org/W2163922914; https://openalex.org/W2166206801; https://openalex.org/W2169488311; https://openalex.org/W2169805405; https://openalex.org/W2800394774; https://openalex.org/W3139812727; https://openalex.org/W4232280717; https://openalex.org/W4249882522; https://openalex.org/W6630820455; https://openalex.org/W6674914833; https://openalex.org/W6683738474; https://openalex.org/W6743198006</t>
         </is>
       </c>
       <c r="Q95" t="inlineStr">
         <is>
-          <t>Feature selection;Machine learning;Computer science;Artificial intelligence;Cluster analysis;Feature (linguistics);Perspective (graphical);Selection (genetic algorithm);Unsupervised learning;Supervised learning;Feature learning;Data mining;Artificial neural network</t>
+          <t>Computer science;Deep learning;Artificial intelligence;Abstraction;Representation (politics);Layer (electronics);Object (grammar);Backpropagation;Convolutional neural network;Feature learning;Pattern recognition (psychology);Speech recognition;Artificial neural network</t>
         </is>
       </c>
       <c r="R95" t="inlineStr"/>
       <c r="S95" t="inlineStr"/>
       <c r="T95" t="inlineStr">
         <is>
-          <t>300</t>
-        </is>
-      </c>
-      <c r="U95" t="inlineStr"/>
+          <t>521</t>
+        </is>
+      </c>
+      <c r="U95" t="inlineStr">
+        <is>
+          <t>7553</t>
+        </is>
+      </c>
       <c r="V95" t="inlineStr">
         <is>
-          <t>70</t>
+          <t>436</t>
         </is>
       </c>
       <c r="W95" t="inlineStr">
         <is>
-          <t>79</t>
+          <t>444</t>
         </is>
       </c>
       <c r="X95" t="inlineStr">
         <is>
-          <t>Jie Cai, 2018, Neurocomputing</t>
+          <t>Yann LeCun, 2015, Nature</t>
         </is>
       </c>
       <c r="Y95" t="inlineStr">
         <is>
-          <t>Jie Cai, 2018, Neurocomputing</t>
+          <t>Yann LeCun, 2015, Nature</t>
         </is>
       </c>
     </row>
@@ -9464,7 +9464,7 @@
         </is>
       </c>
       <c r="K96" t="n">
-        <v>2080</v>
+        <v>2085</v>
       </c>
       <c r="L96" t="inlineStr">
         <is>
@@ -9571,7 +9571,7 @@
         </is>
       </c>
       <c r="K97" t="n">
-        <v>3080</v>
+        <v>3083</v>
       </c>
       <c r="L97" t="inlineStr">
         <is>
@@ -9753,7 +9753,7 @@
         </is>
       </c>
       <c r="K99" t="n">
-        <v>2404</v>
+        <v>2409</v>
       </c>
       <c r="L99" t="inlineStr">
         <is>
@@ -9814,36 +9814,36 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>https://openalex.org/W2168029744</t>
+          <t>https://openalex.org/W4213308398</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1214/009053607000000677</t>
+          <t>https://doi.org/10.1007/978-3-030-05318-5</t>
         </is>
       </c>
       <c r="D100" t="inlineStr"/>
       <c r="E100" t="inlineStr">
         <is>
-          <t>Kernel methods in machine learning</t>
+          <t>Automated Machine Learning</t>
         </is>
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>The Annals of Statistics</t>
+          <t>The Springer series on challenges in machine learning</t>
         </is>
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>The Annals of Statistics</t>
+          <t>The Springer series on challenges in machine learning</t>
         </is>
       </c>
       <c r="H100" t="n">
-        <v>2008</v>
+        <v>2019</v>
       </c>
       <c r="I100" t="inlineStr">
         <is>
-          <t>article</t>
+          <t>book</t>
         </is>
       </c>
       <c r="J100" t="inlineStr">
@@ -9852,56 +9852,48 @@
         </is>
       </c>
       <c r="K100" t="n">
-        <v>1598</v>
+        <v>1405</v>
       </c>
       <c r="L100" t="inlineStr">
         <is>
-          <t>Thomas Hofmann;Bernhard Schölkopf;Alexander J. Smola</t>
+          <t>Frank Hutter;Lars Kotthoff;Joaquin Vanschoren</t>
         </is>
       </c>
       <c r="M100" t="inlineStr"/>
       <c r="N100" t="inlineStr">
         <is>
-          <t>Thomas Hofmann, Darmstadt University of Technology, Max Planck Institute for Biological Cybernetics and National ICT Australia;Alexander J. Smola, Darmstadt University of Technology, Max Planck Institute for Biological Cybernetics and National ICT Australia;Alexander J. Smola, MAX PLANCK INSTITUTE FOR BIOLOGICAL CYBERNETICS TBINGEN GERMANY</t>
+          <t>Frank Hutter, Department of Computer Science, University of Freiburg, Freiburg, Germany;Lars Kotthoff, University of Wyoming, Laramie, USA;Joaquin Vanschoren, Eindhoven University of Technology, Eindhoven, The Netherlands</t>
         </is>
       </c>
       <c r="O100" t="inlineStr"/>
       <c r="P100" t="inlineStr">
         <is>
-          <t>https://openalex.org/W14071851; https://openalex.org/W56743589; https://openalex.org/W179694669; https://openalex.org/W1490266132; https://openalex.org/W1496189301; https://openalex.org/W1510073064; https://openalex.org/W1512098439; https://openalex.org/W1526146785; https://openalex.org/W1526729636; https://openalex.org/W1542652324; https://openalex.org/W1549656520; https://openalex.org/W1550988992; https://openalex.org/W1560729174; https://openalex.org/W1575431606; https://openalex.org/W1578255497; https://openalex.org/W1587744656; https://openalex.org/W1596052433; https://openalex.org/W1604293137; https://openalex.org/W1638081485; https://openalex.org/W1647376582; https://openalex.org/W1719651905; https://openalex.org/W1774304772; https://openalex.org/W1835509607; https://openalex.org/W1899157803; https://openalex.org/W1966347620; https://openalex.org/W1968934255; https://openalex.org/W1975077471; https://openalex.org/W1982032418; https://openalex.org/W1986931325; https://openalex.org/W1989408439; https://openalex.org/W1990534247; https://openalex.org/W1991200719; https://openalex.org/W1992236290; https://openalex.org/W1992666150; https://openalex.org/W1995558350; https://openalex.org/W1998438337; https://openalex.org/W1999486090; https://openalex.org/W2001792610; https://openalex.org/W2002806284; https://openalex.org/W2007154098; https://openalex.org/W2008400752; https://openalex.org/W2009511046; https://openalex.org/W2014902932; https://openalex.org/W2015904350; https://openalex.org/W2018582985; https://openalex.org/W2020816856; https://openalex.org/W2025341678; https://openalex.org/W2051381803; https://openalex.org/W2060591526; https://openalex.org/W2064976291; https://openalex.org/W2070771761; https://openalex.org/W2075887074; https://openalex.org/W2082100828; https://openalex.org/W2082612735; https://openalex.org/W2083780577; https://openalex.org/W2086404575; https://openalex.org/W2087258353; https://openalex.org/W2087347434; https://openalex.org/W2092182929; https://openalex.org/W2098385651; https://openalex.org/W2101276256; https://openalex.org/W2103657184; https://openalex.org/W2104128541; https://openalex.org/W2105842272; https://openalex.org/W2106353560; https://openalex.org/W2108153239; https://openalex.org/W2112076978; https://openalex.org/W2114281975; https://openalex.org/W2119647652; https://openalex.org/W2120340025; https://openalex.org/W2121127625; https://openalex.org/W2123606421; https://openalex.org/W2123737232; https://openalex.org/W2124101779; https://openalex.org/W2124225821; https://openalex.org/W2125053431; https://openalex.org/W2127713198; https://openalex.org/W2131479089; https://openalex.org/W2132637896; https://openalex.org/W2132870739; https://openalex.org/W2135046866; https://openalex.org/W2135498906; https://openalex.org/W2139686264; https://openalex.org/W2140095548; https://openalex.org/W2141224867; https://openalex.org/W2141407058; https://openalex.org/W2143956139; https://openalex.org/W2144068644; https://openalex.org/W2148018895; https://openalex.org/W2151949149; https://openalex.org/W2156515921; https://openalex.org/W2156909104; https://openalex.org/W2157791002; https://openalex.org/W2159737176; https://openalex.org/W2161920802; https://openalex.org/W2162836072; https://openalex.org/W2164943005; https://openalex.org/W2169945149; https://openalex.org/W2408196097; https://openalex.org/W2554813760; https://openalex.org/W2795528501; https://openalex.org/W2988119488; https://openalex.org/W2994982620; https://openalex.org/W4210636998; https://openalex.org/W4232576706; https://openalex.org/W4234698323; https://openalex.org/W4238284510; https://openalex.org/W4238957295; https://openalex.org/W4239510810; https://openalex.org/W4246066915; https://openalex.org/W4247545571; https://openalex.org/W4249925659; https://openalex.org/W4251085907; https://openalex.org/W4251115686; https://openalex.org/W4298876635; https://openalex.org/W4396738453</t>
+          <t>https://openalex.org/W6908809; https://openalex.org/W24696228; https://openalex.org/W28412257; https://openalex.org/W41730657; https://openalex.org/W54639073; https://openalex.org/W60686164; https://openalex.org/W62188234; https://openalex.org/W76131926; https://openalex.org/W76331760; https://openalex.org/W85803853; https://openalex.org/W100047375; https://openalex.org/W114730584; https://openalex.org/W116375701; https://openalex.org/W122178443; https://openalex.org/W135104305; https://openalex.org/W138547447; https://openalex.org/W145519053; https://openalex.org/W148859753; https://openalex.org/W172742023; https://openalex.org/W174542576; https://openalex.org/W192975702; https://openalex.org/W198580638; https://openalex.org/W202805564; https://openalex.org/W202978992; https://openalex.org/W358897728; https://openalex.org/W603776396; https://openalex.org/W1165382972; https://openalex.org/W1471542436; https://openalex.org/W1480330138; https://openalex.org/W1484746829; https://openalex.org/W1488960379; https://openalex.org/W1491420040; https://openalex.org/W1494192115; https://openalex.org/W1494580925; https://openalex.org/W1500302649; https://openalex.org/W1501110974; https://openalex.org/W1503705371; https://openalex.org/W1507030697; https://openalex.org/W1512747601; https://openalex.org/W1516621661; https://openalex.org/W1519451279; https://openalex.org/W1520992199; https://openalex.org/W1522301498; https://openalex.org/W1528411633; https://openalex.org/W1533803232; https://openalex.org/W1534069108; https://openalex.org/W1534477342; https://openalex.org/W1535039099; https://openalex.org/W1539741229; https://openalex.org/W1542791059; https://openalex.org/W1543201103; https://openalex.org/W1549223806; https://openalex.org/W1556753024; https://openalex.org/W1565746575; https://openalex.org/W1568834902; https://openalex.org/W1569757501; https://openalex.org/W1575029535; https://openalex.org/W1575661061; https://openalex.org/W1577932924; https://openalex.org/W1581066146; https://openalex.org/W1588486985; https://openalex.org/W1588628884; https://openalex.org/W1588959569; https://openalex.org/W1589492330; https://openalex.org/W1593343777; https://openalex.org/W1598052524; https://openalex.org/W1601795611; https://openalex.org/W1604262624; https://openalex.org/W1631708156; https://openalex.org/W1638732406; https://openalex.org/W1640798781; https://openalex.org/W1647221522; https://openalex.org/W1661871015; https://openalex.org/W1663203009; https://openalex.org/W1663583528; https://openalex.org/W1678356000; https://openalex.org/W1680392829; https://openalex.org/W1690919088; https://openalex.org/W1701825639; https://openalex.org/W1758907577; https://openalex.org/W1763644767; https://openalex.org/W1840091437; https://openalex.org/W1868018859; https://openalex.org/W1880189740; https://openalex.org/W1886872224; https://openalex.org/W1922017469; https://openalex.org/W1925428099; https://openalex.org/W1925504357; https://openalex.org/W1935590542; https://openalex.org/W1965555277; https://openalex.org/W1968634175; https://openalex.org/W1969163824; https://openalex.org/W1971713783; https://openalex.org/W1973229481; https://openalex.org/W1979769287; https://openalex.org/W1980264541; https://openalex.org/W1981903823; https://openalex.org/W1984557319; https://openalex.org/W1985995090; https://openalex.org/W1986490585; https://openalex.org/W1986543815; https://openalex.org/W1986929000; https://openalex.org/W1989048657; https://openalex.org/W1994197834; https://openalex.org/W1994326354; https://openalex.org/W2001485654; https://openalex.org/W2040730773; https://openalex.org/W2040884411; https://openalex.org/W2048430744; https://openalex.org/W2050310928; https://openalex.org/W2051346631; https://openalex.org/W2056224615; https://openalex.org/W2057261601; https://openalex.org/W2062118960; https://openalex.org/W2062227835; https://openalex.org/W2064186732; https://openalex.org/W2074702228; https://openalex.org/W2074724805; https://openalex.org/W2078885513; https://openalex.org/W2083542829; https://openalex.org/W2084136177; https://openalex.org/W2084150578; https://openalex.org/W2087817842; https://openalex.org/W2089213632; https://openalex.org/W2089217417; https://openalex.org/W2090136295; https://openalex.org/W2091118421; https://openalex.org/W2095655959; https://openalex.org/W2095705004; https://openalex.org/W2096863518; https://openalex.org/W2097998348; https://openalex.org/W2099201756; https://openalex.org/W2101234009; https://openalex.org/W2101341561; https://openalex.org/W2102770307; https://openalex.org/W2105031846; https://openalex.org/W2106411961; https://openalex.org/W2106614481; https://openalex.org/W2107853397; https://openalex.org/W2108626634; https://openalex.org/W2109042184; https://openalex.org/W2109346685; https://openalex.org/W2111935653; https://openalex.org/W2112204321; https://openalex.org/W2112364454; https://openalex.org/W2113145584; https://openalex.org/W2113207845; https://openalex.org/W2113584252; https://openalex.org/W2115733720; https://openalex.org/W2115763804; https://openalex.org/W2116882733; https://openalex.org/W2117539524; https://openalex.org/W2118789407; https://openalex.org/W2119814172; https://openalex.org/W2120420045; https://openalex.org/W2122053572; https://openalex.org/W2122379760; https://openalex.org/W2122776323; https://openalex.org/W2123395972; https://openalex.org/W2123649031; https://openalex.org/W2124022122; https://openalex.org/W2124290836; https://openalex.org/W2124802506; https://openalex.org/W2125849100; https://openalex.org/W2125877832; https://openalex.org/W2126204609; https://openalex.org/W2126559945; https://openalex.org/W2126964466; https://openalex.org/W2127416213; https://openalex.org/W2129458072; https://openalex.org/W2130942839; https://openalex.org/W2131241448; https://openalex.org/W2131822674; https://openalex.org/W2133418613; https://openalex.org/W2133958955; https://openalex.org/W2136139971; https://openalex.org/W2136636278; https://openalex.org/W2137825550; https://openalex.org/W2138784882; https://openalex.org/W2139805416; https://openalex.org/W2141125852; https://openalex.org/W2141408223; https://openalex.org/W2142334564; https://openalex.org/W2142959074; https://openalex.org/W2143104527; https://openalex.org/W2144656844; https://openalex.org/W2144752499; https://openalex.org/W2144981148; https://openalex.org/W2145287260; https://openalex.org/W2145339207; https://openalex.org/W2145955992; https://openalex.org/W2146502635; https://openalex.org/W2149731329; https://openalex.org/W2150446468; https://openalex.org/W2152589362; https://openalex.org/W2153667946; https://openalex.org/W2154776925; https://openalex.org/W2155853132; https://openalex.org/W2156417353; https://openalex.org/W2157069634; https://openalex.org/W2160644528; https://openalex.org/W2163605009; https://openalex.org/W2163922914; https://openalex.org/W2165607334; https://openalex.org/W2165698076; https://openalex.org/W2165962877; https://openalex.org/W2166107799; https://openalex.org/W2168175751; https://openalex.org/W2168939893; https://openalex.org/W2171033594; https://openalex.org/W2171658832; https://openalex.org/W2181956361; https://openalex.org/W2182070128; https://openalex.org/W2182361439; https://openalex.org/W2183341477; https://openalex.org/W2183704914; https://openalex.org/W2186013251; https://openalex.org/W2189149359; https://openalex.org/W2192203593; https://openalex.org/W2194775991; https://openalex.org/W2200000192; https://openalex.org/W2210969396; https://openalex.org/W2226783037; https://openalex.org/W2234598170; https://openalex.org/W2234898963; https://openalex.org/W2249362929; https://openalex.org/W2250178193; https://openalex.org/W2257979135; https://openalex.org/W2266822037; https://openalex.org/W2270245739; https://openalex.org/W2271971987; https://openalex.org/W2282339125; https://openalex.org/W2295598076; https://openalex.org/W2295739661; https://openalex.org/W2309832917; https://openalex.org/W2317747985; https://openalex.org/W2344075909; https://openalex.org/W2346138280; https://openalex.org/W2346573293; https://openalex.org/W2368061054; https://openalex.org/W2384495648; https://openalex.org/W2395916875; https://openalex.org/W2396466031; https://openalex.org/W2396961612; https://openalex.org/W2397115702; https://openalex.org/W2399500811; https://openalex.org/W2399851305; https://openalex.org/W2400084313; https://openalex.org/W2407014344; https://openalex.org/W2407212869; https://openalex.org/W2418011751; https://openalex.org/W2465345967; https://openalex.org/W2467110937; https://openalex.org/W2472819217; https://openalex.org/W2474440862; https://openalex.org/W2486444208; https://openalex.org/W2504108613; https://openalex.org/W2522203492; https://openalex.org/W2531409750; https://openalex.org/W2549852851; https://openalex.org/W2551342063; https://openalex.org/W2553303224; https://openalex.org/W2555886487; https://openalex.org/W2556372419; https://openalex.org/W2556522401; https://openalex.org/W2560674852; https://openalex.org/W2563364594; https://openalex.org/W2571670780; https://openalex.org/W2578206533; https://openalex.org/W2580087858; https://openalex.org/W2585240214; https://openalex.org/W2587014634; https://openalex.org/W2588803499; https://openalex.org/W2593649365; https://openalex.org/W2593649546; https://openalex.org/W2594475271; https://openalex.org/W2596367596; https://openalex.org/W2601450892; https://openalex.org/W2604763608; https://openalex.org/W2604766410; https://openalex.org/W2608595939; https://openalex.org/W2608702473; https://openalex.org/W2610817424; https://openalex.org/W2613868844; https://openalex.org/W2616180702; https://openalex.org/W2616619952; https://openalex.org/W2618530766; https://openalex.org/W2619184049; https://openalex.org/W2620641980; https://openalex.org/W2620689287; https://openalex.org/W2622730215; https://openalex.org/W2623091261; https://openalex.org/W2624086852; https://openalex.org/W2624473996; https://openalex.org/W2626984672; https://openalex.org/W2725660645; https://openalex.org/W2728797307; https://openalex.org/W2734383650; https://openalex.org/W2740438624; https://openalex.org/W2741261073; https://openalex.org/W2741430497; https://openalex.org/W2746314669; https://openalex.org/W2748513770; https://openalex.org/W2751836095; https://openalex.org/W2752331852; https://openalex.org/W2752852504; https://openalex.org/W2753160622; https://openalex.org/W2753433947; https://openalex.org/W2756085244; https://openalex.org/W2765407302; https://openalex.org/W2768408766; https://openalex.org/W2769653148; https://openalex.org/W2769743674; https://openalex.org/W2772089072; https://openalex.org/W2773108397; https://openalex.org/W2773706593; https://openalex.org/W2774246732; https://openalex.org/W2775233965; https://openalex.org/W2777138789; https://openalex.org/W2777539043; https://openalex.org/W2778618317; https://openalex.org/W2778633128; https://openalex.org/W2778749116; https://openalex.org/W2780562800; https://openalex.org/W2782093256; https://openalex.org/W2783201493; https://openalex.org/W2784287478; https://openalex.org/W2785444061; https://openalex.org/W2785494456; https://openalex.org/W2787035179; https://openalex.org/W2787189300; https://openalex.org/W2787501667; https://openalex.org/W2788079077; https://openalex.org/W2788110787; https://openalex.org/W2788853733; https://openalex.org/W2789487674; https://openalex.org/W2793670633; https://openalex.org/W2793695846; https://openalex.org/W2794356495; https://openalex.org/W2796265726; https://openalex.org/W2803311163; https://openalex.org/W2803435037; https://openalex.org/W2804534929; https://openalex.org/W2808938483; https://openalex.org/W2809054435; https://openalex.org/W2809880372; https://openalex.org/W2809899846; https://openalex.org/W2818275232; https://openalex.org/W2826306652; https://openalex.org/W2884528674; https://openalex.org/W2885311373; https://openalex.org/W2885487916; https://openalex.org/W2885820039; https://openalex.org/W2886200920; https://openalex.org/W2887612286; https://openalex.org/W2889130221; https://openalex.org/W2899771611; https://openalex.org/W2902994895; https://openalex.org/W2903995489; https://openalex.org/W2911090636; https://openalex.org/W2913566062; https://openalex.org/W2913668833; https://openalex.org/W2914694469; https://openalex.org/W2947123069; https://openalex.org/W2949264490; https://openalex.org/W2950277768; https://openalex.org/W2950326163; https://openalex.org/W2950330175; https://openalex.org/W2950680102; https://openalex.org/W2950731343; https://openalex.org/W2951104886; https://openalex.org/W2951775784; https://openalex.org/W2952074906; https://openalex.org/W2952125132; https://openalex.org/W2953384591; https://openalex.org/W2963216850; https://openalex.org/W2963263347; https://openalex.org/W2963305465; https://openalex.org/W2963341924; https://openalex.org/W2963446712; https://openalex.org/W2963474950; https://openalex.org/W2963565814; https://openalex.org/W2963628712; https://openalex.org/W2963775850; https://openalex.org/W2963778169; https://openalex.org/W2963815651; https://openalex.org/W2963821229; https://openalex.org/W2963840672; https://openalex.org/W2963905884; https://openalex.org/W2964025389; https://openalex.org/W2964029277; https://openalex.org/W2964054038; https://openalex.org/W2964081807; https://openalex.org/W2964137095; https://openalex.org/W2965658867; https://openalex.org/W2997644599; https://openalex.org/W3000180494; https://openalex.org/W3006551545; https://openalex.org/W3023169168; https://openalex.org/W3026324026; https://openalex.org/W3035219538; https://openalex.org/W3043188097; https://openalex.org/W3099343340; https://openalex.org/W3099934359; https://openalex.org/W3100055683; https://openalex.org/W3102978735; https://openalex.org/W3118608800; https://openalex.org/W3120740533; https://openalex.org/W3122943284; https://openalex.org/W3124229194; https://openalex.org/W3195149063; https://openalex.org/W4205687621; https://openalex.org/W4211049957; https://openalex.org/W4226503094; https://openalex.org/W4232158517; https://openalex.org/W4233965824; https://openalex.org/W4234228486; https://openalex.org/W4237910115; https://openalex.org/W4239181501; https://openalex.org/W4243562335; https://openalex.org/W4246635279; https://openalex.org/W4247950230; https://openalex.org/W4250224875; https://openalex.org/W4255491615; https://openalex.org/W4289752289; https://openalex.org/W4289763996; https://openalex.org/W4293407356; https://openalex.org/W4293407536; https://openalex.org/W4293870975; https://openalex.org/W4294375521; https://openalex.org/W4294646197; https://openalex.org/W4295185264; https://openalex.org/W4295292688; https://openalex.org/W4295727797; https://openalex.org/W4297670622; https://openalex.org/W4297733768; https://openalex.org/W4297778814; https://openalex.org/W4297800546; https://openalex.org/W4297803580; https://openalex.org/W4297917482; https://openalex.org/W4298052809; https://openalex.org/W4298342842; https://openalex.org/W4298826872; https://openalex.org/W4299518610; https://openalex.org/W4300001399; https://openalex.org/W4300197707; https://openalex.org/W4300427683; https://openalex.org/W4300687381; https://openalex.org/W4300687870; https://openalex.org/W4300716136; https://openalex.org/W4300799480; https://openalex.org/W4300971732; https://openalex.org/W4301181331; https://openalex.org/W4301260059; https://openalex.org/W4302594429; https://openalex.org/W4302768905; https://openalex.org/W4302793682; https://openalex.org/W4303633609; https://openalex.org/W4313169793; https://openalex.org/W4324106947; https://openalex.org/W4387808640; https://openalex.org/W4394633966; https://openalex.org/W4394672493</t>
         </is>
       </c>
       <c r="Q100" t="inlineStr">
         <is>
-          <t>Reproducing kernel Hilbert space;Kernel (algebra);Kernel method;Hilbert space;Binary classification;Range (aeronautics);Kernel embedding of distributions;Representer theorem;Pattern recognition (psychology);Radial basis function kernel</t>
+          <t>Computer science;Artificial intelligence;Machine learning</t>
         </is>
       </c>
       <c r="R100" t="inlineStr"/>
       <c r="S100" t="inlineStr">
         <is>
-          <t>We review machine learning methods employing positive definite kernels. These methods formulate learning and estimation problems in a reproducing kernel Hilbert space (RKHS) of functions defined on the data domain, expanded in terms of a kernel. Working in linear spaces of function has the benefit of facilitating the construction and analysis of learning algorithms while at the same time allowing large classes of functions. The latter include nonlinear functions as well as functions defined on nonvectorial data. We cover a wide range of methods, ranging from binary classifiers to sophisticated methods for estimation with structured data.</t>
-        </is>
-      </c>
-      <c r="T100" t="inlineStr">
-        <is>
-          <t>36</t>
-        </is>
-      </c>
-      <c r="U100" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
+          <t>This open access book gives the first comprehensive overview of general methods in Automatic Machine Learning, AutoML, collects descriptions of existing AutoML systems based on these methods, and discusses the first international challenge of AutoML systems.</t>
+        </is>
+      </c>
+      <c r="T100" t="inlineStr"/>
+      <c r="U100" t="inlineStr"/>
       <c r="V100" t="inlineStr"/>
       <c r="W100" t="inlineStr"/>
       <c r="X100" t="inlineStr">
         <is>
-          <t>Thomas Hofmann, 2008, The Annals of Statistics</t>
+          <t>Frank Hutter, 2019, The Springer series on challenges in machine learning</t>
         </is>
       </c>
       <c r="Y100" t="inlineStr">
         <is>
-          <t>Thomas Hofmann, 2008, The Annals of Statistics</t>
+          <t>Frank Hutter, 2019, The Springer series on challenges in machine learning</t>
         </is>
       </c>
     </row>
@@ -9913,36 +9905,36 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>https://openalex.org/W4213308398</t>
+          <t>https://openalex.org/W2168029744</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1007/978-3-030-05318-5</t>
+          <t>https://doi.org/10.1214/009053607000000677</t>
         </is>
       </c>
       <c r="D101" t="inlineStr"/>
       <c r="E101" t="inlineStr">
         <is>
-          <t>Automated Machine Learning</t>
+          <t>Kernel methods in machine learning</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>The Springer series on challenges in machine learning</t>
+          <t>The Annals of Statistics</t>
         </is>
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>The Springer series on challenges in machine learning</t>
+          <t>The Annals of Statistics</t>
         </is>
       </c>
       <c r="H101" t="n">
-        <v>2019</v>
+        <v>2008</v>
       </c>
       <c r="I101" t="inlineStr">
         <is>
-          <t>book</t>
+          <t>article</t>
         </is>
       </c>
       <c r="J101" t="inlineStr">
@@ -9951,48 +9943,56 @@
         </is>
       </c>
       <c r="K101" t="n">
-        <v>1402</v>
+        <v>1600</v>
       </c>
       <c r="L101" t="inlineStr">
         <is>
-          <t>Frank Hutter;Lars Kotthoff;Joaquin Vanschoren</t>
+          <t>Thomas Hofmann;Bernhard Schölkopf;Alexander J. Smola</t>
         </is>
       </c>
       <c r="M101" t="inlineStr"/>
       <c r="N101" t="inlineStr">
         <is>
-          <t>Frank Hutter, Department of Computer Science, University of Freiburg, Freiburg, Germany;Lars Kotthoff, University of Wyoming, Laramie, USA;Joaquin Vanschoren, Eindhoven University of Technology, Eindhoven, The Netherlands</t>
+          <t>Thomas Hofmann, Darmstadt University of Technology, Max Planck Institute for Biological Cybernetics and National ICT Australia;Alexander J. Smola, Darmstadt University of Technology, Max Planck Institute for Biological Cybernetics and National ICT Australia;Alexander J. Smola, MAX PLANCK INSTITUTE FOR BIOLOGICAL CYBERNETICS TBINGEN GERMANY</t>
         </is>
       </c>
       <c r="O101" t="inlineStr"/>
       <c r="P101" t="inlineStr">
         <is>
-          <t>https://openalex.org/W6908809; https://openalex.org/W24696228; https://openalex.org/W28412257; https://openalex.org/W41730657; https://openalex.org/W54639073; https://openalex.org/W60686164; https://openalex.org/W62188234; https://openalex.org/W76131926; https://openalex.org/W76331760; https://openalex.org/W85803853; https://openalex.org/W100047375; https://openalex.org/W114730584; https://openalex.org/W116375701; https://openalex.org/W122178443; https://openalex.org/W135104305; https://openalex.org/W138547447; https://openalex.org/W145519053; https://openalex.org/W148859753; https://openalex.org/W172742023; https://openalex.org/W174542576; https://openalex.org/W192975702; https://openalex.org/W198580638; https://openalex.org/W202805564; https://openalex.org/W202978992; https://openalex.org/W358897728; https://openalex.org/W603776396; https://openalex.org/W1165382972; https://openalex.org/W1471542436; https://openalex.org/W1480330138; https://openalex.org/W1484746829; https://openalex.org/W1488960379; https://openalex.org/W1491420040; https://openalex.org/W1494192115; https://openalex.org/W1494580925; https://openalex.org/W1500302649; https://openalex.org/W1501110974; https://openalex.org/W1503705371; https://openalex.org/W1507030697; https://openalex.org/W1512747601; https://openalex.org/W1516621661; https://openalex.org/W1519451279; https://openalex.org/W1520992199; https://openalex.org/W1522301498; https://openalex.org/W1528411633; https://openalex.org/W1533803232; https://openalex.org/W1534069108; https://openalex.org/W1534477342; https://openalex.org/W1535039099; https://openalex.org/W1539741229; https://openalex.org/W1542791059; https://openalex.org/W1543201103; https://openalex.org/W1549223806; https://openalex.org/W1556753024; https://openalex.org/W1565746575; https://openalex.org/W1568834902; https://openalex.org/W1569757501; https://openalex.org/W1575029535; https://openalex.org/W1575661061; https://openalex.org/W1577932924; https://openalex.org/W1581066146; https://openalex.org/W1588486985; https://openalex.org/W1588628884; https://openalex.org/W1588959569; https://openalex.org/W1589492330; https://openalex.org/W1593343777; https://openalex.org/W1598052524; https://openalex.org/W1601795611; https://openalex.org/W1604262624; https://openalex.org/W1631708156; https://openalex.org/W1638732406; https://openalex.org/W1640798781; https://openalex.org/W1647221522; https://openalex.org/W1661871015; https://openalex.org/W1663203009; https://openalex.org/W1663583528; https://openalex.org/W1678356000; https://openalex.org/W1680392829; https://openalex.org/W1690919088; https://openalex.org/W1701825639; https://openalex.org/W1758907577; https://openalex.org/W1763644767; https://openalex.org/W1840091437; https://openalex.org/W1868018859; https://openalex.org/W1880189740; https://openalex.org/W1886872224; https://openalex.org/W1922017469; https://openalex.org/W1925428099; https://openalex.org/W1925504357; https://openalex.org/W1935590542; https://openalex.org/W1965555277; https://openalex.org/W1968634175; https://openalex.org/W1969163824; https://openalex.org/W1971713783; https://openalex.org/W1973229481; https://openalex.org/W1979769287; https://openalex.org/W1980264541; https://openalex.org/W1981903823; https://openalex.org/W1984557319; https://openalex.org/W1985995090; https://openalex.org/W1986490585; https://openalex.org/W1986543815; https://openalex.org/W1986929000; https://openalex.org/W1989048657; https://openalex.org/W1994197834; https://openalex.org/W1994326354; https://openalex.org/W2001485654; https://openalex.org/W2040730773; https://openalex.org/W2040884411; https://openalex.org/W2048430744; https://openalex.org/W2050310928; https://openalex.org/W2051346631; https://openalex.org/W2056224615; https://openalex.org/W2057261601; https://openalex.org/W2062118960; https://openalex.org/W2062227835; https://openalex.org/W2064186732; https://openalex.org/W2074702228; https://openalex.org/W2074724805; https://openalex.org/W2078885513; https://openalex.org/W2083542829; https://openalex.org/W2084136177; https://openalex.org/W2084150578; https://openalex.org/W2087817842; https://openalex.org/W2089213632; https://openalex.org/W2089217417; https://openalex.org/W2090136295; https://openalex.org/W2091118421; https://openalex.org/W2095655959; https://openalex.org/W2095705004; https://openalex.org/W2096863518; https://openalex.org/W2097998348; https://openalex.org/W2099201756; https://openalex.org/W2101234009; https://openalex.org/W2101341561; https://openalex.org/W2102770307; https://openalex.org/W2105031846; https://openalex.org/W2106411961; https://openalex.org/W2106614481; https://openalex.org/W2107853397; https://openalex.org/W2108626634; https://openalex.org/W2109042184; https://openalex.org/W2109346685; https://openalex.org/W2111935653; https://openalex.org/W2112204321; https://openalex.org/W2112364454; https://openalex.org/W2113145584; https://openalex.org/W2113207845; https://openalex.org/W2113584252; https://openalex.org/W2115733720; https://openalex.org/W2115763804; https://openalex.org/W2116882733; https://openalex.org/W2117539524; https://openalex.org/W2118789407; https://openalex.org/W2119814172; https://openalex.org/W2120420045; https://openalex.org/W2122053572; https://openalex.org/W2122379760; https://openalex.org/W2122776323; https://openalex.org/W2123395972; https://openalex.org/W2123649031; https://openalex.org/W2124022122; https://openalex.org/W2124290836; https://openalex.org/W2124802506; https://openalex.org/W2125849100; https://openalex.org/W2125877832; https://openalex.org/W2126204609; https://openalex.org/W2126559945; https://openalex.org/W2126964466; https://openalex.org/W2127416213; https://openalex.org/W2129458072; https://openalex.org/W2130942839; https://openalex.org/W2131241448; https://openalex.org/W2131822674; https://openalex.org/W2133418613; https://openalex.org/W2133958955; https://openalex.org/W2136139971; https://openalex.org/W2136636278; https://openalex.org/W2137825550; https://openalex.org/W2138784882; https://openalex.org/W2139805416; https://openalex.org/W2141125852; https://openalex.org/W2141408223; https://openalex.org/W2142334564; https://openalex.org/W2142959074; https://openalex.org/W2143104527; https://openalex.org/W2144656844; https://openalex.org/W2144752499; https://openalex.org/W2144981148; https://openalex.org/W2145287260; https://openalex.org/W2145339207; https://openalex.org/W2145955992; https://openalex.org/W2146502635; https://openalex.org/W2149731329; https://openalex.org/W2150446468; https://openalex.org/W2152589362; https://openalex.org/W2153667946; https://openalex.org/W2154776925; https://openalex.org/W2155853132; https://openalex.org/W2156417353; https://openalex.org/W2157069634; https://openalex.org/W2160644528; https://openalex.org/W2163605009; https://openalex.org/W2163922914; https://openalex.org/W2165607334; https://openalex.org/W2165698076; https://openalex.org/W2165962877; https://openalex.org/W2166107799; https://openalex.org/W2168175751; https://openalex.org/W2168939893; https://openalex.org/W2171033594; https://openalex.org/W2171658832; https://openalex.org/W2181956361; https://openalex.org/W2182070128; https://openalex.org/W2182361439; https://openalex.org/W2183341477; https://openalex.org/W2183704914; https://openalex.org/W2186013251; https://openalex.org/W2189149359; https://openalex.org/W2192203593; https://openalex.org/W2194775991; https://openalex.org/W2200000192; https://openalex.org/W2210969396; https://openalex.org/W2226783037; https://openalex.org/W2234598170; https://openalex.org/W2234898963; https://openalex.org/W2249362929; https://openalex.org/W2250178193; https://openalex.org/W2257979135; https://openalex.org/W2266822037; https://openalex.org/W2270245739; https://openalex.org/W2271971987; https://openalex.org/W2282339125; https://openalex.org/W2295598076; https://openalex.org/W2295739661; https://openalex.org/W2309832917; https://openalex.org/W2317747985; https://openalex.org/W2344075909; https://openalex.org/W2346138280; https://openalex.org/W2346573293; https://openalex.org/W2368061054; https://openalex.org/W2384495648; https://openalex.org/W2395916875; https://openalex.org/W2396466031; https://openalex.org/W2396961612; https://openalex.org/W2397115702; https://openalex.org/W2399500811; https://openalex.org/W2399851305; https://openalex.org/W2400084313; https://openalex.org/W2407014344; https://openalex.org/W2407212869; https://openalex.org/W2418011751; https://openalex.org/W2465345967; https://openalex.org/W2467110937; https://openalex.org/W2472819217; https://openalex.org/W2474440862; https://openalex.org/W2486444208; https://openalex.org/W2504108613; https://openalex.org/W2522203492; https://openalex.org/W2531409750; https://openalex.org/W2549852851; https://openalex.org/W2551342063; https://openalex.org/W2553303224; https://openalex.org/W2555886487; https://openalex.org/W2556372419; https://openalex.org/W2556522401; https://openalex.org/W2560674852; https://openalex.org/W2563364594; https://openalex.org/W2571670780; https://openalex.org/W2578206533; https://openalex.org/W2580087858; https://openalex.org/W2585240214; https://openalex.org/W2587014634; https://openalex.org/W2588803499; https://openalex.org/W2593649365; https://openalex.org/W2593649546; https://openalex.org/W2594475271; https://openalex.org/W2596367596; https://openalex.org/W2601450892; https://openalex.org/W2604763608; https://openalex.org/W2604766410; https://openalex.org/W2608595939; https://openalex.org/W2608702473; https://openalex.org/W2610817424; https://openalex.org/W2613868844; https://openalex.org/W2616180702; https://openalex.org/W2616619952; https://openalex.org/W2618530766; https://openalex.org/W2619184049; https://openalex.org/W2620641980; https://openalex.org/W2620689287; https://openalex.org/W2622730215; https://openalex.org/W2623091261; https://openalex.org/W2624086852; https://openalex.org/W2624473996; https://openalex.org/W2626984672; https://openalex.org/W2725660645; https://openalex.org/W2728797307; https://openalex.org/W2734383650; https://openalex.org/W2740438624; https://openalex.org/W2741261073; https://openalex.org/W2741430497; https://openalex.org/W2746314669; https://openalex.org/W2748513770; https://openalex.org/W2751836095; https://openalex.org/W2752331852; https://openalex.org/W2752852504; https://openalex.org/W2753160622; https://openalex.org/W2753433947; https://openalex.org/W2756085244; https://openalex.org/W2765407302; https://openalex.org/W2768408766; https://openalex.org/W2769653148; https://openalex.org/W2769743674; https://openalex.org/W2772089072; https://openalex.org/W2773108397; https://openalex.org/W2773706593; https://openalex.org/W2774246732; https://openalex.org/W2775233965; https://openalex.org/W2777138789; https://openalex.org/W2777539043; https://openalex.org/W2778618317; https://openalex.org/W2778633128; https://openalex.org/W2778749116; https://openalex.org/W2780562800; https://openalex.org/W2782093256; https://openalex.org/W2783201493; https://openalex.org/W2784287478; https://openalex.org/W2785444061; https://openalex.org/W2785494456; https://openalex.org/W2787035179; https://openalex.org/W2787189300; https://openalex.org/W2787501667; https://openalex.org/W2788079077; https://openalex.org/W2788110787; https://openalex.org/W2788853733; https://openalex.org/W2789487674; https://openalex.org/W2793670633; https://openalex.org/W2793695846; https://openalex.org/W2794356495; https://openalex.org/W2796265726; https://openalex.org/W2803311163; https://openalex.org/W2803435037; https://openalex.org/W2804534929; https://openalex.org/W2808938483; https://openalex.org/W2809054435; https://openalex.org/W2809880372; https://openalex.org/W2809899846; https://openalex.org/W2818275232; https://openalex.org/W2826306652; https://openalex.org/W2884528674; https://openalex.org/W2885311373; https://openalex.org/W2885487916; https://openalex.org/W2885820039; https://openalex.org/W2886200920; https://openalex.org/W2887612286; https://openalex.org/W2889130221; https://openalex.org/W2899771611; https://openalex.org/W2902994895; https://openalex.org/W2903995489; https://openalex.org/W2911090636; https://openalex.org/W2913566062; https://openalex.org/W2913668833; https://openalex.org/W2914694469; https://openalex.org/W2947123069; https://openalex.org/W2949264490; https://openalex.org/W2950277768; https://openalex.org/W2950326163; https://openalex.org/W2950330175; https://openalex.org/W2950680102; https://openalex.org/W2950731343; https://openalex.org/W2951104886; https://openalex.org/W2951775784; https://openalex.org/W2952074906; https://openalex.org/W2952125132; https://openalex.org/W2953384591; https://openalex.org/W2963216850; https://openalex.org/W2963263347; https://openalex.org/W2963305465; https://openalex.org/W2963341924; https://openalex.org/W2963446712; https://openalex.org/W2963474950; https://openalex.org/W2963565814; https://openalex.org/W2963628712; https://openalex.org/W2963775850; https://openalex.org/W2963778169; https://openalex.org/W2963815651; https://openalex.org/W2963821229; https://openalex.org/W2963840672; https://openalex.org/W2963905884; https://openalex.org/W2964025389; https://openalex.org/W2964029277; https://openalex.org/W2964054038; https://openalex.org/W2964081807; https://openalex.org/W2964137095; https://openalex.org/W2965658867; https://openalex.org/W2997644599; https://openalex.org/W3000180494; https://openalex.org/W3006551545; https://openalex.org/W3023169168; https://openalex.org/W3026324026; https://openalex.org/W3035219538; https://openalex.org/W3043188097; https://openalex.org/W3099343340; https://openalex.org/W3099934359; https://openalex.org/W3100055683; https://openalex.org/W3102978735; https://openalex.org/W3118608800; https://openalex.org/W3120740533; https://openalex.org/W3122943284; https://openalex.org/W3124229194; https://openalex.org/W3195149063; https://openalex.org/W4205687621; https://openalex.org/W4211049957; https://openalex.org/W4226503094; https://openalex.org/W4232158517; https://openalex.org/W4233965824; https://openalex.org/W4234228486; https://openalex.org/W4237910115; https://openalex.org/W4239181501; https://openalex.org/W4243562335; https://openalex.org/W4246635279; https://openalex.org/W4247950230; https://openalex.org/W4250224875; https://openalex.org/W4255491615; https://openalex.org/W4289752289; https://openalex.org/W4289763996; https://openalex.org/W4293407356; https://openalex.org/W4293407536; https://openalex.org/W4293870975; https://openalex.org/W4294375521; https://openalex.org/W4294646197; https://openalex.org/W4295185264; https://openalex.org/W4295292688; https://openalex.org/W4295727797; https://openalex.org/W4297670622; https://openalex.org/W4297733768; https://openalex.org/W4297778814; https://openalex.org/W4297800546; https://openalex.org/W4297803580; https://openalex.org/W4297917482; https://openalex.org/W4298052809; https://openalex.org/W4298342842; https://openalex.org/W4298826872; https://openalex.org/W4299518610; https://openalex.org/W4300001399; https://openalex.org/W4300197707; https://openalex.org/W4300427683; https://openalex.org/W4300687381; https://openalex.org/W4300687870; https://openalex.org/W4300716136; https://openalex.org/W4300799480; https://openalex.org/W4300971732; https://openalex.org/W4301181331; https://openalex.org/W4301260059; https://openalex.org/W4302594429; https://openalex.org/W4302768905; https://openalex.org/W4302793682; https://openalex.org/W4303633609; https://openalex.org/W4313169793; https://openalex.org/W4324106947; https://openalex.org/W4387808640; https://openalex.org/W4394633966; https://openalex.org/W4394672493</t>
+          <t>https://openalex.org/W14071851; https://openalex.org/W56743589; https://openalex.org/W179694669; https://openalex.org/W1490266132; https://openalex.org/W1496189301; https://openalex.org/W1510073064; https://openalex.org/W1512098439; https://openalex.org/W1526146785; https://openalex.org/W1526729636; https://openalex.org/W1542652324; https://openalex.org/W1549656520; https://openalex.org/W1550988992; https://openalex.org/W1560729174; https://openalex.org/W1575431606; https://openalex.org/W1578255497; https://openalex.org/W1587744656; https://openalex.org/W1596052433; https://openalex.org/W1604293137; https://openalex.org/W1638081485; https://openalex.org/W1647376582; https://openalex.org/W1719651905; https://openalex.org/W1774304772; https://openalex.org/W1835509607; https://openalex.org/W1899157803; https://openalex.org/W1966347620; https://openalex.org/W1968934255; https://openalex.org/W1975077471; https://openalex.org/W1982032418; https://openalex.org/W1986931325; https://openalex.org/W1989408439; https://openalex.org/W1990534247; https://openalex.org/W1991200719; https://openalex.org/W1992236290; https://openalex.org/W1992666150; https://openalex.org/W1995558350; https://openalex.org/W1998438337; https://openalex.org/W1999486090; https://openalex.org/W2001792610; https://openalex.org/W2002806284; https://openalex.org/W2007154098; https://openalex.org/W2008400752; https://openalex.org/W2009511046; https://openalex.org/W2014902932; https://openalex.org/W2015904350; https://openalex.org/W2018582985; https://openalex.org/W2020816856; https://openalex.org/W2025341678; https://openalex.org/W2051381803; https://openalex.org/W2060591526; https://openalex.org/W2064976291; https://openalex.org/W2070771761; https://openalex.org/W2075887074; https://openalex.org/W2082100828; https://openalex.org/W2082612735; https://openalex.org/W2083780577; https://openalex.org/W2086404575; https://openalex.org/W2087258353; https://openalex.org/W2087347434; https://openalex.org/W2092182929; https://openalex.org/W2098385651; https://openalex.org/W2101276256; https://openalex.org/W2103657184; https://openalex.org/W2104128541; https://openalex.org/W2105842272; https://openalex.org/W2106353560; https://openalex.org/W2108153239; https://openalex.org/W2112076978; https://openalex.org/W2114281975; https://openalex.org/W2119647652; https://openalex.org/W2120340025; https://openalex.org/W2121127625; https://openalex.org/W2123606421; https://openalex.org/W2123737232; https://openalex.org/W2124101779; https://openalex.org/W2124225821; https://openalex.org/W2125053431; https://openalex.org/W2127713198; https://openalex.org/W2131479089; https://openalex.org/W2132637896; https://openalex.org/W2132870739; https://openalex.org/W2135046866; https://openalex.org/W2135498906; https://openalex.org/W2139686264; https://openalex.org/W2140095548; https://openalex.org/W2141224867; https://openalex.org/W2141407058; https://openalex.org/W2143956139; https://openalex.org/W2144068644; https://openalex.org/W2148018895; https://openalex.org/W2151949149; https://openalex.org/W2156515921; https://openalex.org/W2156909104; https://openalex.org/W2157791002; https://openalex.org/W2159737176; https://openalex.org/W2161920802; https://openalex.org/W2162836072; https://openalex.org/W2164943005; https://openalex.org/W2169945149; https://openalex.org/W2408196097; https://openalex.org/W2554813760; https://openalex.org/W2795528501; https://openalex.org/W2988119488; https://openalex.org/W2994982620; https://openalex.org/W4210636998; https://openalex.org/W4232576706; https://openalex.org/W4234698323; https://openalex.org/W4238284510; https://openalex.org/W4238957295; https://openalex.org/W4239510810; https://openalex.org/W4246066915; https://openalex.org/W4247545571; https://openalex.org/W4249925659; https://openalex.org/W4251085907; https://openalex.org/W4251115686; https://openalex.org/W4298876635; https://openalex.org/W4396738453</t>
         </is>
       </c>
       <c r="Q101" t="inlineStr">
         <is>
-          <t>Computer science;Artificial intelligence;Machine learning</t>
+          <t>Reproducing kernel Hilbert space;Kernel (algebra);Kernel method;Hilbert space;Binary classification;Range (aeronautics);Kernel embedding of distributions;Representer theorem;Pattern recognition (psychology);Radial basis function kernel</t>
         </is>
       </c>
       <c r="R101" t="inlineStr"/>
       <c r="S101" t="inlineStr">
         <is>
-          <t>This open access book gives the first comprehensive overview of general methods in Automatic Machine Learning, AutoML, collects descriptions of existing AutoML systems based on these methods, and discusses the first international challenge of AutoML systems.</t>
-        </is>
-      </c>
-      <c r="T101" t="inlineStr"/>
-      <c r="U101" t="inlineStr"/>
+          <t>We review machine learning methods employing positive definite kernels. These methods formulate learning and estimation problems in a reproducing kernel Hilbert space (RKHS) of functions defined on the data domain, expanded in terms of a kernel. Working in linear spaces of function has the benefit of facilitating the construction and analysis of learning algorithms while at the same time allowing large classes of functions. The latter include nonlinear functions as well as functions defined on nonvectorial data. We cover a wide range of methods, ranging from binary classifiers to sophisticated methods for estimation with structured data.</t>
+        </is>
+      </c>
+      <c r="T101" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
+      <c r="U101" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="V101" t="inlineStr"/>
       <c r="W101" t="inlineStr"/>
       <c r="X101" t="inlineStr">
         <is>
-          <t>Frank Hutter, 2019, The Springer series on challenges in machine learning</t>
+          <t>Thomas Hofmann, 2008, The Annals of Statistics</t>
         </is>
       </c>
       <c r="Y101" t="inlineStr">
         <is>
-          <t>Frank Hutter, 2019, The Springer series on challenges in machine learning</t>
+          <t>Thomas Hofmann, 2008, The Annals of Statistics</t>
         </is>
       </c>
     </row>

</xml_diff>